<commit_message>
Capture temuan pindah ke folder Google Drive
Tombol di lembar Defect membuka folder Drive; tiap baris menampung
tautan berkasnya. Drive tidak bisa dituju lewat nama berkas, jadi yang
ditempel adalah tautan — bukan nama seperti saat foldernya lokal.

Lembar makro dibuang: VBA tidak bisa mengunggah ke Drive tanpa
kredensial API, dan kredensial di dalam berkas yang dikirim ke banyak
orang sama saja dengan diumumkan. Digantikan satu halaman cara pakai,
termasuk pengingat menyetel akses tautan — tautan yang hanya bisa
dibuka pemiliknya sama saja dengan tidak dilampirkan.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/TEST-CASE-KAATAGO.xlsx
+++ b/docs/TEST-CASE-KAATAGO.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kasus Uji" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prasyarat" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tombol Makro (opsional)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cara Lampirkan Capture" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kasus Uji'!$A$1:$I$244</definedName>
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="19">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -73,18 +73,9 @@
     <font>
       <b val="1"/>
       <color rgb="004F46E5"/>
-      <sz val="13"/>
+      <sz val="12"/>
     </font>
     <font>
-      <sz val="10.5"/>
-    </font>
-    <font>
-      <name val="Menlo"/>
-      <sz val="9.5"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="006E728C"/>
       <sz val="10.5"/>
     </font>
     <font>
@@ -104,11 +95,6 @@
     <font>
       <i val="1"/>
       <color rgb="00B91C1C"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="004F46E5"/>
-      <sz val="12"/>
     </font>
   </fonts>
   <fills count="4">
@@ -199,11 +185,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -215,9 +201,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -267,12 +253,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -10326,8 +10307,8 @@
     <col width="16" customWidth="1" min="17" max="17"/>
     <col width="15" customWidth="1" min="18" max="18"/>
     <col width="15" customWidth="1" min="19" max="19"/>
-    <col width="22" customWidth="1" min="20" max="20"/>
-    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="40" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
     <col width="34" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
@@ -10339,20 +10320,20 @@
       </c>
       <c r="C1" s="24" t="inlineStr">
         <is>
-          <t>Isi satu baris per temuan. Simpan tangkapan layarnya di folder defect-capture, lalu tulis nama berkasnya di kolom Capture.</t>
+          <t>Isi satu baris per temuan. Unggah tangkapan layarnya ke folder Drive, lalu tempel tautan berkasnya di kolom Link Capture.</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="25">
-        <f>HYPERLINK("defect-capture", "📎  BUKA FOLDER CAPTURE")</f>
+        <f>HYPERLINK("https://drive.google.com/drive/folders/1MonfUjlqV0aABrLDleDZhugd3pULLIOf?usp=sharing", "BUKA FOLDER CAPTURE")</f>
         <v/>
       </c>
       <c r="B2" s="26" t="n"/>
       <c r="C2" s="27" t="n"/>
       <c r="D2" s="28" t="inlineStr">
         <is>
-          <t>Seret tangkapan layarnya ke folder itu, beri nama sesuai ID temuan (DF-001.jpg), lalu tulis namanya di kolom Capture.</t>
+          <t>Unggah ke folder itu, beri nama sesuai ID temuan (DF-001.jpg), lalu Salin Tautan berkasnya dan tempel di kolom Link Capture.</t>
         </is>
       </c>
     </row>
@@ -10454,12 +10435,12 @@
       </c>
       <c r="T4" s="12" t="inlineStr">
         <is>
-          <t>Capture</t>
+          <t>Link Capture</t>
         </is>
       </c>
       <c r="U4" s="12" t="inlineStr">
         <is>
-          <t>Buka Capture</t>
+          <t>Buka</t>
         </is>
       </c>
       <c r="V4" s="12" t="inlineStr">
@@ -10490,7 +10471,7 @@
       <c r="S5" s="13" t="n"/>
       <c r="T5" s="13" t="n"/>
       <c r="U5" s="29">
-        <f>IF(T5="","",HYPERLINK("defect-capture/"&amp;T5,"Buka"))</f>
+        <f>IF(T5="","",HYPERLINK(T5,"Buka"))</f>
         <v/>
       </c>
       <c r="V5" s="13" t="n"/>
@@ -10517,7 +10498,7 @@
       <c r="S6" s="16" t="n"/>
       <c r="T6" s="16" t="n"/>
       <c r="U6" s="30">
-        <f>IF(T6="","",HYPERLINK("defect-capture/"&amp;T6,"Buka"))</f>
+        <f>IF(T6="","",HYPERLINK(T6,"Buka"))</f>
         <v/>
       </c>
       <c r="V6" s="16" t="n"/>
@@ -10544,7 +10525,7 @@
       <c r="S7" s="13" t="n"/>
       <c r="T7" s="13" t="n"/>
       <c r="U7" s="29">
-        <f>IF(T7="","",HYPERLINK("defect-capture/"&amp;T7,"Buka"))</f>
+        <f>IF(T7="","",HYPERLINK(T7,"Buka"))</f>
         <v/>
       </c>
       <c r="V7" s="13" t="n"/>
@@ -10571,7 +10552,7 @@
       <c r="S8" s="16" t="n"/>
       <c r="T8" s="16" t="n"/>
       <c r="U8" s="30">
-        <f>IF(T8="","",HYPERLINK("defect-capture/"&amp;T8,"Buka"))</f>
+        <f>IF(T8="","",HYPERLINK(T8,"Buka"))</f>
         <v/>
       </c>
       <c r="V8" s="16" t="n"/>
@@ -10598,7 +10579,7 @@
       <c r="S9" s="13" t="n"/>
       <c r="T9" s="13" t="n"/>
       <c r="U9" s="29">
-        <f>IF(T9="","",HYPERLINK("defect-capture/"&amp;T9,"Buka"))</f>
+        <f>IF(T9="","",HYPERLINK(T9,"Buka"))</f>
         <v/>
       </c>
       <c r="V9" s="13" t="n"/>
@@ -10625,7 +10606,7 @@
       <c r="S10" s="16" t="n"/>
       <c r="T10" s="16" t="n"/>
       <c r="U10" s="30">
-        <f>IF(T10="","",HYPERLINK("defect-capture/"&amp;T10,"Buka"))</f>
+        <f>IF(T10="","",HYPERLINK(T10,"Buka"))</f>
         <v/>
       </c>
       <c r="V10" s="16" t="n"/>
@@ -10652,7 +10633,7 @@
       <c r="S11" s="13" t="n"/>
       <c r="T11" s="13" t="n"/>
       <c r="U11" s="29">
-        <f>IF(T11="","",HYPERLINK("defect-capture/"&amp;T11,"Buka"))</f>
+        <f>IF(T11="","",HYPERLINK(T11,"Buka"))</f>
         <v/>
       </c>
       <c r="V11" s="13" t="n"/>
@@ -10679,7 +10660,7 @@
       <c r="S12" s="16" t="n"/>
       <c r="T12" s="16" t="n"/>
       <c r="U12" s="30">
-        <f>IF(T12="","",HYPERLINK("defect-capture/"&amp;T12,"Buka"))</f>
+        <f>IF(T12="","",HYPERLINK(T12,"Buka"))</f>
         <v/>
       </c>
       <c r="V12" s="16" t="n"/>
@@ -10706,7 +10687,7 @@
       <c r="S13" s="13" t="n"/>
       <c r="T13" s="13" t="n"/>
       <c r="U13" s="29">
-        <f>IF(T13="","",HYPERLINK("defect-capture/"&amp;T13,"Buka"))</f>
+        <f>IF(T13="","",HYPERLINK(T13,"Buka"))</f>
         <v/>
       </c>
       <c r="V13" s="13" t="n"/>
@@ -10733,7 +10714,7 @@
       <c r="S14" s="16" t="n"/>
       <c r="T14" s="16" t="n"/>
       <c r="U14" s="30">
-        <f>IF(T14="","",HYPERLINK("defect-capture/"&amp;T14,"Buka"))</f>
+        <f>IF(T14="","",HYPERLINK(T14,"Buka"))</f>
         <v/>
       </c>
       <c r="V14" s="16" t="n"/>
@@ -10760,7 +10741,7 @@
       <c r="S15" s="13" t="n"/>
       <c r="T15" s="13" t="n"/>
       <c r="U15" s="29">
-        <f>IF(T15="","",HYPERLINK("defect-capture/"&amp;T15,"Buka"))</f>
+        <f>IF(T15="","",HYPERLINK(T15,"Buka"))</f>
         <v/>
       </c>
       <c r="V15" s="13" t="n"/>
@@ -10787,7 +10768,7 @@
       <c r="S16" s="16" t="n"/>
       <c r="T16" s="16" t="n"/>
       <c r="U16" s="30">
-        <f>IF(T16="","",HYPERLINK("defect-capture/"&amp;T16,"Buka"))</f>
+        <f>IF(T16="","",HYPERLINK(T16,"Buka"))</f>
         <v/>
       </c>
       <c r="V16" s="16" t="n"/>
@@ -10814,7 +10795,7 @@
       <c r="S17" s="13" t="n"/>
       <c r="T17" s="13" t="n"/>
       <c r="U17" s="29">
-        <f>IF(T17="","",HYPERLINK("defect-capture/"&amp;T17,"Buka"))</f>
+        <f>IF(T17="","",HYPERLINK(T17,"Buka"))</f>
         <v/>
       </c>
       <c r="V17" s="13" t="n"/>
@@ -10841,7 +10822,7 @@
       <c r="S18" s="16" t="n"/>
       <c r="T18" s="16" t="n"/>
       <c r="U18" s="30">
-        <f>IF(T18="","",HYPERLINK("defect-capture/"&amp;T18,"Buka"))</f>
+        <f>IF(T18="","",HYPERLINK(T18,"Buka"))</f>
         <v/>
       </c>
       <c r="V18" s="16" t="n"/>
@@ -10868,7 +10849,7 @@
       <c r="S19" s="13" t="n"/>
       <c r="T19" s="13" t="n"/>
       <c r="U19" s="29">
-        <f>IF(T19="","",HYPERLINK("defect-capture/"&amp;T19,"Buka"))</f>
+        <f>IF(T19="","",HYPERLINK(T19,"Buka"))</f>
         <v/>
       </c>
       <c r="V19" s="13" t="n"/>
@@ -10895,7 +10876,7 @@
       <c r="S20" s="16" t="n"/>
       <c r="T20" s="16" t="n"/>
       <c r="U20" s="30">
-        <f>IF(T20="","",HYPERLINK("defect-capture/"&amp;T20,"Buka"))</f>
+        <f>IF(T20="","",HYPERLINK(T20,"Buka"))</f>
         <v/>
       </c>
       <c r="V20" s="16" t="n"/>
@@ -10922,7 +10903,7 @@
       <c r="S21" s="13" t="n"/>
       <c r="T21" s="13" t="n"/>
       <c r="U21" s="29">
-        <f>IF(T21="","",HYPERLINK("defect-capture/"&amp;T21,"Buka"))</f>
+        <f>IF(T21="","",HYPERLINK(T21,"Buka"))</f>
         <v/>
       </c>
       <c r="V21" s="13" t="n"/>
@@ -10949,7 +10930,7 @@
       <c r="S22" s="16" t="n"/>
       <c r="T22" s="16" t="n"/>
       <c r="U22" s="30">
-        <f>IF(T22="","",HYPERLINK("defect-capture/"&amp;T22,"Buka"))</f>
+        <f>IF(T22="","",HYPERLINK(T22,"Buka"))</f>
         <v/>
       </c>
       <c r="V22" s="16" t="n"/>
@@ -10976,7 +10957,7 @@
       <c r="S23" s="13" t="n"/>
       <c r="T23" s="13" t="n"/>
       <c r="U23" s="29">
-        <f>IF(T23="","",HYPERLINK("defect-capture/"&amp;T23,"Buka"))</f>
+        <f>IF(T23="","",HYPERLINK(T23,"Buka"))</f>
         <v/>
       </c>
       <c r="V23" s="13" t="n"/>
@@ -11003,7 +10984,7 @@
       <c r="S24" s="16" t="n"/>
       <c r="T24" s="16" t="n"/>
       <c r="U24" s="30">
-        <f>IF(T24="","",HYPERLINK("defect-capture/"&amp;T24,"Buka"))</f>
+        <f>IF(T24="","",HYPERLINK(T24,"Buka"))</f>
         <v/>
       </c>
       <c r="V24" s="16" t="n"/>
@@ -11030,7 +11011,7 @@
       <c r="S25" s="13" t="n"/>
       <c r="T25" s="13" t="n"/>
       <c r="U25" s="29">
-        <f>IF(T25="","",HYPERLINK("defect-capture/"&amp;T25,"Buka"))</f>
+        <f>IF(T25="","",HYPERLINK(T25,"Buka"))</f>
         <v/>
       </c>
       <c r="V25" s="13" t="n"/>
@@ -11057,7 +11038,7 @@
       <c r="S26" s="16" t="n"/>
       <c r="T26" s="16" t="n"/>
       <c r="U26" s="30">
-        <f>IF(T26="","",HYPERLINK("defect-capture/"&amp;T26,"Buka"))</f>
+        <f>IF(T26="","",HYPERLINK(T26,"Buka"))</f>
         <v/>
       </c>
       <c r="V26" s="16" t="n"/>
@@ -11084,7 +11065,7 @@
       <c r="S27" s="13" t="n"/>
       <c r="T27" s="13" t="n"/>
       <c r="U27" s="29">
-        <f>IF(T27="","",HYPERLINK("defect-capture/"&amp;T27,"Buka"))</f>
+        <f>IF(T27="","",HYPERLINK(T27,"Buka"))</f>
         <v/>
       </c>
       <c r="V27" s="13" t="n"/>
@@ -11111,7 +11092,7 @@
       <c r="S28" s="16" t="n"/>
       <c r="T28" s="16" t="n"/>
       <c r="U28" s="30">
-        <f>IF(T28="","",HYPERLINK("defect-capture/"&amp;T28,"Buka"))</f>
+        <f>IF(T28="","",HYPERLINK(T28,"Buka"))</f>
         <v/>
       </c>
       <c r="V28" s="16" t="n"/>
@@ -11138,7 +11119,7 @@
       <c r="S29" s="13" t="n"/>
       <c r="T29" s="13" t="n"/>
       <c r="U29" s="29">
-        <f>IF(T29="","",HYPERLINK("defect-capture/"&amp;T29,"Buka"))</f>
+        <f>IF(T29="","",HYPERLINK(T29,"Buka"))</f>
         <v/>
       </c>
       <c r="V29" s="13" t="n"/>
@@ -11165,7 +11146,7 @@
       <c r="S30" s="16" t="n"/>
       <c r="T30" s="16" t="n"/>
       <c r="U30" s="30">
-        <f>IF(T30="","",HYPERLINK("defect-capture/"&amp;T30,"Buka"))</f>
+        <f>IF(T30="","",HYPERLINK(T30,"Buka"))</f>
         <v/>
       </c>
       <c r="V30" s="16" t="n"/>
@@ -11192,7 +11173,7 @@
       <c r="S31" s="13" t="n"/>
       <c r="T31" s="13" t="n"/>
       <c r="U31" s="29">
-        <f>IF(T31="","",HYPERLINK("defect-capture/"&amp;T31,"Buka"))</f>
+        <f>IF(T31="","",HYPERLINK(T31,"Buka"))</f>
         <v/>
       </c>
       <c r="V31" s="13" t="n"/>
@@ -11219,7 +11200,7 @@
       <c r="S32" s="16" t="n"/>
       <c r="T32" s="16" t="n"/>
       <c r="U32" s="30">
-        <f>IF(T32="","",HYPERLINK("defect-capture/"&amp;T32,"Buka"))</f>
+        <f>IF(T32="","",HYPERLINK(T32,"Buka"))</f>
         <v/>
       </c>
       <c r="V32" s="16" t="n"/>
@@ -11246,7 +11227,7 @@
       <c r="S33" s="13" t="n"/>
       <c r="T33" s="13" t="n"/>
       <c r="U33" s="29">
-        <f>IF(T33="","",HYPERLINK("defect-capture/"&amp;T33,"Buka"))</f>
+        <f>IF(T33="","",HYPERLINK(T33,"Buka"))</f>
         <v/>
       </c>
       <c r="V33" s="13" t="n"/>
@@ -11273,7 +11254,7 @@
       <c r="S34" s="16" t="n"/>
       <c r="T34" s="16" t="n"/>
       <c r="U34" s="30">
-        <f>IF(T34="","",HYPERLINK("defect-capture/"&amp;T34,"Buka"))</f>
+        <f>IF(T34="","",HYPERLINK(T34,"Buka"))</f>
         <v/>
       </c>
       <c r="V34" s="16" t="n"/>
@@ -11300,7 +11281,7 @@
       <c r="S35" s="13" t="n"/>
       <c r="T35" s="13" t="n"/>
       <c r="U35" s="29">
-        <f>IF(T35="","",HYPERLINK("defect-capture/"&amp;T35,"Buka"))</f>
+        <f>IF(T35="","",HYPERLINK(T35,"Buka"))</f>
         <v/>
       </c>
       <c r="V35" s="13" t="n"/>
@@ -11327,7 +11308,7 @@
       <c r="S36" s="16" t="n"/>
       <c r="T36" s="16" t="n"/>
       <c r="U36" s="30">
-        <f>IF(T36="","",HYPERLINK("defect-capture/"&amp;T36,"Buka"))</f>
+        <f>IF(T36="","",HYPERLINK(T36,"Buka"))</f>
         <v/>
       </c>
       <c r="V36" s="16" t="n"/>
@@ -11354,7 +11335,7 @@
       <c r="S37" s="13" t="n"/>
       <c r="T37" s="13" t="n"/>
       <c r="U37" s="29">
-        <f>IF(T37="","",HYPERLINK("defect-capture/"&amp;T37,"Buka"))</f>
+        <f>IF(T37="","",HYPERLINK(T37,"Buka"))</f>
         <v/>
       </c>
       <c r="V37" s="13" t="n"/>
@@ -11381,7 +11362,7 @@
       <c r="S38" s="16" t="n"/>
       <c r="T38" s="16" t="n"/>
       <c r="U38" s="30">
-        <f>IF(T38="","",HYPERLINK("defect-capture/"&amp;T38,"Buka"))</f>
+        <f>IF(T38="","",HYPERLINK(T38,"Buka"))</f>
         <v/>
       </c>
       <c r="V38" s="16" t="n"/>
@@ -11408,7 +11389,7 @@
       <c r="S39" s="13" t="n"/>
       <c r="T39" s="13" t="n"/>
       <c r="U39" s="29">
-        <f>IF(T39="","",HYPERLINK("defect-capture/"&amp;T39,"Buka"))</f>
+        <f>IF(T39="","",HYPERLINK(T39,"Buka"))</f>
         <v/>
       </c>
       <c r="V39" s="13" t="n"/>
@@ -11435,7 +11416,7 @@
       <c r="S40" s="16" t="n"/>
       <c r="T40" s="16" t="n"/>
       <c r="U40" s="30">
-        <f>IF(T40="","",HYPERLINK("defect-capture/"&amp;T40,"Buka"))</f>
+        <f>IF(T40="","",HYPERLINK(T40,"Buka"))</f>
         <v/>
       </c>
       <c r="V40" s="16" t="n"/>
@@ -11462,7 +11443,7 @@
       <c r="S41" s="13" t="n"/>
       <c r="T41" s="13" t="n"/>
       <c r="U41" s="29">
-        <f>IF(T41="","",HYPERLINK("defect-capture/"&amp;T41,"Buka"))</f>
+        <f>IF(T41="","",HYPERLINK(T41,"Buka"))</f>
         <v/>
       </c>
       <c r="V41" s="13" t="n"/>
@@ -11489,7 +11470,7 @@
       <c r="S42" s="16" t="n"/>
       <c r="T42" s="16" t="n"/>
       <c r="U42" s="30">
-        <f>IF(T42="","",HYPERLINK("defect-capture/"&amp;T42,"Buka"))</f>
+        <f>IF(T42="","",HYPERLINK(T42,"Buka"))</f>
         <v/>
       </c>
       <c r="V42" s="16" t="n"/>
@@ -11516,7 +11497,7 @@
       <c r="S43" s="13" t="n"/>
       <c r="T43" s="13" t="n"/>
       <c r="U43" s="29">
-        <f>IF(T43="","",HYPERLINK("defect-capture/"&amp;T43,"Buka"))</f>
+        <f>IF(T43="","",HYPERLINK(T43,"Buka"))</f>
         <v/>
       </c>
       <c r="V43" s="13" t="n"/>
@@ -11543,7 +11524,7 @@
       <c r="S44" s="16" t="n"/>
       <c r="T44" s="16" t="n"/>
       <c r="U44" s="30">
-        <f>IF(T44="","",HYPERLINK("defect-capture/"&amp;T44,"Buka"))</f>
+        <f>IF(T44="","",HYPERLINK(T44,"Buka"))</f>
         <v/>
       </c>
       <c r="V44" s="16" t="n"/>
@@ -11570,7 +11551,7 @@
       <c r="S45" s="13" t="n"/>
       <c r="T45" s="13" t="n"/>
       <c r="U45" s="29">
-        <f>IF(T45="","",HYPERLINK("defect-capture/"&amp;T45,"Buka"))</f>
+        <f>IF(T45="","",HYPERLINK(T45,"Buka"))</f>
         <v/>
       </c>
       <c r="V45" s="13" t="n"/>
@@ -11597,7 +11578,7 @@
       <c r="S46" s="16" t="n"/>
       <c r="T46" s="16" t="n"/>
       <c r="U46" s="30">
-        <f>IF(T46="","",HYPERLINK("defect-capture/"&amp;T46,"Buka"))</f>
+        <f>IF(T46="","",HYPERLINK(T46,"Buka"))</f>
         <v/>
       </c>
       <c r="V46" s="16" t="n"/>
@@ -11624,7 +11605,7 @@
       <c r="S47" s="13" t="n"/>
       <c r="T47" s="13" t="n"/>
       <c r="U47" s="29">
-        <f>IF(T47="","",HYPERLINK("defect-capture/"&amp;T47,"Buka"))</f>
+        <f>IF(T47="","",HYPERLINK(T47,"Buka"))</f>
         <v/>
       </c>
       <c r="V47" s="13" t="n"/>
@@ -11651,7 +11632,7 @@
       <c r="S48" s="16" t="n"/>
       <c r="T48" s="16" t="n"/>
       <c r="U48" s="30">
-        <f>IF(T48="","",HYPERLINK("defect-capture/"&amp;T48,"Buka"))</f>
+        <f>IF(T48="","",HYPERLINK(T48,"Buka"))</f>
         <v/>
       </c>
       <c r="V48" s="16" t="n"/>
@@ -11678,7 +11659,7 @@
       <c r="S49" s="13" t="n"/>
       <c r="T49" s="13" t="n"/>
       <c r="U49" s="29">
-        <f>IF(T49="","",HYPERLINK("defect-capture/"&amp;T49,"Buka"))</f>
+        <f>IF(T49="","",HYPERLINK(T49,"Buka"))</f>
         <v/>
       </c>
       <c r="V49" s="13" t="n"/>
@@ -11705,7 +11686,7 @@
       <c r="S50" s="16" t="n"/>
       <c r="T50" s="16" t="n"/>
       <c r="U50" s="30">
-        <f>IF(T50="","",HYPERLINK("defect-capture/"&amp;T50,"Buka"))</f>
+        <f>IF(T50="","",HYPERLINK(T50,"Buka"))</f>
         <v/>
       </c>
       <c r="V50" s="16" t="n"/>
@@ -11732,7 +11713,7 @@
       <c r="S51" s="13" t="n"/>
       <c r="T51" s="13" t="n"/>
       <c r="U51" s="29">
-        <f>IF(T51="","",HYPERLINK("defect-capture/"&amp;T51,"Buka"))</f>
+        <f>IF(T51="","",HYPERLINK(T51,"Buka"))</f>
         <v/>
       </c>
       <c r="V51" s="13" t="n"/>
@@ -11759,7 +11740,7 @@
       <c r="S52" s="16" t="n"/>
       <c r="T52" s="16" t="n"/>
       <c r="U52" s="30">
-        <f>IF(T52="","",HYPERLINK("defect-capture/"&amp;T52,"Buka"))</f>
+        <f>IF(T52="","",HYPERLINK(T52,"Buka"))</f>
         <v/>
       </c>
       <c r="V52" s="16" t="n"/>
@@ -11786,7 +11767,7 @@
       <c r="S53" s="13" t="n"/>
       <c r="T53" s="13" t="n"/>
       <c r="U53" s="29">
-        <f>IF(T53="","",HYPERLINK("defect-capture/"&amp;T53,"Buka"))</f>
+        <f>IF(T53="","",HYPERLINK(T53,"Buka"))</f>
         <v/>
       </c>
       <c r="V53" s="13" t="n"/>
@@ -11813,7 +11794,7 @@
       <c r="S54" s="16" t="n"/>
       <c r="T54" s="16" t="n"/>
       <c r="U54" s="30">
-        <f>IF(T54="","",HYPERLINK("defect-capture/"&amp;T54,"Buka"))</f>
+        <f>IF(T54="","",HYPERLINK(T54,"Buka"))</f>
         <v/>
       </c>
       <c r="V54" s="16" t="n"/>
@@ -11840,7 +11821,7 @@
       <c r="S55" s="13" t="n"/>
       <c r="T55" s="13" t="n"/>
       <c r="U55" s="29">
-        <f>IF(T55="","",HYPERLINK("defect-capture/"&amp;T55,"Buka"))</f>
+        <f>IF(T55="","",HYPERLINK(T55,"Buka"))</f>
         <v/>
       </c>
       <c r="V55" s="13" t="n"/>
@@ -11867,7 +11848,7 @@
       <c r="S56" s="16" t="n"/>
       <c r="T56" s="16" t="n"/>
       <c r="U56" s="30">
-        <f>IF(T56="","",HYPERLINK("defect-capture/"&amp;T56,"Buka"))</f>
+        <f>IF(T56="","",HYPERLINK(T56,"Buka"))</f>
         <v/>
       </c>
       <c r="V56" s="16" t="n"/>
@@ -11894,7 +11875,7 @@
       <c r="S57" s="13" t="n"/>
       <c r="T57" s="13" t="n"/>
       <c r="U57" s="29">
-        <f>IF(T57="","",HYPERLINK("defect-capture/"&amp;T57,"Buka"))</f>
+        <f>IF(T57="","",HYPERLINK(T57,"Buka"))</f>
         <v/>
       </c>
       <c r="V57" s="13" t="n"/>
@@ -11921,7 +11902,7 @@
       <c r="S58" s="16" t="n"/>
       <c r="T58" s="16" t="n"/>
       <c r="U58" s="30">
-        <f>IF(T58="","",HYPERLINK("defect-capture/"&amp;T58,"Buka"))</f>
+        <f>IF(T58="","",HYPERLINK(T58,"Buka"))</f>
         <v/>
       </c>
       <c r="V58" s="16" t="n"/>
@@ -11948,7 +11929,7 @@
       <c r="S59" s="13" t="n"/>
       <c r="T59" s="13" t="n"/>
       <c r="U59" s="29">
-        <f>IF(T59="","",HYPERLINK("defect-capture/"&amp;T59,"Buka"))</f>
+        <f>IF(T59="","",HYPERLINK(T59,"Buka"))</f>
         <v/>
       </c>
       <c r="V59" s="13" t="n"/>
@@ -11975,7 +11956,7 @@
       <c r="S60" s="16" t="n"/>
       <c r="T60" s="16" t="n"/>
       <c r="U60" s="30">
-        <f>IF(T60="","",HYPERLINK("defect-capture/"&amp;T60,"Buka"))</f>
+        <f>IF(T60="","",HYPERLINK(T60,"Buka"))</f>
         <v/>
       </c>
       <c r="V60" s="16" t="n"/>
@@ -12002,7 +11983,7 @@
       <c r="S61" s="13" t="n"/>
       <c r="T61" s="13" t="n"/>
       <c r="U61" s="29">
-        <f>IF(T61="","",HYPERLINK("defect-capture/"&amp;T61,"Buka"))</f>
+        <f>IF(T61="","",HYPERLINK(T61,"Buka"))</f>
         <v/>
       </c>
       <c r="V61" s="13" t="n"/>
@@ -12029,7 +12010,7 @@
       <c r="S62" s="16" t="n"/>
       <c r="T62" s="16" t="n"/>
       <c r="U62" s="30">
-        <f>IF(T62="","",HYPERLINK("defect-capture/"&amp;T62,"Buka"))</f>
+        <f>IF(T62="","",HYPERLINK(T62,"Buka"))</f>
         <v/>
       </c>
       <c r="V62" s="16" t="n"/>
@@ -12056,7 +12037,7 @@
       <c r="S63" s="13" t="n"/>
       <c r="T63" s="13" t="n"/>
       <c r="U63" s="29">
-        <f>IF(T63="","",HYPERLINK("defect-capture/"&amp;T63,"Buka"))</f>
+        <f>IF(T63="","",HYPERLINK(T63,"Buka"))</f>
         <v/>
       </c>
       <c r="V63" s="13" t="n"/>
@@ -12083,7 +12064,7 @@
       <c r="S64" s="16" t="n"/>
       <c r="T64" s="16" t="n"/>
       <c r="U64" s="30">
-        <f>IF(T64="","",HYPERLINK("defect-capture/"&amp;T64,"Buka"))</f>
+        <f>IF(T64="","",HYPERLINK(T64,"Buka"))</f>
         <v/>
       </c>
       <c r="V64" s="16" t="n"/>
@@ -12308,281 +12289,125 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B46"/>
+  <dimension ref="B1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="110" customWidth="1" min="2" max="2"/>
+    <col width="108" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="31" t="inlineStr">
-        <is>
-          <t>Tombol unggah capture — kalau memakai Excel desktop</t>
+      <c r="B1" s="10" t="inlineStr">
+        <is>
+          <t>Melampirkan tangkapan layar temuan</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="32" t="inlineStr"/>
+      <c r="B2" s="31" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="B3" s="32" t="inlineStr">
-        <is>
-          <t>Tombol ungu di lembar Defect membuka folder capture, lalu gambarnya diseret ke sana. Itu bekerja di Excel, LibreOffice, maupun Numbers, dan tidak butuh izin apa pun.</t>
+      <c r="B3" s="31" t="inlineStr">
+        <is>
+          <t>1.  Ambil tangkapan layar di HP saat temuannya terlihat.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="32" t="inlineStr"/>
+      <c r="B4" s="31" t="inlineStr">
+        <is>
+          <t>2.  Klik tombol BUKA FOLDER CAPTURE di lembar Defect — folder Drive-nya terbuka di peramban.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="B5" s="32" t="inlineStr">
-        <is>
-          <t>Kalau ingin tombol yang benar-benar membuka jendela pilih berkas lalu menyalin gambarnya sendiri, itu butuh makro — dan makro hanya hidup di berkas .xlsm. Sekali pasang:</t>
+      <c r="B5" s="31" t="inlineStr">
+        <is>
+          <t>3.  Unggah gambarnya ke sana, beri nama sesuai ID temuan: DF-001.jpg. Kalau butuh lebih dari satu, tambahkan keterangan: DF-001-sebelum.jpg, DF-001-sesudah.jpg.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="32" t="inlineStr"/>
+      <c r="B6" s="31" t="inlineStr">
+        <is>
+          <t>4.  Klik kanan berkasnya di Drive - Bagikan - Salin tautan.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="B7" s="32" t="inlineStr">
-        <is>
-          <t>1.  Simpan berkas ini sebagai .xlsm  (File - Save As - Excel Macro-Enabled Workbook)</t>
+      <c r="B7" s="31" t="inlineStr">
+        <is>
+          <t>5.  Tempel tautannya di kolom Link Capture pada baris temuan itu. Kolom Buka di sebelahnya berubah sendiri jadi tautan yang bisa diklik.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="32" t="inlineStr">
-        <is>
-          <t>2.  Alt+F11, atau Tools - Macro - Visual Basic Editor di Mac</t>
-        </is>
-      </c>
+      <c r="B8" s="31" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="B9" s="32" t="inlineStr">
-        <is>
-          <t>3.  Insert - Module, tempel kode di bawah</t>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Pastikan aksesnya "Siapa saja yang memiliki link"</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="32" t="inlineStr">
-        <is>
-          <t>4.  Kembali ke lembar Defect, Developer - Insert - Button, tautkan ke UnggahCapture</t>
-        </is>
-      </c>
+      <c r="B10" s="31" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="B11" s="32" t="inlineStr"/>
+      <c r="B11" s="31" t="inlineStr">
+        <is>
+          <t>Tautan yang hanya bisa dibuka pemiliknya sama saja dengan tidak dilampirkan: yang membaca laporan ini nanti bukan orang yang mengunggahnya, dan dia akan berhenti di halaman minta izin.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="B12" s="31" t="inlineStr">
-        <is>
-          <t>KODE VBA</t>
-        </is>
-      </c>
+      <c r="B12" s="31" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="B13" s="32" t="inlineStr"/>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Kenapa gambarnya tidak ditempel langsung ke Excel</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="B14" s="33" t="inlineStr">
-        <is>
-          <t>Sub UnggahCapture()</t>
-        </is>
-      </c>
+      <c r="B14" s="31" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="B15" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Dim asal As Variant, tujuan As String, folder As String</t>
+      <c r="B15" s="31" t="inlineStr">
+        <is>
+          <t>Satu tangkapan layar HP berukuran 300-800 KB. Tiga puluh temuan sudah cukup membuat berkas ini terlalu berat untuk dikirim lewat chat mana pun — dan berkas yang tidak bisa dikirim tidak dipakai siapa-siapa.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Dim baris As Long, idTemuan As String, ext As String</t>
-        </is>
-      </c>
+      <c r="B16" s="31" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="B17" s="33" t="inlineStr"/>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Kenapa tombolnya berupa tautan, bukan makro</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="B18" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    baris = ActiveCell.Row</t>
-        </is>
-      </c>
+      <c r="B18" s="31" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="B19" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    If baris &lt; 5 Then</t>
+      <c r="B19" s="31" t="inlineStr">
+        <is>
+          <t>Tombol yang menjalankan perintah di Excel butuh makro, dan makro tidak bisa mengunggah ke Google Drive tanpa kredensial API yang harus dititipkan di dalam berkasnya — kredensial di dalam berkas yang dikirim ke banyak orang sama saja dengan diumumkan.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        MsgBox "Klik dulu baris temuannya."</t>
-        </is>
-      </c>
+      <c r="B20" s="31" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="B21" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        Exit Sub</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    End If</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="33" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="B24" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    idTemuan = Trim(Cells(baris, 1).Value)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    If idTemuan = "" Then</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        MsgBox "Isi dulu ID temuannya di kolom A."</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        Exit Sub</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    End If</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="33" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="B30" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    asal = Application.GetOpenFilename( _</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="B31" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        "Gambar (*.jpg;*.jpeg;*.png),*.jpg;*.jpeg;*.png", , _</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="B32" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        "Pilih tangkapan layar untuk " &amp; idTemuan)</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    If asal = False Then Exit Sub</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="33" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="B35" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    folder = ThisWorkbook.Path &amp; Application.PathSeparator &amp; "defect-capture"</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    If Dir(folder, vbDirectory) = "" Then MkDir folder</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="B37" s="33" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="B38" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ext = Mid(asal, InStrRev(asal, "."))</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="B39" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    tujuan = folder &amp; Application.PathSeparator &amp; idTemuan &amp; ext</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="B40" s="33" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="B41" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    FileCopy CStr(asal), tujuan</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="B42" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Cells(baris, 20).Value = idTemuan &amp; ext</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="B43" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    MsgBox "Tersimpan: " &amp; idTemuan &amp; ext</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="B44" s="33" t="inlineStr">
-        <is>
-          <t>End Sub</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="B46" s="34" t="inlineStr">
-        <is>
-          <t>Angka 20 di baris Cells(baris, 20) adalah kolom Capture. Kalau urutan kolom di lembar Defect diubah, angka itu harus ikut diubah — makronya tidak akan mengeluh, ia hanya menulis ke kolom yang salah.</t>
+      <c r="B21" s="31" t="inlineStr">
+        <is>
+          <t>Selain itu makro hanya hidup di berkas .xlsm: mati di Google Sheets, mati di Numbers, dan ditolak sebagian penyetelan keamanan kantor. Tautan bekerja di semuanya, dan satu klik membuka folder tempat unggahannya memang dilakukan.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Billing langganan resto: harga & tanggal per resto, kunci saat menunggak
Harga dan tanggal jatuh tempo diatur Super Admin per resto. H-3 muncul
pita pengingat; lewat tenggang dan belum dibayar, restonya terkunci.

Penguncian dipasang sebagai kebijakan RLS restrictive, bukan hanya di
layar. Aplikasi ini bicara langsung ke Postgres tanpa server perantara
— layar yang terkunci hanyalah layar, dan siapa pun yang memegang kunci
publik proyek bisa memanggil API-nya langsung.

Tiga hal sengaja tidak dikunci: membaca tagihan, mengunggah bukti, dan
keluar akun. Mengunci jalan keluarnya sendiri akan meninggalkan resto
yang sudah membayar tanpa cara memberi tahu siapa pun.

Bukti yang sudah diunggah menahan penguncian selama diperiksa. Transfer
antarbank yang dikirim Jumat sore baru terlihat Senin, dan menghentikan
penjualan sehari penuh karena keterlambatan yang bukan salahnya adalah
kesalahan yang paling mahal di seluruh fitur ini.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/TEST-CASE-KAATAGO.xlsx
+++ b/docs/TEST-CASE-KAATAGO.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cara Lampirkan Capture" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kasus Uji'!$A$1:$I$244</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kasus Uji'!$A$1:$I$270</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Defect'!$A$4:$V$64</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -621,7 +621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -691,23 +691,23 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIF('Kasus Uji'!C2:C244,"P1")</f>
+        <f>COUNTIF('Kasus Uji'!C2:C270,"P1")</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C244,"P1",'Kasus Uji'!G2:G244,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C270,"P1",'Kasus Uji'!G2:G270,"Lulus")</f>
         <v/>
       </c>
       <c r="D5" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C244,"P1",'Kasus Uji'!G2:G244,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C270,"P1",'Kasus Uji'!G2:G270,"Gagal")</f>
         <v/>
       </c>
       <c r="E5" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C244,"P1",'Kasus Uji'!G2:G244,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C270,"P1",'Kasus Uji'!G2:G270,"Terblokir")</f>
         <v/>
       </c>
       <c r="F5" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C244,"P1",'Kasus Uji'!G2:G244,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C270,"P1",'Kasus Uji'!G2:G270,"Dilewati")</f>
         <v/>
       </c>
       <c r="G5" s="5">
@@ -722,23 +722,23 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('Kasus Uji'!C2:C244,"P2")</f>
+        <f>COUNTIF('Kasus Uji'!C2:C270,"P2")</f>
         <v/>
       </c>
       <c r="C6" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C244,"P2",'Kasus Uji'!G2:G244,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C270,"P2",'Kasus Uji'!G2:G270,"Lulus")</f>
         <v/>
       </c>
       <c r="D6" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C244,"P2",'Kasus Uji'!G2:G244,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C270,"P2",'Kasus Uji'!G2:G270,"Gagal")</f>
         <v/>
       </c>
       <c r="E6" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C244,"P2",'Kasus Uji'!G2:G244,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C270,"P2",'Kasus Uji'!G2:G270,"Terblokir")</f>
         <v/>
       </c>
       <c r="F6" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C244,"P2",'Kasus Uji'!G2:G244,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C270,"P2",'Kasus Uji'!G2:G270,"Dilewati")</f>
         <v/>
       </c>
       <c r="G6" s="5">
@@ -753,23 +753,23 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('Kasus Uji'!C2:C244,"P3")</f>
+        <f>COUNTIF('Kasus Uji'!C2:C270,"P3")</f>
         <v/>
       </c>
       <c r="C7" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C244,"P3",'Kasus Uji'!G2:G244,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C270,"P3",'Kasus Uji'!G2:G270,"Lulus")</f>
         <v/>
       </c>
       <c r="D7" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C244,"P3",'Kasus Uji'!G2:G244,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C270,"P3",'Kasus Uji'!G2:G270,"Gagal")</f>
         <v/>
       </c>
       <c r="E7" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C244,"P3",'Kasus Uji'!G2:G244,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C270,"P3",'Kasus Uji'!G2:G270,"Terblokir")</f>
         <v/>
       </c>
       <c r="F7" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C244,"P3",'Kasus Uji'!G2:G244,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C270,"P3",'Kasus Uji'!G2:G270,"Dilewati")</f>
         <v/>
       </c>
       <c r="G7" s="5">
@@ -859,23 +859,23 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A244,"Pelanggan")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A270,"Pelanggan")</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Pelanggan",'Kasus Uji'!G2:G244,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Pelanggan",'Kasus Uji'!G2:G270,"Lulus")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Pelanggan",'Kasus Uji'!G2:G244,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Pelanggan",'Kasus Uji'!G2:G270,"Gagal")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Pelanggan",'Kasus Uji'!G2:G244,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Pelanggan",'Kasus Uji'!G2:G270,"Terblokir")</f>
         <v/>
       </c>
       <c r="F12" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Pelanggan",'Kasus Uji'!G2:G244,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Pelanggan",'Kasus Uji'!G2:G270,"Dilewati")</f>
         <v/>
       </c>
       <c r="G12" s="5">
@@ -890,23 +890,23 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A244,"Kasir")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A270,"Kasir")</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Kasir",'Kasus Uji'!G2:G244,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Kasir",'Kasus Uji'!G2:G270,"Lulus")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Kasir",'Kasus Uji'!G2:G244,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Kasir",'Kasus Uji'!G2:G270,"Gagal")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Kasir",'Kasus Uji'!G2:G244,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Kasir",'Kasus Uji'!G2:G270,"Terblokir")</f>
         <v/>
       </c>
       <c r="F13" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Kasir",'Kasus Uji'!G2:G244,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Kasir",'Kasus Uji'!G2:G270,"Dilewati")</f>
         <v/>
       </c>
       <c r="G13" s="5">
@@ -921,23 +921,23 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A244,"Pending Payment")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A270,"Pending Payment")</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Pending Payment",'Kasus Uji'!G2:G244,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Pending Payment",'Kasus Uji'!G2:G270,"Lulus")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Pending Payment",'Kasus Uji'!G2:G244,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Pending Payment",'Kasus Uji'!G2:G270,"Gagal")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Pending Payment",'Kasus Uji'!G2:G244,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Pending Payment",'Kasus Uji'!G2:G270,"Terblokir")</f>
         <v/>
       </c>
       <c r="F14" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Pending Payment",'Kasus Uji'!G2:G244,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Pending Payment",'Kasus Uji'!G2:G270,"Dilewati")</f>
         <v/>
       </c>
       <c r="G14" s="5">
@@ -952,23 +952,23 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A244,"Dapur")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A270,"Dapur")</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Dapur",'Kasus Uji'!G2:G244,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Dapur",'Kasus Uji'!G2:G270,"Lulus")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Dapur",'Kasus Uji'!G2:G244,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Dapur",'Kasus Uji'!G2:G270,"Gagal")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Dapur",'Kasus Uji'!G2:G244,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Dapur",'Kasus Uji'!G2:G270,"Terblokir")</f>
         <v/>
       </c>
       <c r="F15" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Dapur",'Kasus Uji'!G2:G244,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Dapur",'Kasus Uji'!G2:G270,"Dilewati")</f>
         <v/>
       </c>
       <c r="G15" s="5">
@@ -983,23 +983,23 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A244,"Keuangan")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A270,"Keuangan")</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Keuangan",'Kasus Uji'!G2:G244,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Keuangan",'Kasus Uji'!G2:G270,"Lulus")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Keuangan",'Kasus Uji'!G2:G244,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Keuangan",'Kasus Uji'!G2:G270,"Gagal")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Keuangan",'Kasus Uji'!G2:G244,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Keuangan",'Kasus Uji'!G2:G270,"Terblokir")</f>
         <v/>
       </c>
       <c r="F16" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Keuangan",'Kasus Uji'!G2:G244,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Keuangan",'Kasus Uji'!G2:G270,"Dilewati")</f>
         <v/>
       </c>
       <c r="G16" s="5">
@@ -1014,23 +1014,23 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A244,"Setor Saldo Cash")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A270,"Setor Saldo Cash")</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Setor Saldo Cash",'Kasus Uji'!G2:G244,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Setor Saldo Cash",'Kasus Uji'!G2:G270,"Lulus")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Setor Saldo Cash",'Kasus Uji'!G2:G244,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Setor Saldo Cash",'Kasus Uji'!G2:G270,"Gagal")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Setor Saldo Cash",'Kasus Uji'!G2:G244,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Setor Saldo Cash",'Kasus Uji'!G2:G270,"Terblokir")</f>
         <v/>
       </c>
       <c r="F17" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Setor Saldo Cash",'Kasus Uji'!G2:G244,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Setor Saldo Cash",'Kasus Uji'!G2:G270,"Dilewati")</f>
         <v/>
       </c>
       <c r="G17" s="5">
@@ -1045,23 +1045,23 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A244,"Katalog &amp; Pengaturan")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A270,"Katalog &amp; Pengaturan")</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Katalog &amp; Pengaturan",'Kasus Uji'!G2:G244,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Katalog &amp; Pengaturan",'Kasus Uji'!G2:G270,"Lulus")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Katalog &amp; Pengaturan",'Kasus Uji'!G2:G244,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Katalog &amp; Pengaturan",'Kasus Uji'!G2:G270,"Gagal")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Katalog &amp; Pengaturan",'Kasus Uji'!G2:G244,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Katalog &amp; Pengaturan",'Kasus Uji'!G2:G270,"Terblokir")</f>
         <v/>
       </c>
       <c r="F18" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Katalog &amp; Pengaturan",'Kasus Uji'!G2:G244,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Katalog &amp; Pengaturan",'Kasus Uji'!G2:G270,"Dilewati")</f>
         <v/>
       </c>
       <c r="G18" s="5">
@@ -1076,23 +1076,23 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A244,"QR Meja")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A270,"QR Meja")</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"QR Meja",'Kasus Uji'!G2:G244,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"QR Meja",'Kasus Uji'!G2:G270,"Lulus")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"QR Meja",'Kasus Uji'!G2:G244,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"QR Meja",'Kasus Uji'!G2:G270,"Gagal")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"QR Meja",'Kasus Uji'!G2:G244,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"QR Meja",'Kasus Uji'!G2:G270,"Terblokir")</f>
         <v/>
       </c>
       <c r="F19" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"QR Meja",'Kasus Uji'!G2:G244,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"QR Meja",'Kasus Uji'!G2:G270,"Dilewati")</f>
         <v/>
       </c>
       <c r="G19" s="5">
@@ -1107,23 +1107,23 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A244,"Diskon")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A270,"Diskon")</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Diskon",'Kasus Uji'!G2:G244,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Diskon",'Kasus Uji'!G2:G270,"Lulus")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Diskon",'Kasus Uji'!G2:G244,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Diskon",'Kasus Uji'!G2:G270,"Gagal")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Diskon",'Kasus Uji'!G2:G244,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Diskon",'Kasus Uji'!G2:G270,"Terblokir")</f>
         <v/>
       </c>
       <c r="F20" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Diskon",'Kasus Uji'!G2:G244,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Diskon",'Kasus Uji'!G2:G270,"Dilewati")</f>
         <v/>
       </c>
       <c r="G20" s="5">
@@ -1138,23 +1138,23 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A244,"Kotak Masuk &amp; Pengumuman")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A270,"Kotak Masuk &amp; Pengumuman")</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Kotak Masuk &amp; Pengumuman",'Kasus Uji'!G2:G244,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Kotak Masuk &amp; Pengumuman",'Kasus Uji'!G2:G270,"Lulus")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Kotak Masuk &amp; Pengumuman",'Kasus Uji'!G2:G244,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Kotak Masuk &amp; Pengumuman",'Kasus Uji'!G2:G270,"Gagal")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Kotak Masuk &amp; Pengumuman",'Kasus Uji'!G2:G244,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Kotak Masuk &amp; Pengumuman",'Kasus Uji'!G2:G270,"Terblokir")</f>
         <v/>
       </c>
       <c r="F21" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Kotak Masuk &amp; Pengumuman",'Kasus Uji'!G2:G244,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Kotak Masuk &amp; Pengumuman",'Kasus Uji'!G2:G270,"Dilewati")</f>
         <v/>
       </c>
       <c r="G21" s="5">
@@ -1169,23 +1169,23 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A244,"Pembayaran QRIS")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A270,"Pembayaran QRIS")</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Pembayaran QRIS",'Kasus Uji'!G2:G244,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Pembayaran QRIS",'Kasus Uji'!G2:G270,"Lulus")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Pembayaran QRIS",'Kasus Uji'!G2:G244,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Pembayaran QRIS",'Kasus Uji'!G2:G270,"Gagal")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Pembayaran QRIS",'Kasus Uji'!G2:G244,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Pembayaran QRIS",'Kasus Uji'!G2:G270,"Terblokir")</f>
         <v/>
       </c>
       <c r="F22" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Pembayaran QRIS",'Kasus Uji'!G2:G244,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Pembayaran QRIS",'Kasus Uji'!G2:G270,"Dilewati")</f>
         <v/>
       </c>
       <c r="G22" s="5">
@@ -1200,23 +1200,23 @@
         </is>
       </c>
       <c r="B23" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A244,"Pembatalan &amp; Kedaluwarsa")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A270,"Pembatalan &amp; Kedaluwarsa")</f>
         <v/>
       </c>
       <c r="C23" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Pembatalan &amp; Kedaluwarsa",'Kasus Uji'!G2:G244,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Pembatalan &amp; Kedaluwarsa",'Kasus Uji'!G2:G270,"Lulus")</f>
         <v/>
       </c>
       <c r="D23" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Pembatalan &amp; Kedaluwarsa",'Kasus Uji'!G2:G244,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Pembatalan &amp; Kedaluwarsa",'Kasus Uji'!G2:G270,"Gagal")</f>
         <v/>
       </c>
       <c r="E23" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Pembatalan &amp; Kedaluwarsa",'Kasus Uji'!G2:G244,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Pembatalan &amp; Kedaluwarsa",'Kasus Uji'!G2:G270,"Terblokir")</f>
         <v/>
       </c>
       <c r="F23" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Pembatalan &amp; Kedaluwarsa",'Kasus Uji'!G2:G244,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Pembatalan &amp; Kedaluwarsa",'Kasus Uji'!G2:G270,"Dilewati")</f>
         <v/>
       </c>
       <c r="G23" s="5">
@@ -1231,23 +1231,23 @@
         </is>
       </c>
       <c r="B24" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A244,"Sesi Meja &amp; Identitas")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A270,"Sesi Meja &amp; Identitas")</f>
         <v/>
       </c>
       <c r="C24" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Sesi Meja &amp; Identitas",'Kasus Uji'!G2:G244,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Sesi Meja &amp; Identitas",'Kasus Uji'!G2:G270,"Lulus")</f>
         <v/>
       </c>
       <c r="D24" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Sesi Meja &amp; Identitas",'Kasus Uji'!G2:G244,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Sesi Meja &amp; Identitas",'Kasus Uji'!G2:G270,"Gagal")</f>
         <v/>
       </c>
       <c r="E24" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Sesi Meja &amp; Identitas",'Kasus Uji'!G2:G244,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Sesi Meja &amp; Identitas",'Kasus Uji'!G2:G270,"Terblokir")</f>
         <v/>
       </c>
       <c r="F24" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Sesi Meja &amp; Identitas",'Kasus Uji'!G2:G244,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Sesi Meja &amp; Identitas",'Kasus Uji'!G2:G270,"Dilewati")</f>
         <v/>
       </c>
       <c r="G24" s="5">
@@ -1262,23 +1262,23 @@
         </is>
       </c>
       <c r="B25" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A244,"Tampilan")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A270,"Tampilan")</f>
         <v/>
       </c>
       <c r="C25" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Tampilan",'Kasus Uji'!G2:G244,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Tampilan",'Kasus Uji'!G2:G270,"Lulus")</f>
         <v/>
       </c>
       <c r="D25" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Tampilan",'Kasus Uji'!G2:G244,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Tampilan",'Kasus Uji'!G2:G270,"Gagal")</f>
         <v/>
       </c>
       <c r="E25" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Tampilan",'Kasus Uji'!G2:G244,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Tampilan",'Kasus Uji'!G2:G270,"Terblokir")</f>
         <v/>
       </c>
       <c r="F25" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Tampilan",'Kasus Uji'!G2:G244,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Tampilan",'Kasus Uji'!G2:G270,"Dilewati")</f>
         <v/>
       </c>
       <c r="G25" s="5">
@@ -1293,23 +1293,23 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A244,"Super Admin")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A270,"Super Admin")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Super Admin",'Kasus Uji'!G2:G244,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Super Admin",'Kasus Uji'!G2:G270,"Lulus")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Super Admin",'Kasus Uji'!G2:G244,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Super Admin",'Kasus Uji'!G2:G270,"Gagal")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Super Admin",'Kasus Uji'!G2:G244,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Super Admin",'Kasus Uji'!G2:G270,"Terblokir")</f>
         <v/>
       </c>
       <c r="F26" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Super Admin",'Kasus Uji'!G2:G244,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Super Admin",'Kasus Uji'!G2:G270,"Dilewati")</f>
         <v/>
       </c>
       <c r="G26" s="5">
@@ -1324,23 +1324,23 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A244,"Pembaruan Aplikasi")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A270,"Pembaruan Aplikasi")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Pembaruan Aplikasi",'Kasus Uji'!G2:G244,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Pembaruan Aplikasi",'Kasus Uji'!G2:G270,"Lulus")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Pembaruan Aplikasi",'Kasus Uji'!G2:G244,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Pembaruan Aplikasi",'Kasus Uji'!G2:G270,"Gagal")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Pembaruan Aplikasi",'Kasus Uji'!G2:G244,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Pembaruan Aplikasi",'Kasus Uji'!G2:G270,"Terblokir")</f>
         <v/>
       </c>
       <c r="F27" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Pembaruan Aplikasi",'Kasus Uji'!G2:G244,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Pembaruan Aplikasi",'Kasus Uji'!G2:G270,"Dilewati")</f>
         <v/>
       </c>
       <c r="G27" s="5">
@@ -1351,27 +1351,27 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A244,"Uji Teknis (lingkup TSD)")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A270,"## 19b. Langganan &amp; Tagihan Resto")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Uji Teknis (lingkup TSD)",'Kasus Uji'!G2:G244,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"## 19b. Langganan &amp; Tagihan Resto",'Kasus Uji'!G2:G270,"Lulus")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Uji Teknis (lingkup TSD)",'Kasus Uji'!G2:G244,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"## 19b. Langganan &amp; Tagihan Resto",'Kasus Uji'!G2:G270,"Gagal")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Uji Teknis (lingkup TSD)",'Kasus Uji'!G2:G244,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"## 19b. Langganan &amp; Tagihan Resto",'Kasus Uji'!G2:G270,"Terblokir")</f>
         <v/>
       </c>
       <c r="F28" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Uji Teknis (lingkup TSD)",'Kasus Uji'!G2:G244,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"## 19b. Langganan &amp; Tagihan Resto",'Kasus Uji'!G2:G270,"Dilewati")</f>
         <v/>
       </c>
       <c r="G28" s="5">
@@ -1382,27 +1382,27 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>Uji Teknis (lingkup TSD)</t>
         </is>
       </c>
       <c r="B29" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A244,"Regresi — bug yang pernah terjadi")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A270,"Uji Teknis (lingkup TSD)")</f>
         <v/>
       </c>
       <c r="C29" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Regresi — bug yang pernah terjadi",'Kasus Uji'!G2:G244,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Uji Teknis (lingkup TSD)",'Kasus Uji'!G2:G270,"Lulus")</f>
         <v/>
       </c>
       <c r="D29" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Regresi — bug yang pernah terjadi",'Kasus Uji'!G2:G244,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Uji Teknis (lingkup TSD)",'Kasus Uji'!G2:G270,"Gagal")</f>
         <v/>
       </c>
       <c r="E29" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Regresi — bug yang pernah terjadi",'Kasus Uji'!G2:G244,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Uji Teknis (lingkup TSD)",'Kasus Uji'!G2:G270,"Terblokir")</f>
         <v/>
       </c>
       <c r="F29" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Regresi — bug yang pernah terjadi",'Kasus Uji'!G2:G244,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Uji Teknis (lingkup TSD)",'Kasus Uji'!G2:G270,"Dilewati")</f>
         <v/>
       </c>
       <c r="G29" s="5">
@@ -1413,27 +1413,27 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>Uji Ujung-ke-Ujung</t>
+          <t>Regresi — bug yang pernah terjadi</t>
         </is>
       </c>
       <c r="B30" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A244,"Uji Ujung-ke-Ujung")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A270,"Regresi — bug yang pernah terjadi")</f>
         <v/>
       </c>
       <c r="C30" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Uji Ujung-ke-Ujung",'Kasus Uji'!G2:G244,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Regresi — bug yang pernah terjadi",'Kasus Uji'!G2:G270,"Lulus")</f>
         <v/>
       </c>
       <c r="D30" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Uji Ujung-ke-Ujung",'Kasus Uji'!G2:G244,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Regresi — bug yang pernah terjadi",'Kasus Uji'!G2:G270,"Gagal")</f>
         <v/>
       </c>
       <c r="E30" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Uji Ujung-ke-Ujung",'Kasus Uji'!G2:G244,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Regresi — bug yang pernah terjadi",'Kasus Uji'!G2:G270,"Terblokir")</f>
         <v/>
       </c>
       <c r="F30" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A244,"Uji Ujung-ke-Ujung",'Kasus Uji'!G2:G244,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Regresi — bug yang pernah terjadi",'Kasus Uji'!G2:G270,"Dilewati")</f>
         <v/>
       </c>
       <c r="G30" s="5">
@@ -1441,214 +1441,245 @@
         <v/>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="9" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Uji Ujung-ke-Ujung</t>
+        </is>
+      </c>
+      <c r="B31" s="5">
+        <f>COUNTIF('Kasus Uji'!A2:A270,"Uji Ujung-ke-Ujung")</f>
+        <v/>
+      </c>
+      <c r="C31" s="5">
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Uji Ujung-ke-Ujung",'Kasus Uji'!G2:G270,"Lulus")</f>
+        <v/>
+      </c>
+      <c r="D31" s="5">
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Uji Ujung-ke-Ujung",'Kasus Uji'!G2:G270,"Gagal")</f>
+        <v/>
+      </c>
+      <c r="E31" s="5">
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Uji Ujung-ke-Ujung",'Kasus Uji'!G2:G270,"Terblokir")</f>
+        <v/>
+      </c>
+      <c r="F31" s="5">
+        <f>COUNTIFS('Kasus Uji'!A2:A270,"Uji Ujung-ke-Ujung",'Kasus Uji'!G2:G270,"Dilewati")</f>
+        <v/>
+      </c>
+      <c r="G31" s="5">
+        <f>B31-SUM(C31:F31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="9" t="inlineStr">
         <is>
           <t>Rilis ditahan selama masih ada P1 yang Gagal.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="10" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="10" t="inlineStr">
         <is>
           <t>Temuan</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="11" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>Jumlah</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr">
+      <c r="C36" s="3" t="inlineStr">
         <is>
           <t>Baru</t>
         </is>
       </c>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="D36" s="3" t="inlineStr">
         <is>
           <t>Dikonfirmasi</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr">
+      <c r="E36" s="3" t="inlineStr">
         <is>
           <t>Sedang diperbaiki</t>
         </is>
       </c>
-      <c r="F35" s="3" t="inlineStr">
+      <c r="F36" s="3" t="inlineStr">
         <is>
           <t>Menunggu retest</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G36" s="3" t="inlineStr">
         <is>
           <t>Ditutup</t>
         </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>Blocker</t>
-        </is>
-      </c>
-      <c r="B36" s="5">
-        <f>COUNTIF(Defect!M5:M64,"Blocker")</f>
-        <v/>
-      </c>
-      <c r="C36" s="5">
-        <f>COUNTIFS(Defect!M5:M64,"Blocker",Defect!P5:P64,"Baru")</f>
-        <v/>
-      </c>
-      <c r="D36" s="5">
-        <f>COUNTIFS(Defect!M5:M64,"Blocker",Defect!P5:P64,"Dikonfirmasi")</f>
-        <v/>
-      </c>
-      <c r="E36" s="5">
-        <f>COUNTIFS(Defect!M5:M64,"Blocker",Defect!P5:P64,"Sedang diperbaiki")</f>
-        <v/>
-      </c>
-      <c r="F36" s="5">
-        <f>COUNTIFS(Defect!M5:M64,"Blocker",Defect!P5:P64,"Menunggu retest")</f>
-        <v/>
-      </c>
-      <c r="G36" s="5">
-        <f>COUNTIFS(Defect!M5:M64,"Blocker",Defect!P5:P64,"Ditutup")</f>
-        <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Blocker</t>
         </is>
       </c>
       <c r="B37" s="5">
-        <f>COUNTIF(Defect!M5:M64,"Major")</f>
+        <f>COUNTIF(Defect!M5:M64,"Blocker")</f>
         <v/>
       </c>
       <c r="C37" s="5">
-        <f>COUNTIFS(Defect!M5:M64,"Major",Defect!P5:P64,"Baru")</f>
+        <f>COUNTIFS(Defect!M5:M64,"Blocker",Defect!P5:P64,"Baru")</f>
         <v/>
       </c>
       <c r="D37" s="5">
-        <f>COUNTIFS(Defect!M5:M64,"Major",Defect!P5:P64,"Dikonfirmasi")</f>
+        <f>COUNTIFS(Defect!M5:M64,"Blocker",Defect!P5:P64,"Dikonfirmasi")</f>
         <v/>
       </c>
       <c r="E37" s="5">
-        <f>COUNTIFS(Defect!M5:M64,"Major",Defect!P5:P64,"Sedang diperbaiki")</f>
+        <f>COUNTIFS(Defect!M5:M64,"Blocker",Defect!P5:P64,"Sedang diperbaiki")</f>
         <v/>
       </c>
       <c r="F37" s="5">
-        <f>COUNTIFS(Defect!M5:M64,"Major",Defect!P5:P64,"Menunggu retest")</f>
+        <f>COUNTIFS(Defect!M5:M64,"Blocker",Defect!P5:P64,"Menunggu retest")</f>
         <v/>
       </c>
       <c r="G37" s="5">
-        <f>COUNTIFS(Defect!M5:M64,"Major",Defect!P5:P64,"Ditutup")</f>
+        <f>COUNTIFS(Defect!M5:M64,"Blocker",Defect!P5:P64,"Ditutup")</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="B38" s="5">
-        <f>COUNTIF(Defect!M5:M64,"Minor")</f>
+        <f>COUNTIF(Defect!M5:M64,"Major")</f>
         <v/>
       </c>
       <c r="C38" s="5">
-        <f>COUNTIFS(Defect!M5:M64,"Minor",Defect!P5:P64,"Baru")</f>
+        <f>COUNTIFS(Defect!M5:M64,"Major",Defect!P5:P64,"Baru")</f>
         <v/>
       </c>
       <c r="D38" s="5">
-        <f>COUNTIFS(Defect!M5:M64,"Minor",Defect!P5:P64,"Dikonfirmasi")</f>
+        <f>COUNTIFS(Defect!M5:M64,"Major",Defect!P5:P64,"Dikonfirmasi")</f>
         <v/>
       </c>
       <c r="E38" s="5">
-        <f>COUNTIFS(Defect!M5:M64,"Minor",Defect!P5:P64,"Sedang diperbaiki")</f>
+        <f>COUNTIFS(Defect!M5:M64,"Major",Defect!P5:P64,"Sedang diperbaiki")</f>
         <v/>
       </c>
       <c r="F38" s="5">
-        <f>COUNTIFS(Defect!M5:M64,"Minor",Defect!P5:P64,"Menunggu retest")</f>
+        <f>COUNTIFS(Defect!M5:M64,"Major",Defect!P5:P64,"Menunggu retest")</f>
         <v/>
       </c>
       <c r="G38" s="5">
-        <f>COUNTIFS(Defect!M5:M64,"Minor",Defect!P5:P64,"Ditutup")</f>
+        <f>COUNTIFS(Defect!M5:M64,"Major",Defect!P5:P64,"Ditutup")</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="B39" s="5">
+        <f>COUNTIF(Defect!M5:M64,"Minor")</f>
+        <v/>
+      </c>
+      <c r="C39" s="5">
+        <f>COUNTIFS(Defect!M5:M64,"Minor",Defect!P5:P64,"Baru")</f>
+        <v/>
+      </c>
+      <c r="D39" s="5">
+        <f>COUNTIFS(Defect!M5:M64,"Minor",Defect!P5:P64,"Dikonfirmasi")</f>
+        <v/>
+      </c>
+      <c r="E39" s="5">
+        <f>COUNTIFS(Defect!M5:M64,"Minor",Defect!P5:P64,"Sedang diperbaiki")</f>
+        <v/>
+      </c>
+      <c r="F39" s="5">
+        <f>COUNTIFS(Defect!M5:M64,"Minor",Defect!P5:P64,"Menunggu retest")</f>
+        <v/>
+      </c>
+      <c r="G39" s="5">
+        <f>COUNTIFS(Defect!M5:M64,"Minor",Defect!P5:P64,"Ditutup")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
           <t>Trivial</t>
         </is>
       </c>
-      <c r="B39" s="5">
+      <c r="B40" s="5">
         <f>COUNTIF(Defect!M5:M64,"Trivial")</f>
         <v/>
       </c>
-      <c r="C39" s="5">
+      <c r="C40" s="5">
         <f>COUNTIFS(Defect!M5:M64,"Trivial",Defect!P5:P64,"Baru")</f>
         <v/>
       </c>
-      <c r="D39" s="5">
+      <c r="D40" s="5">
         <f>COUNTIFS(Defect!M5:M64,"Trivial",Defect!P5:P64,"Dikonfirmasi")</f>
         <v/>
       </c>
-      <c r="E39" s="5">
+      <c r="E40" s="5">
         <f>COUNTIFS(Defect!M5:M64,"Trivial",Defect!P5:P64,"Sedang diperbaiki")</f>
         <v/>
       </c>
-      <c r="F39" s="5">
+      <c r="F40" s="5">
         <f>COUNTIFS(Defect!M5:M64,"Trivial",Defect!P5:P64,"Menunggu retest")</f>
         <v/>
       </c>
-      <c r="G39" s="5">
+      <c r="G40" s="5">
         <f>COUNTIFS(Defect!M5:M64,"Trivial",Defect!P5:P64,"Ditutup")</f>
         <v/>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="6" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B40" s="7">
-        <f>SUM(B36:B39)</f>
-        <v/>
-      </c>
-      <c r="C40" s="7">
-        <f>SUM(C36:C39)</f>
-        <v/>
-      </c>
-      <c r="D40" s="7">
-        <f>SUM(D36:D39)</f>
-        <v/>
-      </c>
-      <c r="E40" s="7">
-        <f>SUM(E36:E39)</f>
-        <v/>
-      </c>
-      <c r="F40" s="7">
-        <f>SUM(F36:F39)</f>
-        <v/>
-      </c>
-      <c r="G40" s="7">
-        <f>SUM(G36:G39)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="9" t="inlineStr">
+      <c r="B41" s="7">
+        <f>SUM(B37:B40)</f>
+        <v/>
+      </c>
+      <c r="C41" s="7">
+        <f>SUM(C37:C40)</f>
+        <v/>
+      </c>
+      <c r="D41" s="7">
+        <f>SUM(D37:D40)</f>
+        <v/>
+      </c>
+      <c r="E41" s="7">
+        <f>SUM(E37:E40)</f>
+        <v/>
+      </c>
+      <c r="F41" s="7">
+        <f>SUM(F37:F40)</f>
+        <v/>
+      </c>
+      <c r="G41" s="7">
+        <f>SUM(G37:G40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="9" t="inlineStr">
         <is>
           <t>Blocker yang belum Ditutup menahan rilis.</t>
         </is>
@@ -1665,7 +1696,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I244"/>
+  <dimension ref="A1:I270"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -8799,32 +8830,32 @@
     <row r="204">
       <c r="A204" s="13" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B204" s="14" t="inlineStr">
         <is>
-          <t>TC-TS-01</t>
-        </is>
-      </c>
-      <c r="C204" s="15" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>TC-BL-01</t>
+        </is>
+      </c>
+      <c r="C204" s="19" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D204" s="13" t="inlineStr">
         <is>
-          <t>Panggil GET /rest/v1/orders memakai kunci anon tanpa login</t>
+          <t>Super Admin → Billing Resto → atur harga dan tanggal untuk sebuah resto</t>
         </is>
       </c>
       <c r="E204" s="13" t="inlineStr">
         <is>
-          <t>Tidak mengembalikan pesanan resto mana pun</t>
+          <t>Tersimpan; kartu restonya menampilkan harga, tanggal, dan tenggangnya</t>
         </is>
       </c>
       <c r="F204" s="13" t="inlineStr">
         <is>
-          <t>TSD §5</t>
+          <t>F-BL-01, F-BL-02</t>
         </is>
       </c>
       <c r="G204" s="13" t="inlineStr"/>
@@ -8834,32 +8865,32 @@
     <row r="205">
       <c r="A205" s="16" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B205" s="17" t="inlineStr">
         <is>
-          <t>TC-TS-02</t>
-        </is>
-      </c>
-      <c r="C205" s="18" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>TC-BL-02</t>
+        </is>
+      </c>
+      <c r="C205" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D205" s="16" t="inlineStr">
         <is>
-          <t>Login sebagai karyawan resto A, baca orders resto B lewat API</t>
+          <t>Buat resto baru, buka Billing Resto</t>
         </is>
       </c>
       <c r="E205" s="16" t="inlineStr">
         <is>
-          <t>Kosong — bukan galat, tapi juga bukan data</t>
+          <t>Sudah punya barisnya sendiri, berstatus Gratis</t>
         </is>
       </c>
       <c r="F205" s="16" t="inlineStr">
         <is>
-          <t>TSD §5</t>
+          <t>F-BL-06</t>
         </is>
       </c>
       <c r="G205" s="16" t="inlineStr"/>
@@ -8869,12 +8900,12 @@
     <row r="206">
       <c r="A206" s="13" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B206" s="14" t="inlineStr">
         <is>
-          <t>TC-TS-03</t>
+          <t>TC-BL-03</t>
         </is>
       </c>
       <c r="C206" s="15" t="inlineStr">
@@ -8884,17 +8915,17 @@
       </c>
       <c r="D206" s="13" t="inlineStr">
         <is>
-          <t>Login sebagai Owner, buka tiap layar resto miliknya</t>
+          <t>Setel harga Rp 0, lewatkan tanggal jatuh tempo jauh</t>
         </is>
       </c>
       <c r="E206" s="13" t="inlineStr">
         <is>
-          <t>Tidak ada layar yang kosong karena RLS — owner harus disebut di setiap daftar peran</t>
+          <t>Tidak pernah terbit tagihan, tidak pernah terkunci</t>
         </is>
       </c>
       <c r="F206" s="13" t="inlineStr">
         <is>
-          <t>TSD §5</t>
+          <t>F-BL-04</t>
         </is>
       </c>
       <c r="G206" s="13" t="inlineStr"/>
@@ -8904,12 +8935,12 @@
     <row r="207">
       <c r="A207" s="16" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B207" s="17" t="inlineStr">
         <is>
-          <t>TC-TS-04</t>
+          <t>TC-BL-04</t>
         </is>
       </c>
       <c r="C207" s="18" t="inlineStr">
@@ -8919,17 +8950,17 @@
       </c>
       <c r="D207" s="16" t="inlineStr">
         <is>
-          <t>Login sebagai Kasir, baca gl_journal_entries</t>
+          <t>Matikan saklar langganan pada resto berbayar yang menunggak</t>
         </is>
       </c>
       <c r="E207" s="16" t="inlineStr">
         <is>
-          <t>Hanya yang terkait catatan yang memang boleh dia lihat</t>
+          <t>Tidak terkunci</t>
         </is>
       </c>
       <c r="F207" s="16" t="inlineStr">
         <is>
-          <t>F-KS-13, TSD §5.1</t>
+          <t>F-BL-05</t>
         </is>
       </c>
       <c r="G207" s="16" t="inlineStr"/>
@@ -8939,32 +8970,32 @@
     <row r="208">
       <c r="A208" s="13" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B208" s="14" t="inlineStr">
         <is>
-          <t>TC-TS-05</t>
-        </is>
-      </c>
-      <c r="C208" s="15" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>TC-BL-05</t>
+        </is>
+      </c>
+      <c r="C208" s="19" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D208" s="13" t="inlineStr">
         <is>
-          <t>Coba UPDATE products langsung lewat API sebagai pelanggan</t>
+          <t>Coba pilih tanggal tagihan 29, 30, atau 31</t>
         </is>
       </c>
       <c r="E208" s="13" t="inlineStr">
         <is>
-          <t>Ditolak; pengurangan stok hanya lewat decrement_stock</t>
+          <t>Tidak tersedia di pilihan — hanya 1 sampai 28</t>
         </is>
       </c>
       <c r="F208" s="13" t="inlineStr">
         <is>
-          <t>TSD §5.2</t>
+          <t>F-BL-02</t>
         </is>
       </c>
       <c r="G208" s="13" t="inlineStr"/>
@@ -8974,32 +9005,32 @@
     <row r="209">
       <c r="A209" s="16" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B209" s="17" t="inlineStr">
         <is>
-          <t>TC-TS-06</t>
-        </is>
-      </c>
-      <c r="C209" s="18" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>TC-BL-06</t>
+        </is>
+      </c>
+      <c r="C209" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D209" s="16" t="inlineStr">
         <is>
-          <t>Panggil cancel_my_order untuk pesanan milik orang lain</t>
+          <t>Ketuk Terbitkan tagihan sekarang dua kali beruntun</t>
         </is>
       </c>
       <c r="E209" s="16" t="inlineStr">
         <is>
-          <t>Ditolak</t>
+          <t>Tagihan tetap satu untuk periode itu</t>
         </is>
       </c>
       <c r="F209" s="16" t="inlineStr">
         <is>
-          <t>TSD §5.2</t>
+          <t>F-BL-08</t>
         </is>
       </c>
       <c r="G209" s="16" t="inlineStr"/>
@@ -9009,12 +9040,12 @@
     <row r="210">
       <c r="A210" s="13" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B210" s="14" t="inlineStr">
         <is>
-          <t>TC-TS-07</t>
+          <t>TC-BL-07</t>
         </is>
       </c>
       <c r="C210" s="15" t="inlineStr">
@@ -9024,17 +9055,17 @@
       </c>
       <c r="D210" s="13" t="inlineStr">
         <is>
-          <t>Jalankan ulang seluruh JALANKAN-INI.sql di database yang sudah terisi</t>
+          <t>Setel jatuh tempo 3 hari lagi, buka aplikasi sebagai Kasir</t>
         </is>
       </c>
       <c r="E210" s="13" t="inlineStr">
         <is>
-          <t>Selesai tanpa galat; tidak ada data yang berubah</t>
+          <t>Pita pengingat tampil di atas layar; isi layarnya tetap bisa dipakai</t>
         </is>
       </c>
       <c r="F210" s="13" t="inlineStr">
         <is>
-          <t>TSD §11</t>
+          <t>F-BL-09</t>
         </is>
       </c>
       <c r="G210" s="13" t="inlineStr"/>
@@ -9044,32 +9075,32 @@
     <row r="211">
       <c r="A211" s="16" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B211" s="17" t="inlineStr">
         <is>
-          <t>TC-TS-08</t>
-        </is>
-      </c>
-      <c r="C211" s="18" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>TC-BL-08</t>
+        </is>
+      </c>
+      <c r="C211" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D211" s="16" t="inlineStr">
         <is>
-          <t>Jalankan ulang satu berkas SQL lama saja, misal cash_payment_expiry.sql</t>
+          <t>Setel jatuh tempo 4 hari lagi</t>
         </is>
       </c>
       <c r="E211" s="16" t="inlineStr">
         <is>
-          <t>Tidak menyempitkan daftar nilai batasan mana pun</t>
+          <t>Pita belum tampil</t>
         </is>
       </c>
       <c r="F211" s="16" t="inlineStr">
         <is>
-          <t>TSD §11.1</t>
+          <t>F-BL-09</t>
         </is>
       </c>
       <c r="G211" s="16" t="inlineStr"/>
@@ -9079,12 +9110,12 @@
     <row r="212">
       <c r="A212" s="13" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B212" s="14" t="inlineStr">
         <is>
-          <t>TC-TS-09</t>
+          <t>TC-BL-09</t>
         </is>
       </c>
       <c r="C212" s="15" t="inlineStr">
@@ -9094,17 +9125,17 @@
       </c>
       <c r="D212" s="13" t="inlineStr">
         <is>
-          <t>Buat resto baru dari Super Admin</t>
+          <t>Lewati jatuh tempo, masih dalam tenggang</t>
         </is>
       </c>
       <c r="E212" s="13" t="inlineStr">
         <is>
-          <t>Bagan akun GL 12 jenis dan tarif PPN/service langsung terisi</t>
+          <t>Pita berubah merah; aplikasi belum terkunci</t>
         </is>
       </c>
       <c r="F212" s="13" t="inlineStr">
         <is>
-          <t>A-19, TSD §6.2</t>
+          <t>F-BL-03, F-BL-10</t>
         </is>
       </c>
       <c r="G212" s="13" t="inlineStr"/>
@@ -9114,12 +9145,12 @@
     <row r="213">
       <c r="A213" s="16" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B213" s="17" t="inlineStr">
         <is>
-          <t>TC-TS-10</t>
+          <t>TC-BL-10</t>
         </is>
       </c>
       <c r="C213" s="18" t="inlineStr">
@@ -9129,17 +9160,17 @@
       </c>
       <c r="D213" s="16" t="inlineStr">
         <is>
-          <t>Kosongkan satu nomor GL, lalu buat transaksi</t>
+          <t>Lewati tenggang, tagihan belum dibayar</t>
         </is>
       </c>
       <c r="E213" s="16" t="inlineStr">
         <is>
-          <t>Jurnal untuk baris itu tidak terbentuk — pastikan gejalanya dikenali penguji</t>
+          <t>Seluruh layar diganti halaman Aplikasi Terkunci Sementara</t>
         </is>
       </c>
       <c r="F213" s="16" t="inlineStr">
         <is>
-          <t>TSD §6.2</t>
+          <t>F-BL-15</t>
         </is>
       </c>
       <c r="G213" s="16" t="inlineStr"/>
@@ -9149,32 +9180,32 @@
     <row r="214">
       <c r="A214" s="13" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B214" s="14" t="inlineStr">
         <is>
-          <t>TC-TS-11</t>
-        </is>
-      </c>
-      <c r="C214" s="19" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-BL-11</t>
+        </is>
+      </c>
+      <c r="C214" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D214" s="13" t="inlineStr">
         <is>
-          <t>Periksa push_outbox sesudah pengumuman terbit</t>
+          <t>Pada keadaan terkunci, coba buat pesanan lewat API langsung</t>
         </is>
       </c>
       <c r="E214" s="13" t="inlineStr">
         <is>
-          <t>Baris masuk, lalu sent_at terisi</t>
+          <t>Ditolak database — bukan hanya layarnya yang menutup</t>
         </is>
       </c>
       <c r="F214" s="13" t="inlineStr">
         <is>
-          <t>TSD §8</t>
+          <t>F-BL-18, TSD §7.3</t>
         </is>
       </c>
       <c r="G214" s="13" t="inlineStr"/>
@@ -9184,32 +9215,32 @@
     <row r="215">
       <c r="A215" s="16" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B215" s="17" t="inlineStr">
         <is>
-          <t>TC-TS-12</t>
-        </is>
-      </c>
-      <c r="C215" s="20" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-BL-12</t>
+        </is>
+      </c>
+      <c r="C215" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D215" s="16" t="inlineStr">
         <is>
-          <t>Matikan sambungan, pakai aplikasi</t>
+          <t>Pada keadaan terkunci, ketuk Lihat &amp; Bayar Tagihan</t>
         </is>
       </c>
       <c r="E215" s="16" t="inlineStr">
         <is>
-          <t>Katalog tetap tampil; pesanan tunai tetap bisa dibuat</t>
+          <t>Layar tagihan terbuka dan bisa dipakai</t>
         </is>
       </c>
       <c r="F215" s="16" t="inlineStr">
         <is>
-          <t>TSD §10, FSD §5.6</t>
+          <t>F-BL-16</t>
         </is>
       </c>
       <c r="G215" s="16" t="inlineStr"/>
@@ -9219,32 +9250,32 @@
     <row r="216">
       <c r="A216" s="13" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B216" s="14" t="inlineStr">
         <is>
-          <t>TC-TS-13</t>
-        </is>
-      </c>
-      <c r="C216" s="19" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-BL-13</t>
+        </is>
+      </c>
+      <c r="C216" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D216" s="13" t="inlineStr">
         <is>
-          <t>Sambungkan lagi</t>
+          <t>Pada keadaan terkunci, ketuk Keluar</t>
         </is>
       </c>
       <c r="E216" s="13" t="inlineStr">
         <is>
-          <t>Pesanan yang dibuat saat luring terkirim</t>
+          <t>Berhasil keluar akun</t>
         </is>
       </c>
       <c r="F216" s="13" t="inlineStr">
         <is>
-          <t>TSD §10</t>
+          <t>F-BL-16</t>
         </is>
       </c>
       <c r="G216" s="13" t="inlineStr"/>
@@ -9254,12 +9285,12 @@
     <row r="217">
       <c r="A217" s="16" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B217" s="17" t="inlineStr">
         <is>
-          <t>TC-TS-14</t>
+          <t>TC-BL-14</t>
         </is>
       </c>
       <c r="C217" s="18" t="inlineStr">
@@ -9269,17 +9300,17 @@
       </c>
       <c r="D217" s="16" t="inlineStr">
         <is>
-          <t>Coba bayar QRIS saat luring</t>
+          <t>Unggah bukti bayar dari layar Tagihan</t>
         </is>
       </c>
       <c r="E217" s="16" t="inlineStr">
         <is>
-          <t>Ditolak dengan jelas — bukan menggantung tanpa kabar</t>
+          <t>Status jadi Menunggu Verifikasi; aplikasi terbuka lagi</t>
         </is>
       </c>
       <c r="F217" s="16" t="inlineStr">
         <is>
-          <t>FSD §5.6</t>
+          <t>F-BL-11, F-BL-12</t>
         </is>
       </c>
       <c r="G217" s="16" t="inlineStr"/>
@@ -9289,12 +9320,12 @@
     <row r="218">
       <c r="A218" s="13" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B218" s="14" t="inlineStr">
         <is>
-          <t>TC-TS-15</t>
+          <t>TC-BL-15</t>
         </is>
       </c>
       <c r="C218" s="15" t="inlineStr">
@@ -9304,17 +9335,17 @@
       </c>
       <c r="D218" s="13" t="inlineStr">
         <is>
-          <t>Panggil create-qris dengan nominal yang dipalsukan di badan permintaan</t>
+          <t>Coba kirim bukti tanpa melampirkan foto</t>
         </is>
       </c>
       <c r="E218" s="13" t="inlineStr">
         <is>
-          <t>Nominal yang dipakai tetap dari basis data</t>
+          <t>Tombol Kirim mati</t>
         </is>
       </c>
       <c r="F218" s="13" t="inlineStr">
         <is>
-          <t>TSD §7.1</t>
+          <t>F-BL-11</t>
         </is>
       </c>
       <c r="G218" s="13" t="inlineStr"/>
@@ -9324,12 +9355,12 @@
     <row r="219">
       <c r="A219" s="16" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B219" s="17" t="inlineStr">
         <is>
-          <t>TC-TS-16</t>
+          <t>TC-BL-16</t>
         </is>
       </c>
       <c r="C219" s="18" t="inlineStr">
@@ -9339,17 +9370,17 @@
       </c>
       <c r="D219" s="16" t="inlineStr">
         <is>
-          <t>Tandai pesanan lunas lewat API tanpa lewat webhook</t>
+          <t>Super Admin → tab Tagihan → Terima</t>
         </is>
       </c>
       <c r="E219" s="16" t="inlineStr">
         <is>
-          <t>Ditolak</t>
+          <t>Status jadi Lunas; resto tetap terbuka; pita hilang</t>
         </is>
       </c>
       <c r="F219" s="16" t="inlineStr">
         <is>
-          <t>F-PG-02, TSD §7.1</t>
+          <t>F-BL-13</t>
         </is>
       </c>
       <c r="G219" s="16" t="inlineStr"/>
@@ -9359,32 +9390,32 @@
     <row r="220">
       <c r="A220" s="13" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B220" s="14" t="inlineStr">
         <is>
-          <t>TC-TS-17</t>
-        </is>
-      </c>
-      <c r="C220" s="19" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-BL-17</t>
+        </is>
+      </c>
+      <c r="C220" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D220" s="13" t="inlineStr">
         <is>
-          <t>Bongkar APK, cari kunci Xendit/FCM/Resend</t>
+          <t>Super Admin → Tolak tanpa mengisi alasan</t>
         </is>
       </c>
       <c r="E220" s="13" t="inlineStr">
         <is>
-          <t>Tidak ada satu pun kunci pengirim di dalamnya</t>
+          <t>Tombol Tolak tidak menyelesaikan apa-apa — alasan wajib</t>
         </is>
       </c>
       <c r="F220" s="13" t="inlineStr">
         <is>
-          <t>TSD §1.2</t>
+          <t>F-BL-14</t>
         </is>
       </c>
       <c r="G220" s="13" t="inlineStr"/>
@@ -9394,32 +9425,32 @@
     <row r="221">
       <c r="A221" s="16" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B221" s="17" t="inlineStr">
         <is>
-          <t>TC-TS-18</t>
-        </is>
-      </c>
-      <c r="C221" s="20" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-BL-18</t>
+        </is>
+      </c>
+      <c r="C221" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D221" s="16" t="inlineStr">
         <is>
-          <t>Pesanan berpindah status lunas lebih dari sekali</t>
+          <t>Tolak berikut alasan, lalu buka layar Tagihan dari sisi resto</t>
         </is>
       </c>
       <c r="E221" s="16" t="inlineStr">
         <is>
-          <t>Jurnalnya tetap satu set — tidak ada baris ganda</t>
+          <t>Alasannya terbaca; kalau sudah lewat tenggang, terkunci lagi</t>
         </is>
       </c>
       <c r="F221" s="16" t="inlineStr">
         <is>
-          <t>TSD §6.5</t>
+          <t>F-BL-14, F-BL-15</t>
         </is>
       </c>
       <c r="G221" s="16" t="inlineStr"/>
@@ -9429,32 +9460,32 @@
     <row r="222">
       <c r="A222" s="13" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B222" s="14" t="inlineStr">
         <is>
-          <t>TC-TS-19</t>
-        </is>
-      </c>
-      <c r="C222" s="19" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-BL-19</t>
+        </is>
+      </c>
+      <c r="C222" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D222" s="13" t="inlineStr">
         <is>
-          <t>Hapus resto uji</t>
+          <t>Login sebagai Super Admin saat ada resto terkunci</t>
         </is>
       </c>
       <c r="E222" s="13" t="inlineStr">
         <is>
-          <t>Seluruh isinya ikut terhapus, termasuk jurnalnya</t>
+          <t>Tidak terkunci sama sekali</t>
         </is>
       </c>
       <c r="F222" s="13" t="inlineStr">
         <is>
-          <t>TSD §4.0</t>
+          <t>F-BL-17</t>
         </is>
       </c>
       <c r="G222" s="13" t="inlineStr"/>
@@ -9464,12 +9495,12 @@
     <row r="223">
       <c r="A223" s="16" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B223" s="17" t="inlineStr">
         <is>
-          <t>TC-RG-01</t>
+          <t>TC-BL-20</t>
         </is>
       </c>
       <c r="C223" s="18" t="inlineStr">
@@ -9479,17 +9510,17 @@
       </c>
       <c r="D223" s="16" t="inlineStr">
         <is>
-          <t>Nominal QRIS kasir memakai subtotal menu, bukan total tagihan</t>
+          <t>Sebagai resto terkunci, coba ubah harga produk</t>
         </is>
       </c>
       <c r="E223" s="16" t="inlineStr">
         <is>
-          <t>Nominal di layar QRIS = total termasuk service dan PPN</t>
+          <t>Ditolak — katalog ikut dibekukan</t>
         </is>
       </c>
       <c r="F223" s="16" t="inlineStr">
         <is>
-          <t>F-KS-09</t>
+          <t>F-BL-18</t>
         </is>
       </c>
       <c r="G223" s="16" t="inlineStr"/>
@@ -9499,12 +9530,12 @@
     <row r="224">
       <c r="A224" s="13" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B224" s="14" t="inlineStr">
         <is>
-          <t>TC-RG-02</t>
+          <t>TC-BL-21</t>
         </is>
       </c>
       <c r="C224" s="15" t="inlineStr">
@@ -9514,17 +9545,17 @@
       </c>
       <c r="D224" s="13" t="inlineStr">
         <is>
-          <t>Pesanan dilunasi lewat QRIS hilang dari Riwayat Kasir</t>
+          <t>Resto A terkunci; buka aplikasi sebagai karyawan resto B</t>
         </is>
       </c>
       <c r="E224" s="13" t="inlineStr">
         <is>
-          <t>Semua cara bayar masuk Riwayat Kasir</t>
+          <t>Resto B tidak terpengaruh</t>
         </is>
       </c>
       <c r="F224" s="13" t="inlineStr">
         <is>
-          <t>F-PP-09, A-13</t>
+          <t>F-BL-15, A-10</t>
         </is>
       </c>
       <c r="G224" s="13" t="inlineStr"/>
@@ -9534,12 +9565,12 @@
     <row r="225">
       <c r="A225" s="16" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B225" s="17" t="inlineStr">
         <is>
-          <t>TC-RG-03</t>
+          <t>TC-BL-22</t>
         </is>
       </c>
       <c r="C225" s="18" t="inlineStr">
@@ -9549,17 +9580,17 @@
       </c>
       <c r="D225" s="16" t="inlineStr">
         <is>
-          <t>Pesanan dibatalkan tampil "Menunggu Pembayaran" di Pesanan Masuk</t>
+          <t>Coba panggil review_billing_payment sebagai Owner resto</t>
         </is>
       </c>
       <c r="E225" s="16" t="inlineStr">
         <is>
-          <t>Tidak muncul sama sekali</t>
+          <t>Ditolak — hanya Super Admin</t>
         </is>
       </c>
       <c r="F225" s="16" t="inlineStr">
         <is>
-          <t>A-17</t>
+          <t>F-BL-13</t>
         </is>
       </c>
       <c r="G225" s="16" t="inlineStr"/>
@@ -9569,12 +9600,12 @@
     <row r="226">
       <c r="A226" s="13" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B226" s="14" t="inlineStr">
         <is>
-          <t>TC-RG-04</t>
+          <t>TC-BL-23</t>
         </is>
       </c>
       <c r="C226" s="15" t="inlineStr">
@@ -9584,17 +9615,17 @@
       </c>
       <c r="D226" s="13" t="inlineStr">
         <is>
-          <t>Top up Rp 100.000 tercatat Rp 200.000 di jurnal</t>
+          <t>Coba UPDATE billing_invoices SET status='paid' sebagai Owner</t>
         </is>
       </c>
       <c r="E226" s="13" t="inlineStr">
         <is>
-          <t>Nominalnya sama dengan yang diajukan</t>
+          <t>Ditolak</t>
         </is>
       </c>
       <c r="F226" s="13" t="inlineStr">
         <is>
-          <t>F-FN-03</t>
+          <t>F-BL-13, TSD §7.3</t>
         </is>
       </c>
       <c r="G226" s="13" t="inlineStr"/>
@@ -9604,32 +9635,32 @@
     <row r="227">
       <c r="A227" s="16" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B227" s="17" t="inlineStr">
         <is>
-          <t>TC-RG-05</t>
-        </is>
-      </c>
-      <c r="C227" s="18" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>TC-BL-24</t>
+        </is>
+      </c>
+      <c r="C227" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D227" s="16" t="inlineStr">
         <is>
-          <t>Diskon tidak berlaku untuk pesanan mandiri pelanggan</t>
+          <t>Matikan sambungan, buka aplikasi resto berbayar yang lancar</t>
         </is>
       </c>
       <c r="E227" s="16" t="inlineStr">
         <is>
-          <t>Berlaku sama di kasir dan HP pelanggan</t>
+          <t>Tidak terkunci karena gagal memeriksa</t>
         </is>
       </c>
       <c r="F227" s="16" t="inlineStr">
         <is>
-          <t>A-14</t>
+          <t>TSD §7.3</t>
         </is>
       </c>
       <c r="G227" s="16" t="inlineStr"/>
@@ -9639,32 +9670,32 @@
     <row r="228">
       <c r="A228" s="13" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B228" s="14" t="inlineStr">
         <is>
-          <t>TC-RG-06</t>
-        </is>
-      </c>
-      <c r="C228" s="15" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>TC-BL-25</t>
+        </is>
+      </c>
+      <c r="C228" s="19" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D228" s="13" t="inlineStr">
         <is>
-          <t>Promo "beli 2" lolos oleh keranjang berisi dua menu berbeda</t>
+          <t>Owner → Tagihan Langganan</t>
         </is>
       </c>
       <c r="E228" s="13" t="inlineStr">
         <is>
-          <t>Syarat jumlah dihitung per menu, dan seluruhnya harus terpenuhi</t>
+          <t>Terbuka, memuat paket dan riwayat tagihan</t>
         </is>
       </c>
       <c r="F228" s="13" t="inlineStr">
         <is>
-          <t>F-DS-10, F-DS-12</t>
+          <t>F-BL-11</t>
         </is>
       </c>
       <c r="G228" s="13" t="inlineStr"/>
@@ -9674,32 +9705,32 @@
     <row r="229">
       <c r="A229" s="16" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>Uji Teknis (lingkup TSD)</t>
         </is>
       </c>
       <c r="B229" s="17" t="inlineStr">
         <is>
-          <t>TC-RG-07</t>
-        </is>
-      </c>
-      <c r="C229" s="20" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-TS-01</t>
+        </is>
+      </c>
+      <c r="C229" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D229" s="16" t="inlineStr">
         <is>
-          <t>Tombol pilih/hapus di kotak masuk tidak bereaksi sama sekali</t>
+          <t>Panggil GET /rest/v1/orders memakai kunci anon tanpa login</t>
         </is>
       </c>
       <c r="E229" s="16" t="inlineStr">
         <is>
-          <t>Bekerja di kotak masuk karyawan dan pelanggan</t>
+          <t>Tidak mengembalikan pesanan resto mana pun</t>
         </is>
       </c>
       <c r="F229" s="16" t="inlineStr">
         <is>
-          <t>F-IN-15</t>
+          <t>TSD §5</t>
         </is>
       </c>
       <c r="G229" s="16" t="inlineStr"/>
@@ -9709,32 +9740,32 @@
     <row r="230">
       <c r="A230" s="13" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>Uji Teknis (lingkup TSD)</t>
         </is>
       </c>
       <c r="B230" s="14" t="inlineStr">
         <is>
-          <t>TC-RG-08</t>
-        </is>
-      </c>
-      <c r="C230" s="19" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-TS-02</t>
+        </is>
+      </c>
+      <c r="C230" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D230" s="13" t="inlineStr">
         <is>
-          <t>Layar Diskon dari hub Kasir menyebut "Belum ada produk di resto ini"</t>
+          <t>Login sebagai karyawan resto A, baca orders resto B lewat API</t>
         </is>
       </c>
       <c r="E230" s="13" t="inlineStr">
         <is>
-          <t>Daftar menu termuat</t>
+          <t>Kosong — bukan galat, tapi juga bukan data</t>
         </is>
       </c>
       <c r="F230" s="13" t="inlineStr">
         <is>
-          <t>F-DS-01</t>
+          <t>TSD §5</t>
         </is>
       </c>
       <c r="G230" s="13" t="inlineStr"/>
@@ -9744,32 +9775,32 @@
     <row r="231">
       <c r="A231" s="16" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>Uji Teknis (lingkup TSD)</t>
         </is>
       </c>
       <c r="B231" s="17" t="inlineStr">
         <is>
-          <t>TC-RG-09</t>
-        </is>
-      </c>
-      <c r="C231" s="20" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-TS-03</t>
+        </is>
+      </c>
+      <c r="C231" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D231" s="16" t="inlineStr">
         <is>
-          <t>Kasir tidak bisa membuka detail jurnal — terlihat seperti GL belum dipetakan</t>
+          <t>Login sebagai Owner, buka tiap layar resto miliknya</t>
         </is>
       </c>
       <c r="E231" s="16" t="inlineStr">
         <is>
-          <t>Detail jurnal terbuka</t>
+          <t>Tidak ada layar yang kosong karena RLS — owner harus disebut di setiap daftar peran</t>
         </is>
       </c>
       <c r="F231" s="16" t="inlineStr">
         <is>
-          <t>F-KS-13</t>
+          <t>TSD §5</t>
         </is>
       </c>
       <c r="G231" s="16" t="inlineStr"/>
@@ -9779,32 +9810,32 @@
     <row r="232">
       <c r="A232" s="13" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>Uji Teknis (lingkup TSD)</t>
         </is>
       </c>
       <c r="B232" s="14" t="inlineStr">
         <is>
-          <t>TC-RG-10</t>
-        </is>
-      </c>
-      <c r="C232" s="19" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-TS-04</t>
+        </is>
+      </c>
+      <c r="C232" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D232" s="13" t="inlineStr">
         <is>
-          <t>Layar dapur meninggalkan jejak warna lama saat tema diganti</t>
+          <t>Login sebagai Kasir, baca gl_journal_entries</t>
         </is>
       </c>
       <c r="E232" s="13" t="inlineStr">
         <is>
-          <t>Seluruh layar berganti bersih</t>
+          <t>Hanya yang terkait catatan yang memang boleh dia lihat</t>
         </is>
       </c>
       <c r="F232" s="13" t="inlineStr">
         <is>
-          <t>A-18</t>
+          <t>F-KS-13, TSD §5.1</t>
         </is>
       </c>
       <c r="G232" s="13" t="inlineStr"/>
@@ -9814,32 +9845,32 @@
     <row r="233">
       <c r="A233" s="16" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>Uji Teknis (lingkup TSD)</t>
         </is>
       </c>
       <c r="B233" s="17" t="inlineStr">
         <is>
-          <t>TC-RG-11</t>
-        </is>
-      </c>
-      <c r="C233" s="20" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-TS-05</t>
+        </is>
+      </c>
+      <c r="C233" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D233" s="16" t="inlineStr">
         <is>
-          <t>Banner promo menempel di atas, tidak ikut tergulir</t>
+          <t>Coba UPDATE products langsung lewat API sebagai pelanggan</t>
         </is>
       </c>
       <c r="E233" s="16" t="inlineStr">
         <is>
-          <t>Ikut tergulir bersama menunya</t>
+          <t>Ditolak; pengurangan stok hanya lewat decrement_stock</t>
         </is>
       </c>
       <c r="F233" s="16" t="inlineStr">
         <is>
-          <t>F-CU-16, A-12</t>
+          <t>TSD §5.2</t>
         </is>
       </c>
       <c r="G233" s="16" t="inlineStr"/>
@@ -9849,32 +9880,32 @@
     <row r="234">
       <c r="A234" s="13" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>Uji Teknis (lingkup TSD)</t>
         </is>
       </c>
       <c r="B234" s="14" t="inlineStr">
         <is>
-          <t>TC-RG-12</t>
-        </is>
-      </c>
-      <c r="C234" s="19" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-TS-06</t>
+        </is>
+      </c>
+      <c r="C234" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D234" s="13" t="inlineStr">
         <is>
-          <t>Owner hanya bisa melihat Info Pembayaran</t>
+          <t>Panggil cancel_my_order untuk pesanan milik orang lain</t>
         </is>
       </c>
       <c r="E234" s="13" t="inlineStr">
         <is>
-          <t>Owner bisa mengubahnya</t>
+          <t>Ditolak</t>
         </is>
       </c>
       <c r="F234" s="13" t="inlineStr">
         <is>
-          <t>F-SD-02</t>
+          <t>TSD §5.2</t>
         </is>
       </c>
       <c r="G234" s="13" t="inlineStr"/>
@@ -9884,12 +9915,12 @@
     <row r="235">
       <c r="A235" s="16" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>Uji Teknis (lingkup TSD)</t>
         </is>
       </c>
       <c r="B235" s="17" t="inlineStr">
         <is>
-          <t>TC-RG-13</t>
+          <t>TC-TS-07</t>
         </is>
       </c>
       <c r="C235" s="18" t="inlineStr">
@@ -9899,17 +9930,17 @@
       </c>
       <c r="D235" s="16" t="inlineStr">
         <is>
-          <t>Migrasi gagal: daftar nilai batasan menyempit saat berkas lama dijalankan ulang</t>
+          <t>Jalankan ulang seluruh JALANKAN-INI.sql di database yang sudah terisi</t>
         </is>
       </c>
       <c r="E235" s="16" t="inlineStr">
         <is>
-          <t>Menjalankan ulang berkas mana pun tidak pernah menolak data yang sudah ada</t>
+          <t>Selesai tanpa galat; tidak ada data yang berubah</t>
         </is>
       </c>
       <c r="F235" s="16" t="inlineStr">
         <is>
-          <t>TSD §11.1</t>
+          <t>TSD §11</t>
         </is>
       </c>
       <c r="G235" s="16" t="inlineStr"/>
@@ -9919,32 +9950,32 @@
     <row r="236">
       <c r="A236" s="13" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>Uji Teknis (lingkup TSD)</t>
         </is>
       </c>
       <c r="B236" s="14" t="inlineStr">
         <is>
-          <t>TC-RG-14</t>
-        </is>
-      </c>
-      <c r="C236" s="19" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-TS-08</t>
+        </is>
+      </c>
+      <c r="C236" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D236" s="13" t="inlineStr">
         <is>
-          <t>QR meja borongan bernomor 07, berbeda dengan mode satu meja</t>
+          <t>Jalankan ulang satu berkas SQL lama saja, misal cash_payment_expiry.sql</t>
         </is>
       </c>
       <c r="E236" s="13" t="inlineStr">
         <is>
-          <t>Keduanya menulis 7</t>
+          <t>Tidak menyempitkan daftar nilai batasan mana pun</t>
         </is>
       </c>
       <c r="F236" s="13" t="inlineStr">
         <is>
-          <t>F-QR-07</t>
+          <t>TSD §11.1</t>
         </is>
       </c>
       <c r="G236" s="13" t="inlineStr"/>
@@ -9954,25 +9985,944 @@
     <row r="237">
       <c r="A237" s="16" t="inlineStr">
         <is>
+          <t>Uji Teknis (lingkup TSD)</t>
+        </is>
+      </c>
+      <c r="B237" s="17" t="inlineStr">
+        <is>
+          <t>TC-TS-09</t>
+        </is>
+      </c>
+      <c r="C237" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D237" s="16" t="inlineStr">
+        <is>
+          <t>Buat resto baru dari Super Admin</t>
+        </is>
+      </c>
+      <c r="E237" s="16" t="inlineStr">
+        <is>
+          <t>Bagan akun GL 12 jenis dan tarif PPN/service langsung terisi</t>
+        </is>
+      </c>
+      <c r="F237" s="16" t="inlineStr">
+        <is>
+          <t>A-19, TSD §6.2</t>
+        </is>
+      </c>
+      <c r="G237" s="16" t="inlineStr"/>
+      <c r="H237" s="16" t="inlineStr"/>
+      <c r="I237" s="16" t="inlineStr"/>
+    </row>
+    <row r="238">
+      <c r="A238" s="13" t="inlineStr">
+        <is>
+          <t>Uji Teknis (lingkup TSD)</t>
+        </is>
+      </c>
+      <c r="B238" s="14" t="inlineStr">
+        <is>
+          <t>TC-TS-10</t>
+        </is>
+      </c>
+      <c r="C238" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D238" s="13" t="inlineStr">
+        <is>
+          <t>Kosongkan satu nomor GL, lalu buat transaksi</t>
+        </is>
+      </c>
+      <c r="E238" s="13" t="inlineStr">
+        <is>
+          <t>Jurnal untuk baris itu tidak terbentuk — pastikan gejalanya dikenali penguji</t>
+        </is>
+      </c>
+      <c r="F238" s="13" t="inlineStr">
+        <is>
+          <t>TSD §6.2</t>
+        </is>
+      </c>
+      <c r="G238" s="13" t="inlineStr"/>
+      <c r="H238" s="13" t="inlineStr"/>
+      <c r="I238" s="13" t="inlineStr"/>
+    </row>
+    <row r="239">
+      <c r="A239" s="16" t="inlineStr">
+        <is>
+          <t>Uji Teknis (lingkup TSD)</t>
+        </is>
+      </c>
+      <c r="B239" s="17" t="inlineStr">
+        <is>
+          <t>TC-TS-11</t>
+        </is>
+      </c>
+      <c r="C239" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D239" s="16" t="inlineStr">
+        <is>
+          <t>Periksa push_outbox sesudah pengumuman terbit</t>
+        </is>
+      </c>
+      <c r="E239" s="16" t="inlineStr">
+        <is>
+          <t>Baris masuk, lalu sent_at terisi</t>
+        </is>
+      </c>
+      <c r="F239" s="16" t="inlineStr">
+        <is>
+          <t>TSD §8</t>
+        </is>
+      </c>
+      <c r="G239" s="16" t="inlineStr"/>
+      <c r="H239" s="16" t="inlineStr"/>
+      <c r="I239" s="16" t="inlineStr"/>
+    </row>
+    <row r="240">
+      <c r="A240" s="13" t="inlineStr">
+        <is>
+          <t>Uji Teknis (lingkup TSD)</t>
+        </is>
+      </c>
+      <c r="B240" s="14" t="inlineStr">
+        <is>
+          <t>TC-TS-12</t>
+        </is>
+      </c>
+      <c r="C240" s="19" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D240" s="13" t="inlineStr">
+        <is>
+          <t>Matikan sambungan, pakai aplikasi</t>
+        </is>
+      </c>
+      <c r="E240" s="13" t="inlineStr">
+        <is>
+          <t>Katalog tetap tampil; pesanan tunai tetap bisa dibuat</t>
+        </is>
+      </c>
+      <c r="F240" s="13" t="inlineStr">
+        <is>
+          <t>TSD §10, FSD §5.6</t>
+        </is>
+      </c>
+      <c r="G240" s="13" t="inlineStr"/>
+      <c r="H240" s="13" t="inlineStr"/>
+      <c r="I240" s="13" t="inlineStr"/>
+    </row>
+    <row r="241">
+      <c r="A241" s="16" t="inlineStr">
+        <is>
+          <t>Uji Teknis (lingkup TSD)</t>
+        </is>
+      </c>
+      <c r="B241" s="17" t="inlineStr">
+        <is>
+          <t>TC-TS-13</t>
+        </is>
+      </c>
+      <c r="C241" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D241" s="16" t="inlineStr">
+        <is>
+          <t>Sambungkan lagi</t>
+        </is>
+      </c>
+      <c r="E241" s="16" t="inlineStr">
+        <is>
+          <t>Pesanan yang dibuat saat luring terkirim</t>
+        </is>
+      </c>
+      <c r="F241" s="16" t="inlineStr">
+        <is>
+          <t>TSD §10</t>
+        </is>
+      </c>
+      <c r="G241" s="16" t="inlineStr"/>
+      <c r="H241" s="16" t="inlineStr"/>
+      <c r="I241" s="16" t="inlineStr"/>
+    </row>
+    <row r="242">
+      <c r="A242" s="13" t="inlineStr">
+        <is>
+          <t>Uji Teknis (lingkup TSD)</t>
+        </is>
+      </c>
+      <c r="B242" s="14" t="inlineStr">
+        <is>
+          <t>TC-TS-14</t>
+        </is>
+      </c>
+      <c r="C242" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D242" s="13" t="inlineStr">
+        <is>
+          <t>Coba bayar QRIS saat luring</t>
+        </is>
+      </c>
+      <c r="E242" s="13" t="inlineStr">
+        <is>
+          <t>Ditolak dengan jelas — bukan menggantung tanpa kabar</t>
+        </is>
+      </c>
+      <c r="F242" s="13" t="inlineStr">
+        <is>
+          <t>FSD §5.6</t>
+        </is>
+      </c>
+      <c r="G242" s="13" t="inlineStr"/>
+      <c r="H242" s="13" t="inlineStr"/>
+      <c r="I242" s="13" t="inlineStr"/>
+    </row>
+    <row r="243">
+      <c r="A243" s="16" t="inlineStr">
+        <is>
+          <t>Uji Teknis (lingkup TSD)</t>
+        </is>
+      </c>
+      <c r="B243" s="17" t="inlineStr">
+        <is>
+          <t>TC-TS-15</t>
+        </is>
+      </c>
+      <c r="C243" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D243" s="16" t="inlineStr">
+        <is>
+          <t>Panggil create-qris dengan nominal yang dipalsukan di badan permintaan</t>
+        </is>
+      </c>
+      <c r="E243" s="16" t="inlineStr">
+        <is>
+          <t>Nominal yang dipakai tetap dari basis data</t>
+        </is>
+      </c>
+      <c r="F243" s="16" t="inlineStr">
+        <is>
+          <t>TSD §7.1</t>
+        </is>
+      </c>
+      <c r="G243" s="16" t="inlineStr"/>
+      <c r="H243" s="16" t="inlineStr"/>
+      <c r="I243" s="16" t="inlineStr"/>
+    </row>
+    <row r="244">
+      <c r="A244" s="13" t="inlineStr">
+        <is>
+          <t>Uji Teknis (lingkup TSD)</t>
+        </is>
+      </c>
+      <c r="B244" s="14" t="inlineStr">
+        <is>
+          <t>TC-TS-16</t>
+        </is>
+      </c>
+      <c r="C244" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D244" s="13" t="inlineStr">
+        <is>
+          <t>Tandai pesanan lunas lewat API tanpa lewat webhook</t>
+        </is>
+      </c>
+      <c r="E244" s="13" t="inlineStr">
+        <is>
+          <t>Ditolak</t>
+        </is>
+      </c>
+      <c r="F244" s="13" t="inlineStr">
+        <is>
+          <t>F-PG-02, TSD §7.1</t>
+        </is>
+      </c>
+      <c r="G244" s="13" t="inlineStr"/>
+      <c r="H244" s="13" t="inlineStr"/>
+      <c r="I244" s="13" t="inlineStr"/>
+    </row>
+    <row r="245">
+      <c r="A245" s="16" t="inlineStr">
+        <is>
+          <t>Uji Teknis (lingkup TSD)</t>
+        </is>
+      </c>
+      <c r="B245" s="17" t="inlineStr">
+        <is>
+          <t>TC-TS-17</t>
+        </is>
+      </c>
+      <c r="C245" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D245" s="16" t="inlineStr">
+        <is>
+          <t>Bongkar APK, cari kunci Xendit/FCM/Resend</t>
+        </is>
+      </c>
+      <c r="E245" s="16" t="inlineStr">
+        <is>
+          <t>Tidak ada satu pun kunci pengirim di dalamnya</t>
+        </is>
+      </c>
+      <c r="F245" s="16" t="inlineStr">
+        <is>
+          <t>TSD §1.2</t>
+        </is>
+      </c>
+      <c r="G245" s="16" t="inlineStr"/>
+      <c r="H245" s="16" t="inlineStr"/>
+      <c r="I245" s="16" t="inlineStr"/>
+    </row>
+    <row r="246">
+      <c r="A246" s="13" t="inlineStr">
+        <is>
+          <t>Uji Teknis (lingkup TSD)</t>
+        </is>
+      </c>
+      <c r="B246" s="14" t="inlineStr">
+        <is>
+          <t>TC-TS-18</t>
+        </is>
+      </c>
+      <c r="C246" s="19" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D246" s="13" t="inlineStr">
+        <is>
+          <t>Pesanan berpindah status lunas lebih dari sekali</t>
+        </is>
+      </c>
+      <c r="E246" s="13" t="inlineStr">
+        <is>
+          <t>Jurnalnya tetap satu set — tidak ada baris ganda</t>
+        </is>
+      </c>
+      <c r="F246" s="13" t="inlineStr">
+        <is>
+          <t>TSD §6.5</t>
+        </is>
+      </c>
+      <c r="G246" s="13" t="inlineStr"/>
+      <c r="H246" s="13" t="inlineStr"/>
+      <c r="I246" s="13" t="inlineStr"/>
+    </row>
+    <row r="247">
+      <c r="A247" s="16" t="inlineStr">
+        <is>
+          <t>Uji Teknis (lingkup TSD)</t>
+        </is>
+      </c>
+      <c r="B247" s="17" t="inlineStr">
+        <is>
+          <t>TC-TS-19</t>
+        </is>
+      </c>
+      <c r="C247" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D247" s="16" t="inlineStr">
+        <is>
+          <t>Hapus resto uji</t>
+        </is>
+      </c>
+      <c r="E247" s="16" t="inlineStr">
+        <is>
+          <t>Seluruh isinya ikut terhapus, termasuk jurnalnya</t>
+        </is>
+      </c>
+      <c r="F247" s="16" t="inlineStr">
+        <is>
+          <t>TSD §4.0</t>
+        </is>
+      </c>
+      <c r="G247" s="16" t="inlineStr"/>
+      <c r="H247" s="16" t="inlineStr"/>
+      <c r="I247" s="16" t="inlineStr"/>
+    </row>
+    <row r="248">
+      <c r="A248" s="13" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B248" s="14" t="inlineStr">
+        <is>
+          <t>TC-RG-01</t>
+        </is>
+      </c>
+      <c r="C248" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D248" s="13" t="inlineStr">
+        <is>
+          <t>Nominal QRIS kasir memakai subtotal menu, bukan total tagihan</t>
+        </is>
+      </c>
+      <c r="E248" s="13" t="inlineStr">
+        <is>
+          <t>Nominal di layar QRIS = total termasuk service dan PPN</t>
+        </is>
+      </c>
+      <c r="F248" s="13" t="inlineStr">
+        <is>
+          <t>F-KS-09</t>
+        </is>
+      </c>
+      <c r="G248" s="13" t="inlineStr"/>
+      <c r="H248" s="13" t="inlineStr"/>
+      <c r="I248" s="13" t="inlineStr"/>
+    </row>
+    <row r="249">
+      <c r="A249" s="16" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B249" s="17" t="inlineStr">
+        <is>
+          <t>TC-RG-02</t>
+        </is>
+      </c>
+      <c r="C249" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D249" s="16" t="inlineStr">
+        <is>
+          <t>Pesanan dilunasi lewat QRIS hilang dari Riwayat Kasir</t>
+        </is>
+      </c>
+      <c r="E249" s="16" t="inlineStr">
+        <is>
+          <t>Semua cara bayar masuk Riwayat Kasir</t>
+        </is>
+      </c>
+      <c r="F249" s="16" t="inlineStr">
+        <is>
+          <t>F-PP-09, A-13</t>
+        </is>
+      </c>
+      <c r="G249" s="16" t="inlineStr"/>
+      <c r="H249" s="16" t="inlineStr"/>
+      <c r="I249" s="16" t="inlineStr"/>
+    </row>
+    <row r="250">
+      <c r="A250" s="13" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B250" s="14" t="inlineStr">
+        <is>
+          <t>TC-RG-03</t>
+        </is>
+      </c>
+      <c r="C250" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D250" s="13" t="inlineStr">
+        <is>
+          <t>Pesanan dibatalkan tampil "Menunggu Pembayaran" di Pesanan Masuk</t>
+        </is>
+      </c>
+      <c r="E250" s="13" t="inlineStr">
+        <is>
+          <t>Tidak muncul sama sekali</t>
+        </is>
+      </c>
+      <c r="F250" s="13" t="inlineStr">
+        <is>
+          <t>A-17</t>
+        </is>
+      </c>
+      <c r="G250" s="13" t="inlineStr"/>
+      <c r="H250" s="13" t="inlineStr"/>
+      <c r="I250" s="13" t="inlineStr"/>
+    </row>
+    <row r="251">
+      <c r="A251" s="16" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B251" s="17" t="inlineStr">
+        <is>
+          <t>TC-RG-04</t>
+        </is>
+      </c>
+      <c r="C251" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D251" s="16" t="inlineStr">
+        <is>
+          <t>Top up Rp 100.000 tercatat Rp 200.000 di jurnal</t>
+        </is>
+      </c>
+      <c r="E251" s="16" t="inlineStr">
+        <is>
+          <t>Nominalnya sama dengan yang diajukan</t>
+        </is>
+      </c>
+      <c r="F251" s="16" t="inlineStr">
+        <is>
+          <t>F-FN-03</t>
+        </is>
+      </c>
+      <c r="G251" s="16" t="inlineStr"/>
+      <c r="H251" s="16" t="inlineStr"/>
+      <c r="I251" s="16" t="inlineStr"/>
+    </row>
+    <row r="252">
+      <c r="A252" s="13" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B252" s="14" t="inlineStr">
+        <is>
+          <t>TC-RG-05</t>
+        </is>
+      </c>
+      <c r="C252" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D252" s="13" t="inlineStr">
+        <is>
+          <t>Diskon tidak berlaku untuk pesanan mandiri pelanggan</t>
+        </is>
+      </c>
+      <c r="E252" s="13" t="inlineStr">
+        <is>
+          <t>Berlaku sama di kasir dan HP pelanggan</t>
+        </is>
+      </c>
+      <c r="F252" s="13" t="inlineStr">
+        <is>
+          <t>A-14</t>
+        </is>
+      </c>
+      <c r="G252" s="13" t="inlineStr"/>
+      <c r="H252" s="13" t="inlineStr"/>
+      <c r="I252" s="13" t="inlineStr"/>
+    </row>
+    <row r="253">
+      <c r="A253" s="16" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B253" s="17" t="inlineStr">
+        <is>
+          <t>TC-RG-06</t>
+        </is>
+      </c>
+      <c r="C253" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D253" s="16" t="inlineStr">
+        <is>
+          <t>Promo "beli 2" lolos oleh keranjang berisi dua menu berbeda</t>
+        </is>
+      </c>
+      <c r="E253" s="16" t="inlineStr">
+        <is>
+          <t>Syarat jumlah dihitung per menu, dan seluruhnya harus terpenuhi</t>
+        </is>
+      </c>
+      <c r="F253" s="16" t="inlineStr">
+        <is>
+          <t>F-DS-10, F-DS-12</t>
+        </is>
+      </c>
+      <c r="G253" s="16" t="inlineStr"/>
+      <c r="H253" s="16" t="inlineStr"/>
+      <c r="I253" s="16" t="inlineStr"/>
+    </row>
+    <row r="254">
+      <c r="A254" s="13" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B254" s="14" t="inlineStr">
+        <is>
+          <t>TC-RG-07</t>
+        </is>
+      </c>
+      <c r="C254" s="19" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D254" s="13" t="inlineStr">
+        <is>
+          <t>Tombol pilih/hapus di kotak masuk tidak bereaksi sama sekali</t>
+        </is>
+      </c>
+      <c r="E254" s="13" t="inlineStr">
+        <is>
+          <t>Bekerja di kotak masuk karyawan dan pelanggan</t>
+        </is>
+      </c>
+      <c r="F254" s="13" t="inlineStr">
+        <is>
+          <t>F-IN-15</t>
+        </is>
+      </c>
+      <c r="G254" s="13" t="inlineStr"/>
+      <c r="H254" s="13" t="inlineStr"/>
+      <c r="I254" s="13" t="inlineStr"/>
+    </row>
+    <row r="255">
+      <c r="A255" s="16" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B255" s="17" t="inlineStr">
+        <is>
+          <t>TC-RG-08</t>
+        </is>
+      </c>
+      <c r="C255" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D255" s="16" t="inlineStr">
+        <is>
+          <t>Layar Diskon dari hub Kasir menyebut "Belum ada produk di resto ini"</t>
+        </is>
+      </c>
+      <c r="E255" s="16" t="inlineStr">
+        <is>
+          <t>Daftar menu termuat</t>
+        </is>
+      </c>
+      <c r="F255" s="16" t="inlineStr">
+        <is>
+          <t>F-DS-01</t>
+        </is>
+      </c>
+      <c r="G255" s="16" t="inlineStr"/>
+      <c r="H255" s="16" t="inlineStr"/>
+      <c r="I255" s="16" t="inlineStr"/>
+    </row>
+    <row r="256">
+      <c r="A256" s="13" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B256" s="14" t="inlineStr">
+        <is>
+          <t>TC-RG-09</t>
+        </is>
+      </c>
+      <c r="C256" s="19" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D256" s="13" t="inlineStr">
+        <is>
+          <t>Kasir tidak bisa membuka detail jurnal — terlihat seperti GL belum dipetakan</t>
+        </is>
+      </c>
+      <c r="E256" s="13" t="inlineStr">
+        <is>
+          <t>Detail jurnal terbuka</t>
+        </is>
+      </c>
+      <c r="F256" s="13" t="inlineStr">
+        <is>
+          <t>F-KS-13</t>
+        </is>
+      </c>
+      <c r="G256" s="13" t="inlineStr"/>
+      <c r="H256" s="13" t="inlineStr"/>
+      <c r="I256" s="13" t="inlineStr"/>
+    </row>
+    <row r="257">
+      <c r="A257" s="16" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B257" s="17" t="inlineStr">
+        <is>
+          <t>TC-RG-10</t>
+        </is>
+      </c>
+      <c r="C257" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D257" s="16" t="inlineStr">
+        <is>
+          <t>Layar dapur meninggalkan jejak warna lama saat tema diganti</t>
+        </is>
+      </c>
+      <c r="E257" s="16" t="inlineStr">
+        <is>
+          <t>Seluruh layar berganti bersih</t>
+        </is>
+      </c>
+      <c r="F257" s="16" t="inlineStr">
+        <is>
+          <t>A-18</t>
+        </is>
+      </c>
+      <c r="G257" s="16" t="inlineStr"/>
+      <c r="H257" s="16" t="inlineStr"/>
+      <c r="I257" s="16" t="inlineStr"/>
+    </row>
+    <row r="258">
+      <c r="A258" s="13" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B258" s="14" t="inlineStr">
+        <is>
+          <t>TC-RG-11</t>
+        </is>
+      </c>
+      <c r="C258" s="19" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D258" s="13" t="inlineStr">
+        <is>
+          <t>Banner promo menempel di atas, tidak ikut tergulir</t>
+        </is>
+      </c>
+      <c r="E258" s="13" t="inlineStr">
+        <is>
+          <t>Ikut tergulir bersama menunya</t>
+        </is>
+      </c>
+      <c r="F258" s="13" t="inlineStr">
+        <is>
+          <t>F-CU-16, A-12</t>
+        </is>
+      </c>
+      <c r="G258" s="13" t="inlineStr"/>
+      <c r="H258" s="13" t="inlineStr"/>
+      <c r="I258" s="13" t="inlineStr"/>
+    </row>
+    <row r="259">
+      <c r="A259" s="16" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B259" s="17" t="inlineStr">
+        <is>
+          <t>TC-RG-12</t>
+        </is>
+      </c>
+      <c r="C259" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D259" s="16" t="inlineStr">
+        <is>
+          <t>Owner hanya bisa melihat Info Pembayaran</t>
+        </is>
+      </c>
+      <c r="E259" s="16" t="inlineStr">
+        <is>
+          <t>Owner bisa mengubahnya</t>
+        </is>
+      </c>
+      <c r="F259" s="16" t="inlineStr">
+        <is>
+          <t>F-SD-02</t>
+        </is>
+      </c>
+      <c r="G259" s="16" t="inlineStr"/>
+      <c r="H259" s="16" t="inlineStr"/>
+      <c r="I259" s="16" t="inlineStr"/>
+    </row>
+    <row r="260">
+      <c r="A260" s="13" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B260" s="14" t="inlineStr">
+        <is>
+          <t>TC-RG-13</t>
+        </is>
+      </c>
+      <c r="C260" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D260" s="13" t="inlineStr">
+        <is>
+          <t>Migrasi gagal: daftar nilai batasan menyempit saat berkas lama dijalankan ulang</t>
+        </is>
+      </c>
+      <c r="E260" s="13" t="inlineStr">
+        <is>
+          <t>Menjalankan ulang berkas mana pun tidak pernah menolak data yang sudah ada</t>
+        </is>
+      </c>
+      <c r="F260" s="13" t="inlineStr">
+        <is>
+          <t>TSD §11.1</t>
+        </is>
+      </c>
+      <c r="G260" s="13" t="inlineStr"/>
+      <c r="H260" s="13" t="inlineStr"/>
+      <c r="I260" s="13" t="inlineStr"/>
+    </row>
+    <row r="261">
+      <c r="A261" s="16" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B261" s="17" t="inlineStr">
+        <is>
+          <t>TC-RG-14</t>
+        </is>
+      </c>
+      <c r="C261" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D261" s="16" t="inlineStr">
+        <is>
+          <t>QR meja borongan bernomor 07, berbeda dengan mode satu meja</t>
+        </is>
+      </c>
+      <c r="E261" s="16" t="inlineStr">
+        <is>
+          <t>Keduanya menulis 7</t>
+        </is>
+      </c>
+      <c r="F261" s="16" t="inlineStr">
+        <is>
+          <t>F-QR-07</t>
+        </is>
+      </c>
+      <c r="G261" s="16" t="inlineStr"/>
+      <c r="H261" s="16" t="inlineStr"/>
+      <c r="I261" s="16" t="inlineStr"/>
+    </row>
+    <row r="262">
+      <c r="A262" s="13" t="inlineStr">
+        <is>
           <t>Uji Ujung-ke-Ujung</t>
         </is>
       </c>
-      <c r="B237" s="17" t="inlineStr">
+      <c r="B262" s="14" t="inlineStr">
+        <is>
+          <t>E2E-09</t>
+        </is>
+      </c>
+      <c r="C262" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D262" s="13" t="inlineStr">
+        <is>
+          <t>Satu siklus langganan penuh</t>
+        </is>
+      </c>
+      <c r="E262" s="13" t="inlineStr">
+        <is>
+          <t>1. Super Admin setel resto uji: Rp 150.000, jatuh tempo 3 hari lagi, tenggang 1 hari
+2. Terbitkan tagihan → periksa muncul di tab Tagihan berstatus Belum Dibayar
+3. Buka aplikasi sebagai Kasir → pita pengingat tampil, layar tetap bisa dipakai
+4. Majukan tanggal melewati jatuh tempo + 1 hari → buka lagi → terkunci
+5. Coba buat pesanan lewat API langsung → ditolak database
+6. Ketuk Lihat &amp; Bayar Tagihan → unggah bukti → status Menunggu Verifikasi
+7. Buka aplikasi lagi → tidak lagi terkunci
+8. Super Admin → Tolak berikut alasan → resto terkunci lagi, alasannya terbaca
+9. Unggah bukti baru → Super Admin → Terima → status Lunas
+10. Buka aplikasi → terbuka, pita hilang</t>
+        </is>
+      </c>
+      <c r="F262" s="13" t="inlineStr">
+        <is>
+          <t>F-BL-07 … F-BL-18, TSD §7.3</t>
+        </is>
+      </c>
+      <c r="G262" s="13" t="inlineStr"/>
+      <c r="H262" s="13" t="inlineStr"/>
+      <c r="I262" s="13" t="inlineStr"/>
+    </row>
+    <row r="263">
+      <c r="A263" s="16" t="inlineStr">
+        <is>
+          <t>Uji Ujung-ke-Ujung</t>
+        </is>
+      </c>
+      <c r="B263" s="17" t="inlineStr">
         <is>
           <t>E2E-01</t>
         </is>
       </c>
-      <c r="C237" s="18" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D237" s="16" t="inlineStr">
+      <c r="C263" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D263" s="16" t="inlineStr">
         <is>
           <t>Pelanggan bayar QRIS</t>
         </is>
       </c>
-      <c r="E237" s="16" t="inlineStr">
+      <c r="E263" s="16" t="inlineStr">
         <is>
           <t>1. Pelanggan scan QR meja → pilih 2 menu → Dine In → isi nama
 2. Pilih QRIS → bayar sungguhan dari aplikasi bank
@@ -9984,37 +10934,37 @@
 8. Periksa Saldo → masuk Non Cash, bukan Cash</t>
         </is>
       </c>
-      <c r="F237" s="16" t="inlineStr">
+      <c r="F263" s="16" t="inlineStr">
         <is>
           <t>F-CU-09, F-PG-02, F-CH-06, TSD §6, TSD §7.1</t>
         </is>
       </c>
-      <c r="G237" s="16" t="inlineStr"/>
-      <c r="H237" s="16" t="inlineStr"/>
-      <c r="I237" s="16" t="inlineStr"/>
-    </row>
-    <row r="238">
-      <c r="A238" s="13" t="inlineStr">
+      <c r="G263" s="16" t="inlineStr"/>
+      <c r="H263" s="16" t="inlineStr"/>
+      <c r="I263" s="16" t="inlineStr"/>
+    </row>
+    <row r="264">
+      <c r="A264" s="13" t="inlineStr">
         <is>
           <t>Uji Ujung-ke-Ujung</t>
         </is>
       </c>
-      <c r="B238" s="14" t="inlineStr">
+      <c r="B264" s="14" t="inlineStr">
         <is>
           <t>E2E-02</t>
         </is>
       </c>
-      <c r="C238" s="15" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D238" s="13" t="inlineStr">
+      <c r="C264" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D264" s="13" t="inlineStr">
         <is>
           <t>Pelanggan bayar tunai di kasir</t>
         </is>
       </c>
-      <c r="E238" s="13" t="inlineStr">
+      <c r="E264" s="13" t="inlineStr">
         <is>
           <t>1. Pelanggan pesan → pilih Tunai → catat nomor pesanannya
 2. Periksa layar pelanggan → hitungan mundur 30 menit berjalan
@@ -10026,74 +10976,74 @@
 8. Periksa Saldo Cash → bertambah sebesar totalnya</t>
         </is>
       </c>
-      <c r="F238" s="13" t="inlineStr">
+      <c r="F264" s="13" t="inlineStr">
         <is>
           <t>F-CU-09, F-PP-01, F-PP-06, F-PP-07, F-CH-06, A-02, A-13</t>
         </is>
       </c>
-      <c r="G238" s="13" t="inlineStr"/>
-      <c r="H238" s="13" t="inlineStr"/>
-      <c r="I238" s="13" t="inlineStr"/>
-    </row>
-    <row r="239">
-      <c r="A239" s="16" t="inlineStr">
+      <c r="G264" s="13" t="inlineStr"/>
+      <c r="H264" s="13" t="inlineStr"/>
+      <c r="I264" s="13" t="inlineStr"/>
+    </row>
+    <row r="265">
+      <c r="A265" s="16" t="inlineStr">
         <is>
           <t>Uji Ujung-ke-Ujung</t>
         </is>
       </c>
-      <c r="B239" s="17" t="inlineStr">
+      <c r="B265" s="17" t="inlineStr">
         <is>
           <t>E2E-03</t>
         </is>
       </c>
-      <c r="C239" s="18" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D239" s="16" t="inlineStr">
+      <c r="C265" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D265" s="16" t="inlineStr">
         <is>
           <t>Tunai dengan cara bayar diganti</t>
         </is>
       </c>
-      <c r="E239" s="16" t="inlineStr">
+      <c r="E265" s="16" t="inlineStr">
         <is>
           <t>1. Ulangi E2E-02, tapi pada langkah 4 ganti cara bayarnya ke QRIS.
 2. Pesanannya harus tetap masuk Riwayat Kasir, dan masuk Non Cash
 3. di Saldo.</t>
         </is>
       </c>
-      <c r="F239" s="16" t="inlineStr">
+      <c r="F265" s="16" t="inlineStr">
         <is>
           <t>F-PP-09, A-13, TSD §4.2</t>
         </is>
       </c>
-      <c r="G239" s="16" t="inlineStr"/>
-      <c r="H239" s="16" t="inlineStr"/>
-      <c r="I239" s="16" t="inlineStr"/>
-    </row>
-    <row r="240">
-      <c r="A240" s="13" t="inlineStr">
+      <c r="G265" s="16" t="inlineStr"/>
+      <c r="H265" s="16" t="inlineStr"/>
+      <c r="I265" s="16" t="inlineStr"/>
+    </row>
+    <row r="266">
+      <c r="A266" s="13" t="inlineStr">
         <is>
           <t>Uji Ujung-ke-Ujung</t>
         </is>
       </c>
-      <c r="B240" s="14" t="inlineStr">
+      <c r="B266" s="14" t="inlineStr">
         <is>
           <t>E2E-04</t>
         </is>
       </c>
-      <c r="C240" s="15" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D240" s="13" t="inlineStr">
+      <c r="C266" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D266" s="13" t="inlineStr">
         <is>
           <t>Setor tunai ke rekening</t>
         </is>
       </c>
-      <c r="E240" s="13" t="inlineStr">
+      <c r="E266" s="13" t="inlineStr">
         <is>
           <t>1. Kasir buka Setor Saldo Cash → catat tunai di laci
 2. Ajukan setoran sebesar sebagian dari itu, lampirkan bukti
@@ -10104,73 +11054,73 @@
 7. Periksa Jurnal GL → titipan suspense dilepas, dana masuk GL Total Saldo</t>
         </is>
       </c>
-      <c r="F240" s="13" t="inlineStr">
+      <c r="F266" s="13" t="inlineStr">
         <is>
           <t>F-SD-01, F-SD-05, A-05, TSD §6.4</t>
         </is>
       </c>
-      <c r="G240" s="13" t="inlineStr"/>
-      <c r="H240" s="13" t="inlineStr"/>
-      <c r="I240" s="13" t="inlineStr"/>
-    </row>
-    <row r="241">
-      <c r="A241" s="16" t="inlineStr">
+      <c r="G266" s="13" t="inlineStr"/>
+      <c r="H266" s="13" t="inlineStr"/>
+      <c r="I266" s="13" t="inlineStr"/>
+    </row>
+    <row r="267">
+      <c r="A267" s="16" t="inlineStr">
         <is>
           <t>Uji Ujung-ke-Ujung</t>
         </is>
       </c>
-      <c r="B241" s="17" t="inlineStr">
+      <c r="B267" s="17" t="inlineStr">
         <is>
           <t>E2E-05</t>
         </is>
       </c>
-      <c r="C241" s="18" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D241" s="16" t="inlineStr">
+      <c r="C267" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D267" s="16" t="inlineStr">
         <is>
           <t>Top up petty cash</t>
         </is>
       </c>
-      <c r="E241" s="16" t="inlineStr">
+      <c r="E267" s="16" t="inlineStr">
         <is>
           <t>1. Sama polanya dengan E2E-04, lewat GL Suspense Petty Cash. Top up
 2. Rp 100.000 harus menambah Petty Cash Rp 100.000 — bukan Rp 200.000.</t>
         </is>
       </c>
-      <c r="F241" s="16" t="inlineStr">
+      <c r="F267" s="16" t="inlineStr">
         <is>
           <t>F-FN-03, TSD §6.4</t>
         </is>
       </c>
-      <c r="G241" s="16" t="inlineStr"/>
-      <c r="H241" s="16" t="inlineStr"/>
-      <c r="I241" s="16" t="inlineStr"/>
-    </row>
-    <row r="242">
-      <c r="A242" s="13" t="inlineStr">
+      <c r="G267" s="16" t="inlineStr"/>
+      <c r="H267" s="16" t="inlineStr"/>
+      <c r="I267" s="16" t="inlineStr"/>
+    </row>
+    <row r="268">
+      <c r="A268" s="13" t="inlineStr">
         <is>
           <t>Uji Ujung-ke-Ujung</t>
         </is>
       </c>
-      <c r="B242" s="14" t="inlineStr">
+      <c r="B268" s="14" t="inlineStr">
         <is>
           <t>E2E-06</t>
         </is>
       </c>
-      <c r="C242" s="15" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D242" s="13" t="inlineStr">
+      <c r="C268" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D268" s="13" t="inlineStr">
         <is>
           <t>Promo bundling dari HP pelanggan</t>
         </is>
       </c>
-      <c r="E242" s="13" t="inlineStr">
+      <c r="E268" s="13" t="inlineStr">
         <is>
           <t>1. Admin buat promo: Nasi Goreng Minimal 2 + Es Teh Minimal 1, potongan 30%
 2. Pelanggan pesan 2 Nasi Goreng saja → tidak ada potongan
@@ -10181,37 +11131,37 @@
 7. Admin hapus promonya → cetak ulang struk tadi → potongannya tetap tertulis</t>
         </is>
       </c>
-      <c r="F242" s="13" t="inlineStr">
+      <c r="F268" s="13" t="inlineStr">
         <is>
           <t>F-DS-10, F-DS-12, F-CU-17, F-DS-08, F-DS-09, A-14</t>
         </is>
       </c>
-      <c r="G242" s="13" t="inlineStr"/>
-      <c r="H242" s="13" t="inlineStr"/>
-      <c r="I242" s="13" t="inlineStr"/>
-    </row>
-    <row r="243">
-      <c r="A243" s="16" t="inlineStr">
+      <c r="G268" s="13" t="inlineStr"/>
+      <c r="H268" s="13" t="inlineStr"/>
+      <c r="I268" s="13" t="inlineStr"/>
+    </row>
+    <row r="269">
+      <c r="A269" s="16" t="inlineStr">
         <is>
           <t>Uji Ujung-ke-Ujung</t>
         </is>
       </c>
-      <c r="B243" s="17" t="inlineStr">
+      <c r="B269" s="17" t="inlineStr">
         <is>
           <t>E2E-07</t>
         </is>
       </c>
-      <c r="C243" s="18" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D243" s="16" t="inlineStr">
+      <c r="C269" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D269" s="16" t="inlineStr">
         <is>
           <t>Pembatalan oleh pelanggan</t>
         </is>
       </c>
-      <c r="E243" s="16" t="inlineStr">
+      <c r="E269" s="16" t="inlineStr">
         <is>
           <t>1. Pelanggan pesan, pilih Tunai
 2. Batalkan dari Pesanan Saya → berhasil
@@ -10221,37 +11171,37 @@
 6. Periksa Riwayat Kasir → tidak ikut terhitung</t>
         </is>
       </c>
-      <c r="F243" s="16" t="inlineStr">
+      <c r="F269" s="16" t="inlineStr">
         <is>
           <t>F-CN-01, A-17</t>
         </is>
       </c>
-      <c r="G243" s="16" t="inlineStr"/>
-      <c r="H243" s="16" t="inlineStr"/>
-      <c r="I243" s="16" t="inlineStr"/>
-    </row>
-    <row r="244">
-      <c r="A244" s="13" t="inlineStr">
+      <c r="G269" s="16" t="inlineStr"/>
+      <c r="H269" s="16" t="inlineStr"/>
+      <c r="I269" s="16" t="inlineStr"/>
+    </row>
+    <row r="270">
+      <c r="A270" s="13" t="inlineStr">
         <is>
           <t>Uji Ujung-ke-Ujung</t>
         </is>
       </c>
-      <c r="B244" s="14" t="inlineStr">
+      <c r="B270" s="14" t="inlineStr">
         <is>
           <t>E2E-08</t>
         </is>
       </c>
-      <c r="C244" s="15" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D244" s="13" t="inlineStr">
+      <c r="C270" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D270" s="13" t="inlineStr">
         <is>
           <t>Isolasi antar cabang</t>
         </is>
       </c>
-      <c r="E244" s="13" t="inlineStr">
+      <c r="E270" s="13" t="inlineStr">
         <is>
           <t>1. Dengan akun Owner yang memiliki dua resto: buat transaksi, promo, dan
 2. pengumuman di resto A, lalu berpindah ke resto B. Tidak satu pun
@@ -10259,19 +11209,19 @@
 4. dan kotak masuk.</t>
         </is>
       </c>
-      <c r="F244" s="13" t="inlineStr">
+      <c r="F270" s="13" t="inlineStr">
         <is>
           <t>F-AD-08, F-IN-10, A-10</t>
         </is>
       </c>
-      <c r="G244" s="13" t="inlineStr"/>
-      <c r="H244" s="13" t="inlineStr"/>
-      <c r="I244" s="13" t="inlineStr"/>
+      <c r="G270" s="13" t="inlineStr"/>
+      <c r="H270" s="13" t="inlineStr"/>
+      <c r="I270" s="13" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I244"/>
+  <autoFilter ref="A1:I270"/>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G244" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G270" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Lulus,Gagal,Terblokir,Dilewati"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Rilis 1.46.2, dan dokumen menyusul temuannya
FSD bertambah 10 kebutuhan untuk Jurnal Semua Resto dan GL Diskon.

TSD 11.1b mencatat pelajarannya: dua layar yang membaca data sama harus
menyebut angka sama. Bentuk kegagalan itu sulit dilihat dari kodenya —
keduanya benar sendiri-sendiri, yang salah cuma kesepakatan di
antaranya, dan yang menemukannya adalah orang yang kebetulan
membandingkan dua angka yang seharusnya cocok.

Batas 1.000 baris pada jurnal lintas resto dicatat sebagai utang
teknis: belum masalah pada 200 baris, tapi kalau terlewati angkanya
akan kurang tanpa terlihat kurang — persis bentuk kesalahan yang baru
saja diperbaiki.

Test case jadi 323 kasus.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/TEST-CASE-KAATAGO.xlsx
+++ b/docs/TEST-CASE-KAATAGO.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cara Lampirkan Capture" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kasus Uji'!$A$1:$I$308</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kasus Uji'!$A$1:$I$324</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Defect'!$A$4:$V$64</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -691,23 +691,23 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIF('Kasus Uji'!C2:C308,"P1")</f>
+        <f>COUNTIF('Kasus Uji'!C2:C324,"P1")</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C308,"P1",'Kasus Uji'!G2:G308,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C324,"P1",'Kasus Uji'!G2:G324,"Lulus")</f>
         <v/>
       </c>
       <c r="D5" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C308,"P1",'Kasus Uji'!G2:G308,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C324,"P1",'Kasus Uji'!G2:G324,"Gagal")</f>
         <v/>
       </c>
       <c r="E5" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C308,"P1",'Kasus Uji'!G2:G308,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C324,"P1",'Kasus Uji'!G2:G324,"Terblokir")</f>
         <v/>
       </c>
       <c r="F5" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C308,"P1",'Kasus Uji'!G2:G308,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C324,"P1",'Kasus Uji'!G2:G324,"Dilewati")</f>
         <v/>
       </c>
       <c r="G5" s="5">
@@ -722,23 +722,23 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('Kasus Uji'!C2:C308,"P2")</f>
+        <f>COUNTIF('Kasus Uji'!C2:C324,"P2")</f>
         <v/>
       </c>
       <c r="C6" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C308,"P2",'Kasus Uji'!G2:G308,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C324,"P2",'Kasus Uji'!G2:G324,"Lulus")</f>
         <v/>
       </c>
       <c r="D6" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C308,"P2",'Kasus Uji'!G2:G308,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C324,"P2",'Kasus Uji'!G2:G324,"Gagal")</f>
         <v/>
       </c>
       <c r="E6" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C308,"P2",'Kasus Uji'!G2:G308,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C324,"P2",'Kasus Uji'!G2:G324,"Terblokir")</f>
         <v/>
       </c>
       <c r="F6" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C308,"P2",'Kasus Uji'!G2:G308,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C324,"P2",'Kasus Uji'!G2:G324,"Dilewati")</f>
         <v/>
       </c>
       <c r="G6" s="5">
@@ -753,23 +753,23 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('Kasus Uji'!C2:C308,"P3")</f>
+        <f>COUNTIF('Kasus Uji'!C2:C324,"P3")</f>
         <v/>
       </c>
       <c r="C7" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C308,"P3",'Kasus Uji'!G2:G308,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C324,"P3",'Kasus Uji'!G2:G324,"Lulus")</f>
         <v/>
       </c>
       <c r="D7" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C308,"P3",'Kasus Uji'!G2:G308,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C324,"P3",'Kasus Uji'!G2:G324,"Gagal")</f>
         <v/>
       </c>
       <c r="E7" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C308,"P3",'Kasus Uji'!G2:G308,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C324,"P3",'Kasus Uji'!G2:G324,"Terblokir")</f>
         <v/>
       </c>
       <c r="F7" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C308,"P3",'Kasus Uji'!G2:G308,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C324,"P3",'Kasus Uji'!G2:G324,"Dilewati")</f>
         <v/>
       </c>
       <c r="G7" s="5">
@@ -859,23 +859,23 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A308,"Pelanggan")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A324,"Pelanggan")</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Pelanggan",'Kasus Uji'!G2:G308,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pelanggan",'Kasus Uji'!G2:G324,"Lulus")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Pelanggan",'Kasus Uji'!G2:G308,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pelanggan",'Kasus Uji'!G2:G324,"Gagal")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Pelanggan",'Kasus Uji'!G2:G308,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pelanggan",'Kasus Uji'!G2:G324,"Terblokir")</f>
         <v/>
       </c>
       <c r="F12" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Pelanggan",'Kasus Uji'!G2:G308,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pelanggan",'Kasus Uji'!G2:G324,"Dilewati")</f>
         <v/>
       </c>
       <c r="G12" s="5">
@@ -890,23 +890,23 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A308,"Kasir")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A324,"Kasir")</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Kasir",'Kasus Uji'!G2:G308,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Kasir",'Kasus Uji'!G2:G324,"Lulus")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Kasir",'Kasus Uji'!G2:G308,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Kasir",'Kasus Uji'!G2:G324,"Gagal")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Kasir",'Kasus Uji'!G2:G308,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Kasir",'Kasus Uji'!G2:G324,"Terblokir")</f>
         <v/>
       </c>
       <c r="F13" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Kasir",'Kasus Uji'!G2:G308,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Kasir",'Kasus Uji'!G2:G324,"Dilewati")</f>
         <v/>
       </c>
       <c r="G13" s="5">
@@ -921,23 +921,23 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A308,"Pending Payment")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A324,"Pending Payment")</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Pending Payment",'Kasus Uji'!G2:G308,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pending Payment",'Kasus Uji'!G2:G324,"Lulus")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Pending Payment",'Kasus Uji'!G2:G308,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pending Payment",'Kasus Uji'!G2:G324,"Gagal")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Pending Payment",'Kasus Uji'!G2:G308,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pending Payment",'Kasus Uji'!G2:G324,"Terblokir")</f>
         <v/>
       </c>
       <c r="F14" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Pending Payment",'Kasus Uji'!G2:G308,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pending Payment",'Kasus Uji'!G2:G324,"Dilewati")</f>
         <v/>
       </c>
       <c r="G14" s="5">
@@ -952,23 +952,23 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A308,"Dapur")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A324,"Dapur")</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Dapur",'Kasus Uji'!G2:G308,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Dapur",'Kasus Uji'!G2:G324,"Lulus")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Dapur",'Kasus Uji'!G2:G308,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Dapur",'Kasus Uji'!G2:G324,"Gagal")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Dapur",'Kasus Uji'!G2:G308,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Dapur",'Kasus Uji'!G2:G324,"Terblokir")</f>
         <v/>
       </c>
       <c r="F15" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Dapur",'Kasus Uji'!G2:G308,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Dapur",'Kasus Uji'!G2:G324,"Dilewati")</f>
         <v/>
       </c>
       <c r="G15" s="5">
@@ -983,23 +983,23 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A308,"Keuangan")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A324,"Keuangan")</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Keuangan",'Kasus Uji'!G2:G308,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Keuangan",'Kasus Uji'!G2:G324,"Lulus")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Keuangan",'Kasus Uji'!G2:G308,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Keuangan",'Kasus Uji'!G2:G324,"Gagal")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Keuangan",'Kasus Uji'!G2:G308,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Keuangan",'Kasus Uji'!G2:G324,"Terblokir")</f>
         <v/>
       </c>
       <c r="F16" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Keuangan",'Kasus Uji'!G2:G308,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Keuangan",'Kasus Uji'!G2:G324,"Dilewati")</f>
         <v/>
       </c>
       <c r="G16" s="5">
@@ -1014,23 +1014,23 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A308,"Setor Saldo Cash")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A324,"Setor Saldo Cash")</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Setor Saldo Cash",'Kasus Uji'!G2:G308,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Setor Saldo Cash",'Kasus Uji'!G2:G324,"Lulus")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Setor Saldo Cash",'Kasus Uji'!G2:G308,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Setor Saldo Cash",'Kasus Uji'!G2:G324,"Gagal")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Setor Saldo Cash",'Kasus Uji'!G2:G308,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Setor Saldo Cash",'Kasus Uji'!G2:G324,"Terblokir")</f>
         <v/>
       </c>
       <c r="F17" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Setor Saldo Cash",'Kasus Uji'!G2:G308,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Setor Saldo Cash",'Kasus Uji'!G2:G324,"Dilewati")</f>
         <v/>
       </c>
       <c r="G17" s="5">
@@ -1045,23 +1045,23 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A308,"Katalog &amp; Pengaturan")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A324,"Katalog &amp; Pengaturan")</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Katalog &amp; Pengaturan",'Kasus Uji'!G2:G308,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Katalog &amp; Pengaturan",'Kasus Uji'!G2:G324,"Lulus")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Katalog &amp; Pengaturan",'Kasus Uji'!G2:G308,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Katalog &amp; Pengaturan",'Kasus Uji'!G2:G324,"Gagal")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Katalog &amp; Pengaturan",'Kasus Uji'!G2:G308,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Katalog &amp; Pengaturan",'Kasus Uji'!G2:G324,"Terblokir")</f>
         <v/>
       </c>
       <c r="F18" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Katalog &amp; Pengaturan",'Kasus Uji'!G2:G308,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Katalog &amp; Pengaturan",'Kasus Uji'!G2:G324,"Dilewati")</f>
         <v/>
       </c>
       <c r="G18" s="5">
@@ -1076,23 +1076,23 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A308,"QR Meja")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A324,"QR Meja")</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"QR Meja",'Kasus Uji'!G2:G308,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"QR Meja",'Kasus Uji'!G2:G324,"Lulus")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"QR Meja",'Kasus Uji'!G2:G308,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"QR Meja",'Kasus Uji'!G2:G324,"Gagal")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"QR Meja",'Kasus Uji'!G2:G308,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"QR Meja",'Kasus Uji'!G2:G324,"Terblokir")</f>
         <v/>
       </c>
       <c r="F19" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"QR Meja",'Kasus Uji'!G2:G308,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"QR Meja",'Kasus Uji'!G2:G324,"Dilewati")</f>
         <v/>
       </c>
       <c r="G19" s="5">
@@ -1107,23 +1107,23 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A308,"Diskon")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A324,"Diskon")</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Diskon",'Kasus Uji'!G2:G308,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Diskon",'Kasus Uji'!G2:G324,"Lulus")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Diskon",'Kasus Uji'!G2:G308,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Diskon",'Kasus Uji'!G2:G324,"Gagal")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Diskon",'Kasus Uji'!G2:G308,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Diskon",'Kasus Uji'!G2:G324,"Terblokir")</f>
         <v/>
       </c>
       <c r="F20" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Diskon",'Kasus Uji'!G2:G308,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Diskon",'Kasus Uji'!G2:G324,"Dilewati")</f>
         <v/>
       </c>
       <c r="G20" s="5">
@@ -1138,23 +1138,23 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A308,"Kotak Masuk &amp; Pengumuman")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A324,"Kotak Masuk &amp; Pengumuman")</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Kotak Masuk &amp; Pengumuman",'Kasus Uji'!G2:G308,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Kotak Masuk &amp; Pengumuman",'Kasus Uji'!G2:G324,"Lulus")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Kotak Masuk &amp; Pengumuman",'Kasus Uji'!G2:G308,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Kotak Masuk &amp; Pengumuman",'Kasus Uji'!G2:G324,"Gagal")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Kotak Masuk &amp; Pengumuman",'Kasus Uji'!G2:G308,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Kotak Masuk &amp; Pengumuman",'Kasus Uji'!G2:G324,"Terblokir")</f>
         <v/>
       </c>
       <c r="F21" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Kotak Masuk &amp; Pengumuman",'Kasus Uji'!G2:G308,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Kotak Masuk &amp; Pengumuman",'Kasus Uji'!G2:G324,"Dilewati")</f>
         <v/>
       </c>
       <c r="G21" s="5">
@@ -1169,23 +1169,23 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A308,"Pembayaran QRIS")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A324,"Pembayaran QRIS")</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Pembayaran QRIS",'Kasus Uji'!G2:G308,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pembayaran QRIS",'Kasus Uji'!G2:G324,"Lulus")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Pembayaran QRIS",'Kasus Uji'!G2:G308,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pembayaran QRIS",'Kasus Uji'!G2:G324,"Gagal")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Pembayaran QRIS",'Kasus Uji'!G2:G308,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pembayaran QRIS",'Kasus Uji'!G2:G324,"Terblokir")</f>
         <v/>
       </c>
       <c r="F22" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Pembayaran QRIS",'Kasus Uji'!G2:G308,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pembayaran QRIS",'Kasus Uji'!G2:G324,"Dilewati")</f>
         <v/>
       </c>
       <c r="G22" s="5">
@@ -1200,23 +1200,23 @@
         </is>
       </c>
       <c r="B23" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A308,"Pembatalan &amp; Kedaluwarsa")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A324,"Pembatalan &amp; Kedaluwarsa")</f>
         <v/>
       </c>
       <c r="C23" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Pembatalan &amp; Kedaluwarsa",'Kasus Uji'!G2:G308,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pembatalan &amp; Kedaluwarsa",'Kasus Uji'!G2:G324,"Lulus")</f>
         <v/>
       </c>
       <c r="D23" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Pembatalan &amp; Kedaluwarsa",'Kasus Uji'!G2:G308,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pembatalan &amp; Kedaluwarsa",'Kasus Uji'!G2:G324,"Gagal")</f>
         <v/>
       </c>
       <c r="E23" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Pembatalan &amp; Kedaluwarsa",'Kasus Uji'!G2:G308,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pembatalan &amp; Kedaluwarsa",'Kasus Uji'!G2:G324,"Terblokir")</f>
         <v/>
       </c>
       <c r="F23" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Pembatalan &amp; Kedaluwarsa",'Kasus Uji'!G2:G308,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pembatalan &amp; Kedaluwarsa",'Kasus Uji'!G2:G324,"Dilewati")</f>
         <v/>
       </c>
       <c r="G23" s="5">
@@ -1231,23 +1231,23 @@
         </is>
       </c>
       <c r="B24" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A308,"Sesi Meja &amp; Identitas")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A324,"Sesi Meja &amp; Identitas")</f>
         <v/>
       </c>
       <c r="C24" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Sesi Meja &amp; Identitas",'Kasus Uji'!G2:G308,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Sesi Meja &amp; Identitas",'Kasus Uji'!G2:G324,"Lulus")</f>
         <v/>
       </c>
       <c r="D24" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Sesi Meja &amp; Identitas",'Kasus Uji'!G2:G308,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Sesi Meja &amp; Identitas",'Kasus Uji'!G2:G324,"Gagal")</f>
         <v/>
       </c>
       <c r="E24" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Sesi Meja &amp; Identitas",'Kasus Uji'!G2:G308,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Sesi Meja &amp; Identitas",'Kasus Uji'!G2:G324,"Terblokir")</f>
         <v/>
       </c>
       <c r="F24" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Sesi Meja &amp; Identitas",'Kasus Uji'!G2:G308,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Sesi Meja &amp; Identitas",'Kasus Uji'!G2:G324,"Dilewati")</f>
         <v/>
       </c>
       <c r="G24" s="5">
@@ -1262,23 +1262,23 @@
         </is>
       </c>
       <c r="B25" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A308,"Tampilan")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A324,"Tampilan")</f>
         <v/>
       </c>
       <c r="C25" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Tampilan",'Kasus Uji'!G2:G308,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Tampilan",'Kasus Uji'!G2:G324,"Lulus")</f>
         <v/>
       </c>
       <c r="D25" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Tampilan",'Kasus Uji'!G2:G308,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Tampilan",'Kasus Uji'!G2:G324,"Gagal")</f>
         <v/>
       </c>
       <c r="E25" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Tampilan",'Kasus Uji'!G2:G308,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Tampilan",'Kasus Uji'!G2:G324,"Terblokir")</f>
         <v/>
       </c>
       <c r="F25" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Tampilan",'Kasus Uji'!G2:G308,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Tampilan",'Kasus Uji'!G2:G324,"Dilewati")</f>
         <v/>
       </c>
       <c r="G25" s="5">
@@ -1293,23 +1293,23 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A308,"Super Admin")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A324,"Super Admin")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Super Admin",'Kasus Uji'!G2:G308,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Super Admin",'Kasus Uji'!G2:G324,"Lulus")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Super Admin",'Kasus Uji'!G2:G308,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Super Admin",'Kasus Uji'!G2:G324,"Gagal")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Super Admin",'Kasus Uji'!G2:G308,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Super Admin",'Kasus Uji'!G2:G324,"Terblokir")</f>
         <v/>
       </c>
       <c r="F26" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Super Admin",'Kasus Uji'!G2:G308,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Super Admin",'Kasus Uji'!G2:G324,"Dilewati")</f>
         <v/>
       </c>
       <c r="G26" s="5">
@@ -1324,23 +1324,23 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A308,"Pembaruan Aplikasi")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A324,"Pembaruan Aplikasi")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Pembaruan Aplikasi",'Kasus Uji'!G2:G308,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pembaruan Aplikasi",'Kasus Uji'!G2:G324,"Lulus")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Pembaruan Aplikasi",'Kasus Uji'!G2:G308,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pembaruan Aplikasi",'Kasus Uji'!G2:G324,"Gagal")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Pembaruan Aplikasi",'Kasus Uji'!G2:G308,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pembaruan Aplikasi",'Kasus Uji'!G2:G324,"Terblokir")</f>
         <v/>
       </c>
       <c r="F27" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Pembaruan Aplikasi",'Kasus Uji'!G2:G308,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pembaruan Aplikasi",'Kasus Uji'!G2:G324,"Dilewati")</f>
         <v/>
       </c>
       <c r="G27" s="5">
@@ -1355,23 +1355,23 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A308,"## 19b. Langganan &amp; Tagihan Resto")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A324,"## 19b. Langganan &amp; Tagihan Resto")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"## 19b. Langganan &amp; Tagihan Resto",'Kasus Uji'!G2:G308,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"## 19b. Langganan &amp; Tagihan Resto",'Kasus Uji'!G2:G324,"Lulus")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"## 19b. Langganan &amp; Tagihan Resto",'Kasus Uji'!G2:G308,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"## 19b. Langganan &amp; Tagihan Resto",'Kasus Uji'!G2:G324,"Gagal")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"## 19b. Langganan &amp; Tagihan Resto",'Kasus Uji'!G2:G308,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"## 19b. Langganan &amp; Tagihan Resto",'Kasus Uji'!G2:G324,"Terblokir")</f>
         <v/>
       </c>
       <c r="F28" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"## 19b. Langganan &amp; Tagihan Resto",'Kasus Uji'!G2:G308,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"## 19b. Langganan &amp; Tagihan Resto",'Kasus Uji'!G2:G324,"Dilewati")</f>
         <v/>
       </c>
       <c r="G28" s="5">
@@ -1386,23 +1386,23 @@
         </is>
       </c>
       <c r="B29" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A308,"## 19c. Finance KaataGo (Super Admin)")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A324,"## 19c. Finance KaataGo (Super Admin)")</f>
         <v/>
       </c>
       <c r="C29" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"## 19c. Finance KaataGo (Super Admin)",'Kasus Uji'!G2:G308,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"## 19c. Finance KaataGo (Super Admin)",'Kasus Uji'!G2:G324,"Lulus")</f>
         <v/>
       </c>
       <c r="D29" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"## 19c. Finance KaataGo (Super Admin)",'Kasus Uji'!G2:G308,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"## 19c. Finance KaataGo (Super Admin)",'Kasus Uji'!G2:G324,"Gagal")</f>
         <v/>
       </c>
       <c r="E29" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"## 19c. Finance KaataGo (Super Admin)",'Kasus Uji'!G2:G308,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"## 19c. Finance KaataGo (Super Admin)",'Kasus Uji'!G2:G324,"Terblokir")</f>
         <v/>
       </c>
       <c r="F29" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"## 19c. Finance KaataGo (Super Admin)",'Kasus Uji'!G2:G308,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"## 19c. Finance KaataGo (Super Admin)",'Kasus Uji'!G2:G324,"Dilewati")</f>
         <v/>
       </c>
       <c r="G29" s="5">
@@ -1417,23 +1417,23 @@
         </is>
       </c>
       <c r="B30" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A308,"Uji Teknis (lingkup TSD)")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A324,"Uji Teknis (lingkup TSD)")</f>
         <v/>
       </c>
       <c r="C30" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Uji Teknis (lingkup TSD)",'Kasus Uji'!G2:G308,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Uji Teknis (lingkup TSD)",'Kasus Uji'!G2:G324,"Lulus")</f>
         <v/>
       </c>
       <c r="D30" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Uji Teknis (lingkup TSD)",'Kasus Uji'!G2:G308,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Uji Teknis (lingkup TSD)",'Kasus Uji'!G2:G324,"Gagal")</f>
         <v/>
       </c>
       <c r="E30" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Uji Teknis (lingkup TSD)",'Kasus Uji'!G2:G308,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Uji Teknis (lingkup TSD)",'Kasus Uji'!G2:G324,"Terblokir")</f>
         <v/>
       </c>
       <c r="F30" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Uji Teknis (lingkup TSD)",'Kasus Uji'!G2:G308,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Uji Teknis (lingkup TSD)",'Kasus Uji'!G2:G324,"Dilewati")</f>
         <v/>
       </c>
       <c r="G30" s="5">
@@ -1448,23 +1448,23 @@
         </is>
       </c>
       <c r="B31" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A308,"Regresi — bug yang pernah terjadi")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A324,"Regresi — bug yang pernah terjadi")</f>
         <v/>
       </c>
       <c r="C31" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Regresi — bug yang pernah terjadi",'Kasus Uji'!G2:G308,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Regresi — bug yang pernah terjadi",'Kasus Uji'!G2:G324,"Lulus")</f>
         <v/>
       </c>
       <c r="D31" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Regresi — bug yang pernah terjadi",'Kasus Uji'!G2:G308,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Regresi — bug yang pernah terjadi",'Kasus Uji'!G2:G324,"Gagal")</f>
         <v/>
       </c>
       <c r="E31" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Regresi — bug yang pernah terjadi",'Kasus Uji'!G2:G308,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Regresi — bug yang pernah terjadi",'Kasus Uji'!G2:G324,"Terblokir")</f>
         <v/>
       </c>
       <c r="F31" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Regresi — bug yang pernah terjadi",'Kasus Uji'!G2:G308,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Regresi — bug yang pernah terjadi",'Kasus Uji'!G2:G324,"Dilewati")</f>
         <v/>
       </c>
       <c r="G31" s="5">
@@ -1479,23 +1479,23 @@
         </is>
       </c>
       <c r="B32" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A308,"Uji Ujung-ke-Ujung")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A324,"Uji Ujung-ke-Ujung")</f>
         <v/>
       </c>
       <c r="C32" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Uji Ujung-ke-Ujung",'Kasus Uji'!G2:G308,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Uji Ujung-ke-Ujung",'Kasus Uji'!G2:G324,"Lulus")</f>
         <v/>
       </c>
       <c r="D32" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Uji Ujung-ke-Ujung",'Kasus Uji'!G2:G308,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Uji Ujung-ke-Ujung",'Kasus Uji'!G2:G324,"Gagal")</f>
         <v/>
       </c>
       <c r="E32" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Uji Ujung-ke-Ujung",'Kasus Uji'!G2:G308,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Uji Ujung-ke-Ujung",'Kasus Uji'!G2:G324,"Terblokir")</f>
         <v/>
       </c>
       <c r="F32" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A308,"Uji Ujung-ke-Ujung",'Kasus Uji'!G2:G308,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A324,"Uji Ujung-ke-Ujung",'Kasus Uji'!G2:G324,"Dilewati")</f>
         <v/>
       </c>
       <c r="G32" s="5">
@@ -1727,7 +1727,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I308"/>
+  <dimension ref="A1:I324"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -10021,27 +10021,27 @@
       </c>
       <c r="B237" s="17" t="inlineStr">
         <is>
-          <t>TC-BL-15</t>
-        </is>
-      </c>
-      <c r="C237" s="18" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>TC-BL-26</t>
+        </is>
+      </c>
+      <c r="C237" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D237" s="16" t="inlineStr">
         <is>
-          <t>Coba kirim bukti tanpa melampirkan foto</t>
+          <t>Dengan kunci uji Xendit, buka tagihan ber-VA</t>
         </is>
       </c>
       <c r="E237" s="16" t="inlineStr">
         <is>
-          <t>Tombol Kirim mati</t>
+          <t>Tombol Simulasikan Pembayaran muncul</t>
         </is>
       </c>
       <c r="F237" s="16" t="inlineStr">
         <is>
-          <t>F-BL-11</t>
+          <t>TSD §7.3</t>
         </is>
       </c>
       <c r="G237" s="16" t="inlineStr"/>
@@ -10056,7 +10056,7 @@
       </c>
       <c r="B238" s="14" t="inlineStr">
         <is>
-          <t>TC-BL-16</t>
+          <t>TC-BL-27</t>
         </is>
       </c>
       <c r="C238" s="15" t="inlineStr">
@@ -10066,17 +10066,17 @@
       </c>
       <c r="D238" s="13" t="inlineStr">
         <is>
-          <t>Super Admin → tab Tagihan → Terima</t>
+          <t>Ketuk Simulasikan Pembayaran</t>
         </is>
       </c>
       <c r="E238" s="13" t="inlineStr">
         <is>
-          <t>Status jadi Lunas; resto tetap terbuka; pita hilang</t>
+          <t>Tagihan jadi Lunas sendiri lewat webhook; kunci resto terbuka</t>
         </is>
       </c>
       <c r="F238" s="13" t="inlineStr">
         <is>
-          <t>F-BL-13</t>
+          <t>F-BL-22</t>
         </is>
       </c>
       <c r="G238" s="13" t="inlineStr"/>
@@ -10091,7 +10091,7 @@
       </c>
       <c r="B239" s="17" t="inlineStr">
         <is>
-          <t>TC-BL-17</t>
+          <t>TC-BL-28</t>
         </is>
       </c>
       <c r="C239" s="18" t="inlineStr">
@@ -10101,17 +10101,17 @@
       </c>
       <c r="D239" s="16" t="inlineStr">
         <is>
-          <t>Super Admin → Tolak tanpa mengisi alasan</t>
+          <t>Pasang kunci produksi Xendit, buka layar yang sama</t>
         </is>
       </c>
       <c r="E239" s="16" t="inlineStr">
         <is>
-          <t>Tombol Tolak tidak menyelesaikan apa-apa — alasan wajib</t>
+          <t>Tombol simulasi hilang sendiri</t>
         </is>
       </c>
       <c r="F239" s="16" t="inlineStr">
         <is>
-          <t>F-BL-14</t>
+          <t>TSD §7.3</t>
         </is>
       </c>
       <c r="G239" s="16" t="inlineStr"/>
@@ -10126,7 +10126,7 @@
       </c>
       <c r="B240" s="14" t="inlineStr">
         <is>
-          <t>TC-BL-18</t>
+          <t>TC-BL-29</t>
         </is>
       </c>
       <c r="C240" s="15" t="inlineStr">
@@ -10136,17 +10136,17 @@
       </c>
       <c r="D240" s="13" t="inlineStr">
         <is>
-          <t>Tolak berikut alasan, lalu buka layar Tagihan dari sisi resto</t>
+          <t>Buat diskon langganan setelah tagihan terbit → ketuk segarkan di Super Admin</t>
         </is>
       </c>
       <c r="E240" s="13" t="inlineStr">
         <is>
-          <t>Alasannya terbaca; kalau sudah lewat tenggang, terkunci lagi</t>
+          <t>Nominal tagihan turun; nomor VA lama dibuang</t>
         </is>
       </c>
       <c r="F240" s="13" t="inlineStr">
         <is>
-          <t>F-BL-14, F-BL-15</t>
+          <t>F-BL-05</t>
         </is>
       </c>
       <c r="G240" s="13" t="inlineStr"/>
@@ -10161,7 +10161,7 @@
       </c>
       <c r="B241" s="17" t="inlineStr">
         <is>
-          <t>TC-BL-19</t>
+          <t>TC-BL-30</t>
         </is>
       </c>
       <c r="C241" s="18" t="inlineStr">
@@ -10171,17 +10171,17 @@
       </c>
       <c r="D241" s="16" t="inlineStr">
         <is>
-          <t>Login sebagai Super Admin saat ada resto terkunci</t>
+          <t>Buat VA baru setelah nominalnya berubah</t>
         </is>
       </c>
       <c r="E241" s="16" t="inlineStr">
         <is>
-          <t>Tidak terkunci sama sekali</t>
+          <t>Nominalnya sesuai yang sudah dipotong</t>
         </is>
       </c>
       <c r="F241" s="16" t="inlineStr">
         <is>
-          <t>F-BL-17</t>
+          <t>F-BL-20</t>
         </is>
       </c>
       <c r="G241" s="16" t="inlineStr"/>
@@ -10196,7 +10196,7 @@
       </c>
       <c r="B242" s="14" t="inlineStr">
         <is>
-          <t>TC-BL-20</t>
+          <t>TC-BL-15</t>
         </is>
       </c>
       <c r="C242" s="15" t="inlineStr">
@@ -10206,17 +10206,17 @@
       </c>
       <c r="D242" s="13" t="inlineStr">
         <is>
-          <t>Sebagai resto terkunci, coba ubah harga produk</t>
+          <t>Coba kirim bukti tanpa melampirkan foto</t>
         </is>
       </c>
       <c r="E242" s="13" t="inlineStr">
         <is>
-          <t>Ditolak — katalog ikut dibekukan</t>
+          <t>Tombol Kirim mati</t>
         </is>
       </c>
       <c r="F242" s="13" t="inlineStr">
         <is>
-          <t>F-BL-18</t>
+          <t>F-BL-11</t>
         </is>
       </c>
       <c r="G242" s="13" t="inlineStr"/>
@@ -10231,7 +10231,7 @@
       </c>
       <c r="B243" s="17" t="inlineStr">
         <is>
-          <t>TC-BL-21</t>
+          <t>TC-BL-16</t>
         </is>
       </c>
       <c r="C243" s="18" t="inlineStr">
@@ -10241,17 +10241,17 @@
       </c>
       <c r="D243" s="16" t="inlineStr">
         <is>
-          <t>Resto A terkunci; buka aplikasi sebagai karyawan resto B</t>
+          <t>Super Admin → tab Tagihan → Terima</t>
         </is>
       </c>
       <c r="E243" s="16" t="inlineStr">
         <is>
-          <t>Resto B tidak terpengaruh</t>
+          <t>Status jadi Lunas; resto tetap terbuka; pita hilang</t>
         </is>
       </c>
       <c r="F243" s="16" t="inlineStr">
         <is>
-          <t>F-BL-15, A-10</t>
+          <t>F-BL-13</t>
         </is>
       </c>
       <c r="G243" s="16" t="inlineStr"/>
@@ -10266,7 +10266,7 @@
       </c>
       <c r="B244" s="14" t="inlineStr">
         <is>
-          <t>TC-BL-22</t>
+          <t>TC-BL-17</t>
         </is>
       </c>
       <c r="C244" s="15" t="inlineStr">
@@ -10276,17 +10276,17 @@
       </c>
       <c r="D244" s="13" t="inlineStr">
         <is>
-          <t>Coba panggil review_billing_payment sebagai Owner resto</t>
+          <t>Super Admin → Tolak tanpa mengisi alasan</t>
         </is>
       </c>
       <c r="E244" s="13" t="inlineStr">
         <is>
-          <t>Ditolak — hanya Super Admin</t>
+          <t>Tombol Tolak tidak menyelesaikan apa-apa — alasan wajib</t>
         </is>
       </c>
       <c r="F244" s="13" t="inlineStr">
         <is>
-          <t>F-BL-13</t>
+          <t>F-BL-14</t>
         </is>
       </c>
       <c r="G244" s="13" t="inlineStr"/>
@@ -10301,7 +10301,7 @@
       </c>
       <c r="B245" s="17" t="inlineStr">
         <is>
-          <t>TC-BL-23</t>
+          <t>TC-BL-18</t>
         </is>
       </c>
       <c r="C245" s="18" t="inlineStr">
@@ -10311,17 +10311,17 @@
       </c>
       <c r="D245" s="16" t="inlineStr">
         <is>
-          <t>Coba UPDATE billing_invoices SET status='paid' sebagai Owner</t>
+          <t>Tolak berikut alasan, lalu buka layar Tagihan dari sisi resto</t>
         </is>
       </c>
       <c r="E245" s="16" t="inlineStr">
         <is>
-          <t>Ditolak</t>
+          <t>Alasannya terbaca; kalau sudah lewat tenggang, terkunci lagi</t>
         </is>
       </c>
       <c r="F245" s="16" t="inlineStr">
         <is>
-          <t>F-BL-13, TSD §7.3</t>
+          <t>F-BL-14, F-BL-15</t>
         </is>
       </c>
       <c r="G245" s="16" t="inlineStr"/>
@@ -10336,27 +10336,27 @@
       </c>
       <c r="B246" s="14" t="inlineStr">
         <is>
-          <t>TC-BL-24</t>
-        </is>
-      </c>
-      <c r="C246" s="19" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-BL-19</t>
+        </is>
+      </c>
+      <c r="C246" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D246" s="13" t="inlineStr">
         <is>
-          <t>Matikan sambungan, buka aplikasi resto berbayar yang lancar</t>
+          <t>Login sebagai Super Admin saat ada resto terkunci</t>
         </is>
       </c>
       <c r="E246" s="13" t="inlineStr">
         <is>
-          <t>Tidak terkunci karena gagal memeriksa</t>
+          <t>Tidak terkunci sama sekali</t>
         </is>
       </c>
       <c r="F246" s="13" t="inlineStr">
         <is>
-          <t>TSD §7.3</t>
+          <t>F-BL-17</t>
         </is>
       </c>
       <c r="G246" s="13" t="inlineStr"/>
@@ -10371,27 +10371,27 @@
       </c>
       <c r="B247" s="17" t="inlineStr">
         <is>
-          <t>TC-BL-25</t>
-        </is>
-      </c>
-      <c r="C247" s="20" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-BL-20</t>
+        </is>
+      </c>
+      <c r="C247" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D247" s="16" t="inlineStr">
         <is>
-          <t>Owner → Tagihan Langganan</t>
+          <t>Sebagai resto terkunci, coba ubah harga produk</t>
         </is>
       </c>
       <c r="E247" s="16" t="inlineStr">
         <is>
-          <t>Terbuka, memuat paket dan riwayat tagihan</t>
+          <t>Ditolak — katalog ikut dibekukan</t>
         </is>
       </c>
       <c r="F247" s="16" t="inlineStr">
         <is>
-          <t>F-BL-11</t>
+          <t>F-BL-18</t>
         </is>
       </c>
       <c r="G247" s="16" t="inlineStr"/>
@@ -10401,12 +10401,12 @@
     <row r="248">
       <c r="A248" s="13" t="inlineStr">
         <is>
-          <t>## 19c. Finance KaataGo (Super Admin)</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B248" s="14" t="inlineStr">
         <is>
-          <t>TC-PF-01</t>
+          <t>TC-BL-21</t>
         </is>
       </c>
       <c r="C248" s="15" t="inlineStr">
@@ -10416,17 +10416,17 @@
       </c>
       <c r="D248" s="13" t="inlineStr">
         <is>
-          <t>Super Admin → Finance → Riwayat Langganan</t>
+          <t>Resto A terkunci; buka aplikasi sebagai karyawan resto B</t>
         </is>
       </c>
       <c r="E248" s="13" t="inlineStr">
         <is>
-          <t>Tagihan lunas tampil, dikelompokkan per bulan, dengan total</t>
+          <t>Resto B tidak terpengaruh</t>
         </is>
       </c>
       <c r="F248" s="13" t="inlineStr">
         <is>
-          <t>F-PF-01</t>
+          <t>F-BL-15, A-10</t>
         </is>
       </c>
       <c r="G248" s="13" t="inlineStr"/>
@@ -10436,32 +10436,32 @@
     <row r="249">
       <c r="A249" s="16" t="inlineStr">
         <is>
-          <t>## 19c. Finance KaataGo (Super Admin)</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B249" s="17" t="inlineStr">
         <is>
-          <t>TC-PF-02</t>
-        </is>
-      </c>
-      <c r="C249" s="20" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-BL-22</t>
+        </is>
+      </c>
+      <c r="C249" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D249" s="16" t="inlineStr">
         <is>
-          <t>Periksa penanda jalur pelunasan tiap baris</t>
+          <t>Coba panggil review_billing_payment sebagai Owner resto</t>
         </is>
       </c>
       <c r="E249" s="16" t="inlineStr">
         <is>
-          <t>Tertulis VA atau manual sesuai cara lunasnya</t>
+          <t>Ditolak — hanya Super Admin</t>
         </is>
       </c>
       <c r="F249" s="16" t="inlineStr">
         <is>
-          <t>F-PF-02</t>
+          <t>F-BL-13</t>
         </is>
       </c>
       <c r="G249" s="16" t="inlineStr"/>
@@ -10471,12 +10471,12 @@
     <row r="250">
       <c r="A250" s="13" t="inlineStr">
         <is>
-          <t>## 19c. Finance KaataGo (Super Admin)</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B250" s="14" t="inlineStr">
         <is>
-          <t>TC-PF-03</t>
+          <t>TC-BL-23</t>
         </is>
       </c>
       <c r="C250" s="15" t="inlineStr">
@@ -10486,17 +10486,17 @@
       </c>
       <c r="D250" s="13" t="inlineStr">
         <is>
-          <t>Buat diskon langganan 20% untuk satu resto → terbitkan tagihan</t>
+          <t>Coba UPDATE billing_invoices SET status='paid' sebagai Owner</t>
         </is>
       </c>
       <c r="E250" s="13" t="inlineStr">
         <is>
-          <t>Tagihan resto itu berkurang 20%; resto lain tetap penuh</t>
+          <t>Ditolak</t>
         </is>
       </c>
       <c r="F250" s="13" t="inlineStr">
         <is>
-          <t>F-PF-03, F-PF-05</t>
+          <t>F-BL-13, TSD §7.3</t>
         </is>
       </c>
       <c r="G250" s="13" t="inlineStr"/>
@@ -10506,32 +10506,32 @@
     <row r="251">
       <c r="A251" s="16" t="inlineStr">
         <is>
-          <t>## 19c. Finance KaataGo (Super Admin)</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B251" s="17" t="inlineStr">
         <is>
-          <t>TC-PF-04</t>
-        </is>
-      </c>
-      <c r="C251" s="18" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>TC-BL-24</t>
+        </is>
+      </c>
+      <c r="C251" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D251" s="16" t="inlineStr">
         <is>
-          <t>Simpan diskon tanpa memilih resto</t>
+          <t>Matikan sambungan, buka aplikasi resto berbayar yang lancar</t>
         </is>
       </c>
       <c r="E251" s="16" t="inlineStr">
         <is>
-          <t>Ditolak — diskon tanpa sasaran tidak mengenai siapa pun</t>
+          <t>Tidak terkunci karena gagal memeriksa</t>
         </is>
       </c>
       <c r="F251" s="16" t="inlineStr">
         <is>
-          <t>F-PF-03</t>
+          <t>TSD §7.3</t>
         </is>
       </c>
       <c r="G251" s="16" t="inlineStr"/>
@@ -10541,12 +10541,12 @@
     <row r="252">
       <c r="A252" s="13" t="inlineStr">
         <is>
-          <t>## 19c. Finance KaataGo (Super Admin)</t>
+          <t>## 19b. Langganan &amp; Tagihan Resto</t>
         </is>
       </c>
       <c r="B252" s="14" t="inlineStr">
         <is>
-          <t>TC-PF-05</t>
+          <t>TC-BL-25</t>
         </is>
       </c>
       <c r="C252" s="19" t="inlineStr">
@@ -10556,17 +10556,17 @@
       </c>
       <c r="D252" s="13" t="inlineStr">
         <is>
-          <t>Buat diskon rupiah lebih besar daripada harga langganan</t>
+          <t>Owner → Tagihan Langganan</t>
         </is>
       </c>
       <c r="E252" s="13" t="inlineStr">
         <is>
-          <t>Potongannya berhenti di harga; tagihan tidak pernah negatif</t>
+          <t>Terbuka, memuat paket dan riwayat tagihan</t>
         </is>
       </c>
       <c r="F252" s="13" t="inlineStr">
         <is>
-          <t>F-PF-03</t>
+          <t>F-BL-11</t>
         </is>
       </c>
       <c r="G252" s="13" t="inlineStr"/>
@@ -10581,27 +10581,27 @@
       </c>
       <c r="B253" s="17" t="inlineStr">
         <is>
-          <t>TC-PF-06</t>
-        </is>
-      </c>
-      <c r="C253" s="20" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-PF-01</t>
+        </is>
+      </c>
+      <c r="C253" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D253" s="16" t="inlineStr">
         <is>
-          <t>Nonaktifkan diskon, terbitkan tagihan berikutnya</t>
+          <t>Super Admin → Finance → Riwayat Langganan</t>
         </is>
       </c>
       <c r="E253" s="16" t="inlineStr">
         <is>
-          <t>Tidak memotong; diskonnya tetap ada di daftar</t>
+          <t>Tagihan lunas tampil, dikelompokkan per bulan, dengan total</t>
         </is>
       </c>
       <c r="F253" s="16" t="inlineStr">
         <is>
-          <t>F-PF-04</t>
+          <t>F-PF-01</t>
         </is>
       </c>
       <c r="G253" s="16" t="inlineStr"/>
@@ -10616,27 +10616,27 @@
       </c>
       <c r="B254" s="14" t="inlineStr">
         <is>
-          <t>TC-PF-07</t>
-        </is>
-      </c>
-      <c r="C254" s="15" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>TC-PF-02</t>
+        </is>
+      </c>
+      <c r="C254" s="19" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D254" s="13" t="inlineStr">
         <is>
-          <t>Hapus diskon setelah tagihan terbit</t>
+          <t>Periksa penanda jalur pelunasan tiap baris</t>
         </is>
       </c>
       <c r="E254" s="13" t="inlineStr">
         <is>
-          <t>Tagihan yang sudah terbit tetap menyebut potongannya</t>
+          <t>Tertulis VA atau manual sesuai cara lunasnya</t>
         </is>
       </c>
       <c r="F254" s="13" t="inlineStr">
         <is>
-          <t>F-PF-05</t>
+          <t>F-PF-02</t>
         </is>
       </c>
       <c r="G254" s="13" t="inlineStr"/>
@@ -10651,7 +10651,7 @@
       </c>
       <c r="B255" s="17" t="inlineStr">
         <is>
-          <t>TC-PF-08</t>
+          <t>TC-PF-03</t>
         </is>
       </c>
       <c r="C255" s="18" t="inlineStr">
@@ -10661,17 +10661,17 @@
       </c>
       <c r="D255" s="16" t="inlineStr">
         <is>
-          <t>Bayar tagihan berdiskon → buka Jurnal GL KaataGo</t>
+          <t>Buat diskon langganan 20% untuk satu resto → terbitkan tagihan</t>
         </is>
       </c>
       <c r="E255" s="16" t="inlineStr">
         <is>
-          <t>Dua baris: pendapatan kredit, diskon debit</t>
+          <t>Tagihan resto itu berkurang 20%; resto lain tetap penuh</t>
         </is>
       </c>
       <c r="F255" s="16" t="inlineStr">
         <is>
-          <t>F-PF-06, F-PF-07</t>
+          <t>F-PF-03, F-PF-05</t>
         </is>
       </c>
       <c r="G255" s="16" t="inlineStr"/>
@@ -10686,7 +10686,7 @@
       </c>
       <c r="B256" s="14" t="inlineStr">
         <is>
-          <t>TC-PF-09</t>
+          <t>TC-PF-04</t>
         </is>
       </c>
       <c r="C256" s="15" t="inlineStr">
@@ -10696,17 +10696,17 @@
       </c>
       <c r="D256" s="13" t="inlineStr">
         <is>
-          <t>Tagihan ditolak lalu diterima lagi</t>
+          <t>Simpan diskon tanpa memilih resto</t>
         </is>
       </c>
       <c r="E256" s="13" t="inlineStr">
         <is>
-          <t>Jurnalnya tetap satu set — pendapatan tidak tercatat dua kali</t>
+          <t>Ditolak — diskon tanpa sasaran tidak mengenai siapa pun</t>
         </is>
       </c>
       <c r="F256" s="13" t="inlineStr">
         <is>
-          <t>F-PF-07</t>
+          <t>F-PF-03</t>
         </is>
       </c>
       <c r="G256" s="13" t="inlineStr"/>
@@ -10721,27 +10721,27 @@
       </c>
       <c r="B257" s="17" t="inlineStr">
         <is>
-          <t>TC-PF-10</t>
-        </is>
-      </c>
-      <c r="C257" s="18" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>TC-PF-05</t>
+        </is>
+      </c>
+      <c r="C257" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D257" s="16" t="inlineStr">
         <is>
-          <t>Buka Jurnal GL resto yang membayar</t>
+          <t>Buat diskon rupiah lebih besar daripada harga langganan</t>
         </is>
       </c>
       <c r="E257" s="16" t="inlineStr">
         <is>
-          <t>Tidak ada baris pendapatan langganan di sana</t>
+          <t>Potongannya berhenti di harga; tagihan tidak pernah negatif</t>
         </is>
       </c>
       <c r="F257" s="16" t="inlineStr">
         <is>
-          <t>F-PF-07</t>
+          <t>F-PF-03</t>
         </is>
       </c>
       <c r="G257" s="16" t="inlineStr"/>
@@ -10756,7 +10756,7 @@
       </c>
       <c r="B258" s="14" t="inlineStr">
         <is>
-          <t>TC-PF-11</t>
+          <t>TC-PF-06</t>
         </is>
       </c>
       <c r="C258" s="19" t="inlineStr">
@@ -10766,17 +10766,17 @@
       </c>
       <c r="D258" s="13" t="inlineStr">
         <is>
-          <t>Buka Mapping GL Account KaataGo</t>
+          <t>Nonaktifkan diskon, terbitkan tagihan berikutnya</t>
         </is>
       </c>
       <c r="E258" s="13" t="inlineStr">
         <is>
-          <t>Bagan akun 11xxxxx lengkap, berbeda dari 19xxxxx milik resto</t>
+          <t>Tidak memotong; diskonnya tetap ada di daftar</t>
         </is>
       </c>
       <c r="F258" s="13" t="inlineStr">
         <is>
-          <t>F-PF-08</t>
+          <t>F-PF-04</t>
         </is>
       </c>
       <c r="G258" s="13" t="inlineStr"/>
@@ -10791,27 +10791,27 @@
       </c>
       <c r="B259" s="17" t="inlineStr">
         <is>
-          <t>TC-PF-12</t>
-        </is>
-      </c>
-      <c r="C259" s="20" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-PF-07</t>
+        </is>
+      </c>
+      <c r="C259" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D259" s="16" t="inlineStr">
         <is>
-          <t>Catat pengeluaran dan top up petty cash KaataGo</t>
+          <t>Hapus diskon setelah tagihan terbit</t>
         </is>
       </c>
       <c r="E259" s="16" t="inlineStr">
         <is>
-          <t>Bekerja sama seperti di resto</t>
+          <t>Tagihan yang sudah terbit tetap menyebut potongannya</t>
         </is>
       </c>
       <c r="F259" s="16" t="inlineStr">
         <is>
-          <t>F-PF-09</t>
+          <t>F-PF-05</t>
         </is>
       </c>
       <c r="G259" s="16" t="inlineStr"/>
@@ -10826,7 +10826,7 @@
       </c>
       <c r="B260" s="14" t="inlineStr">
         <is>
-          <t>TC-PF-13</t>
+          <t>TC-PF-08</t>
         </is>
       </c>
       <c r="C260" s="15" t="inlineStr">
@@ -10836,17 +10836,17 @@
       </c>
       <c r="D260" s="13" t="inlineStr">
         <is>
-          <t>Telusuri menu Finance KaataGo</t>
+          <t>Bayar tagihan berdiskon → buka Jurnal GL KaataGo</t>
         </is>
       </c>
       <c r="E260" s="13" t="inlineStr">
         <is>
-          <t>Tidak ada Setor Saldo Cash</t>
+          <t>Dua baris: pendapatan kredit, diskon debit</t>
         </is>
       </c>
       <c r="F260" s="13" t="inlineStr">
         <is>
-          <t>F-PF-10</t>
+          <t>F-PF-06, F-PF-07</t>
         </is>
       </c>
       <c r="G260" s="13" t="inlineStr"/>
@@ -10861,7 +10861,7 @@
       </c>
       <c r="B261" s="17" t="inlineStr">
         <is>
-          <t>TC-PF-14</t>
+          <t>TC-PF-09</t>
         </is>
       </c>
       <c r="C261" s="18" t="inlineStr">
@@ -10871,17 +10871,17 @@
       </c>
       <c r="D261" s="16" t="inlineStr">
         <is>
-          <t>Buka Jurnal GL Semua Resto</t>
+          <t>Tagihan ditolak lalu diterima lagi</t>
         </is>
       </c>
       <c r="E261" s="16" t="inlineStr">
         <is>
-          <t>Jurnal seluruh resto tampil, bisa disaring per resto</t>
+          <t>Jurnalnya tetap satu set — pendapatan tidak tercatat dua kali</t>
         </is>
       </c>
       <c r="F261" s="16" t="inlineStr">
         <is>
-          <t>F-PF-11</t>
+          <t>F-PF-07</t>
         </is>
       </c>
       <c r="G261" s="16" t="inlineStr"/>
@@ -10896,7 +10896,7 @@
       </c>
       <c r="B262" s="14" t="inlineStr">
         <is>
-          <t>TC-PF-15</t>
+          <t>TC-PF-10</t>
         </is>
       </c>
       <c r="C262" s="15" t="inlineStr">
@@ -10906,17 +10906,17 @@
       </c>
       <c r="D262" s="13" t="inlineStr">
         <is>
-          <t>Cari cara mengubah baris di Jurnal GL Semua Resto</t>
+          <t>Buka Jurnal GL resto yang membayar</t>
         </is>
       </c>
       <c r="E262" s="13" t="inlineStr">
         <is>
-          <t>Tidak ada satu pun — hanya bisa dilihat</t>
+          <t>Tidak ada baris pendapatan langganan di sana</t>
         </is>
       </c>
       <c r="F262" s="13" t="inlineStr">
         <is>
-          <t>F-PF-12</t>
+          <t>F-PF-07</t>
         </is>
       </c>
       <c r="G262" s="13" t="inlineStr"/>
@@ -10931,27 +10931,27 @@
       </c>
       <c r="B263" s="17" t="inlineStr">
         <is>
-          <t>TC-PF-16</t>
-        </is>
-      </c>
-      <c r="C263" s="18" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>TC-PF-11</t>
+        </is>
+      </c>
+      <c r="C263" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D263" s="16" t="inlineStr">
         <is>
-          <t>Coba UPDATE gl_journal_entries sebagai Super Admin lewat API</t>
+          <t>Buka Mapping GL Account KaataGo</t>
         </is>
       </c>
       <c r="E263" s="16" t="inlineStr">
         <is>
-          <t>Ditolak</t>
+          <t>Bagan akun 11xxxxx lengkap, berbeda dari 19xxxxx milik resto</t>
         </is>
       </c>
       <c r="F263" s="16" t="inlineStr">
         <is>
-          <t>F-PF-12, TSD §7.4</t>
+          <t>F-PF-08</t>
         </is>
       </c>
       <c r="G263" s="16" t="inlineStr"/>
@@ -10966,27 +10966,27 @@
       </c>
       <c r="B264" s="14" t="inlineStr">
         <is>
-          <t>TC-PF-17</t>
-        </is>
-      </c>
-      <c r="C264" s="15" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>TC-PF-12</t>
+        </is>
+      </c>
+      <c r="C264" s="19" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D264" s="13" t="inlineStr">
         <is>
-          <t>Buka Pilih Resto sebagai pelanggan</t>
+          <t>Catat pengeluaran dan top up petty cash KaataGo</t>
         </is>
       </c>
       <c r="E264" s="13" t="inlineStr">
         <is>
-          <t>KaataGo tidak muncul di daftar mana pun</t>
+          <t>Bekerja sama seperti di resto</t>
         </is>
       </c>
       <c r="F264" s="13" t="inlineStr">
         <is>
-          <t>TSD §7.4</t>
+          <t>F-PF-09</t>
         </is>
       </c>
       <c r="G264" s="13" t="inlineStr"/>
@@ -11001,7 +11001,7 @@
       </c>
       <c r="B265" s="17" t="inlineStr">
         <is>
-          <t>TC-PF-18</t>
+          <t>TC-PF-13</t>
         </is>
       </c>
       <c r="C265" s="18" t="inlineStr">
@@ -11011,17 +11011,17 @@
       </c>
       <c r="D265" s="16" t="inlineStr">
         <is>
-          <t>Buka List Resto dan Billing Resto sebagai Super Admin</t>
+          <t>Telusuri menu Finance KaataGo</t>
         </is>
       </c>
       <c r="E265" s="16" t="inlineStr">
         <is>
-          <t>KaataGo tidak muncul sebagai resto yang bisa ditagih</t>
+          <t>Tidak ada Setor Saldo Cash</t>
         </is>
       </c>
       <c r="F265" s="16" t="inlineStr">
         <is>
-          <t>TSD §7.4</t>
+          <t>F-PF-10</t>
         </is>
       </c>
       <c r="G265" s="16" t="inlineStr"/>
@@ -11036,27 +11036,27 @@
       </c>
       <c r="B266" s="14" t="inlineStr">
         <is>
-          <t>TC-PF-19</t>
-        </is>
-      </c>
-      <c r="C266" s="19" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-PF-14</t>
+        </is>
+      </c>
+      <c r="C266" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D266" s="13" t="inlineStr">
         <is>
-          <t>Buka Diskon Langganan sebagai Owner resto</t>
+          <t>Buka Jurnal GL Semua Resto</t>
         </is>
       </c>
       <c r="E266" s="13" t="inlineStr">
         <is>
-          <t>Hanya diskon yang mengenai restonya yang terbaca</t>
+          <t>Jurnal seluruh resto tampil, bisa disaring per resto</t>
         </is>
       </c>
       <c r="F266" s="13" t="inlineStr">
         <is>
-          <t>F-PF-03</t>
+          <t>F-PF-11</t>
         </is>
       </c>
       <c r="G266" s="13" t="inlineStr"/>
@@ -11066,12 +11066,12 @@
     <row r="267">
       <c r="A267" s="16" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19c. Finance KaataGo (Super Admin)</t>
         </is>
       </c>
       <c r="B267" s="17" t="inlineStr">
         <is>
-          <t>TC-TS-01</t>
+          <t>TC-PF-15</t>
         </is>
       </c>
       <c r="C267" s="18" t="inlineStr">
@@ -11081,17 +11081,17 @@
       </c>
       <c r="D267" s="16" t="inlineStr">
         <is>
-          <t>Panggil GET /rest/v1/orders memakai kunci anon tanpa login</t>
+          <t>Cari cara mengubah baris di Jurnal GL Semua Resto</t>
         </is>
       </c>
       <c r="E267" s="16" t="inlineStr">
         <is>
-          <t>Tidak mengembalikan pesanan resto mana pun</t>
+          <t>Tidak ada satu pun — hanya bisa dilihat</t>
         </is>
       </c>
       <c r="F267" s="16" t="inlineStr">
         <is>
-          <t>TSD §5</t>
+          <t>F-PF-12</t>
         </is>
       </c>
       <c r="G267" s="16" t="inlineStr"/>
@@ -11101,12 +11101,12 @@
     <row r="268">
       <c r="A268" s="13" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19c. Finance KaataGo (Super Admin)</t>
         </is>
       </c>
       <c r="B268" s="14" t="inlineStr">
         <is>
-          <t>TC-TS-02</t>
+          <t>TC-PF-16</t>
         </is>
       </c>
       <c r="C268" s="15" t="inlineStr">
@@ -11116,17 +11116,17 @@
       </c>
       <c r="D268" s="13" t="inlineStr">
         <is>
-          <t>Login sebagai karyawan resto A, baca orders resto B lewat API</t>
+          <t>Coba UPDATE gl_journal_entries sebagai Super Admin lewat API</t>
         </is>
       </c>
       <c r="E268" s="13" t="inlineStr">
         <is>
-          <t>Kosong — bukan galat, tapi juga bukan data</t>
+          <t>Ditolak</t>
         </is>
       </c>
       <c r="F268" s="13" t="inlineStr">
         <is>
-          <t>TSD §5</t>
+          <t>F-PF-12, TSD §7.4</t>
         </is>
       </c>
       <c r="G268" s="13" t="inlineStr"/>
@@ -11136,12 +11136,12 @@
     <row r="269">
       <c r="A269" s="16" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19c. Finance KaataGo (Super Admin)</t>
         </is>
       </c>
       <c r="B269" s="17" t="inlineStr">
         <is>
-          <t>TC-TS-03</t>
+          <t>TC-PF-17</t>
         </is>
       </c>
       <c r="C269" s="18" t="inlineStr">
@@ -11151,17 +11151,17 @@
       </c>
       <c r="D269" s="16" t="inlineStr">
         <is>
-          <t>Login sebagai Owner, buka tiap layar resto miliknya</t>
+          <t>Buka Pilih Resto sebagai pelanggan</t>
         </is>
       </c>
       <c r="E269" s="16" t="inlineStr">
         <is>
-          <t>Tidak ada layar yang kosong karena RLS — owner harus disebut di setiap daftar peran</t>
+          <t>KaataGo tidak muncul di daftar mana pun</t>
         </is>
       </c>
       <c r="F269" s="16" t="inlineStr">
         <is>
-          <t>TSD §5</t>
+          <t>TSD §7.4</t>
         </is>
       </c>
       <c r="G269" s="16" t="inlineStr"/>
@@ -11171,12 +11171,12 @@
     <row r="270">
       <c r="A270" s="13" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19c. Finance KaataGo (Super Admin)</t>
         </is>
       </c>
       <c r="B270" s="14" t="inlineStr">
         <is>
-          <t>TC-TS-04</t>
+          <t>TC-PF-18</t>
         </is>
       </c>
       <c r="C270" s="15" t="inlineStr">
@@ -11186,17 +11186,17 @@
       </c>
       <c r="D270" s="13" t="inlineStr">
         <is>
-          <t>Login sebagai Kasir, baca gl_journal_entries</t>
+          <t>Buka List Resto dan Billing Resto sebagai Super Admin</t>
         </is>
       </c>
       <c r="E270" s="13" t="inlineStr">
         <is>
-          <t>Hanya yang terkait catatan yang memang boleh dia lihat</t>
+          <t>KaataGo tidak muncul sebagai resto yang bisa ditagih</t>
         </is>
       </c>
       <c r="F270" s="13" t="inlineStr">
         <is>
-          <t>F-KS-13, TSD §5.1</t>
+          <t>TSD §7.4</t>
         </is>
       </c>
       <c r="G270" s="13" t="inlineStr"/>
@@ -11206,32 +11206,32 @@
     <row r="271">
       <c r="A271" s="16" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19c. Finance KaataGo (Super Admin)</t>
         </is>
       </c>
       <c r="B271" s="17" t="inlineStr">
         <is>
-          <t>TC-TS-05</t>
-        </is>
-      </c>
-      <c r="C271" s="18" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>TC-PF-19</t>
+        </is>
+      </c>
+      <c r="C271" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D271" s="16" t="inlineStr">
         <is>
-          <t>Coba UPDATE products langsung lewat API sebagai pelanggan</t>
+          <t>Buka Diskon Langganan sebagai Owner resto</t>
         </is>
       </c>
       <c r="E271" s="16" t="inlineStr">
         <is>
-          <t>Ditolak; pengurangan stok hanya lewat decrement_stock</t>
+          <t>Hanya diskon yang mengenai restonya yang terbaca</t>
         </is>
       </c>
       <c r="F271" s="16" t="inlineStr">
         <is>
-          <t>TSD §5.2</t>
+          <t>F-PF-03</t>
         </is>
       </c>
       <c r="G271" s="16" t="inlineStr"/>
@@ -11241,12 +11241,12 @@
     <row r="272">
       <c r="A272" s="13" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19c. Finance KaataGo (Super Admin)</t>
         </is>
       </c>
       <c r="B272" s="14" t="inlineStr">
         <is>
-          <t>TC-TS-06</t>
+          <t>TC-PF-20</t>
         </is>
       </c>
       <c r="C272" s="15" t="inlineStr">
@@ -11256,17 +11256,17 @@
       </c>
       <c r="D272" s="13" t="inlineStr">
         <is>
-          <t>Panggil cancel_my_order untuk pesanan milik orang lain</t>
+          <t>Bandingkan total debit/kredit Jurnal Semua Resto dengan Jurnal GL resto itu (saring ke resto yang sama)</t>
         </is>
       </c>
       <c r="E272" s="13" t="inlineStr">
         <is>
-          <t>Ditolak</t>
+          <t>Angkanya sama persis</t>
         </is>
       </c>
       <c r="F272" s="13" t="inlineStr">
         <is>
-          <t>TSD §5.2</t>
+          <t>F-PF-14</t>
         </is>
       </c>
       <c r="G272" s="13" t="inlineStr"/>
@@ -11276,12 +11276,12 @@
     <row r="273">
       <c r="A273" s="16" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19c. Finance KaataGo (Super Admin)</t>
         </is>
       </c>
       <c r="B273" s="17" t="inlineStr">
         <is>
-          <t>TC-TS-07</t>
+          <t>TC-PF-21</t>
         </is>
       </c>
       <c r="C273" s="18" t="inlineStr">
@@ -11291,17 +11291,17 @@
       </c>
       <c r="D273" s="16" t="inlineStr">
         <is>
-          <t>Jalankan ulang seluruh JALANKAN-INI.sql di database yang sudah terisi</t>
+          <t>Batalkan sebuah pengeluaran, lihat kedua layar jurnal</t>
         </is>
       </c>
       <c r="E273" s="16" t="inlineStr">
         <is>
-          <t>Selesai tanpa galat; tidak ada data yang berubah</t>
+          <t>Total tidak naik; keterangan "N pembatalan tidak dihitung" muncul</t>
         </is>
       </c>
       <c r="F273" s="16" t="inlineStr">
         <is>
-          <t>TSD §11</t>
+          <t>F-PF-14</t>
         </is>
       </c>
       <c r="G273" s="16" t="inlineStr"/>
@@ -11311,32 +11311,32 @@
     <row r="274">
       <c r="A274" s="13" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19c. Finance KaataGo (Super Admin)</t>
         </is>
       </c>
       <c r="B274" s="14" t="inlineStr">
         <is>
-          <t>TC-TS-08</t>
-        </is>
-      </c>
-      <c r="C274" s="15" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>TC-PF-22</t>
+        </is>
+      </c>
+      <c r="C274" s="19" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D274" s="13" t="inlineStr">
         <is>
-          <t>Jalankan ulang satu berkas SQL lama saja, misal cash_payment_expiry.sql</t>
+          <t>Cari baris pembatalan di daftar</t>
         </is>
       </c>
       <c r="E274" s="13" t="inlineStr">
         <is>
-          <t>Tidak menyempitkan daftar nilai batasan mana pun</t>
+          <t>Tetap tampil, bertanda PEMBATALAN</t>
         </is>
       </c>
       <c r="F274" s="13" t="inlineStr">
         <is>
-          <t>TSD §11.1</t>
+          <t>F-PF-15</t>
         </is>
       </c>
       <c r="G274" s="13" t="inlineStr"/>
@@ -11346,12 +11346,12 @@
     <row r="275">
       <c r="A275" s="16" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19c. Finance KaataGo (Super Admin)</t>
         </is>
       </c>
       <c r="B275" s="17" t="inlineStr">
         <is>
-          <t>TC-TS-09</t>
+          <t>TC-PF-23</t>
         </is>
       </c>
       <c r="C275" s="18" t="inlineStr">
@@ -11361,17 +11361,17 @@
       </c>
       <c r="D275" s="16" t="inlineStr">
         <is>
-          <t>Buat resto baru dari Super Admin</t>
+          <t>Saring ke sebuah resto, lalu pilih Semua resto lagi</t>
         </is>
       </c>
       <c r="E275" s="16" t="inlineStr">
         <is>
-          <t>Bagan akun GL 12 jenis dan tarif PPN/service langsung terisi</t>
+          <t>Kembali menampilkan seluruh resto — bukan tetap tersaring</t>
         </is>
       </c>
       <c r="F275" s="16" t="inlineStr">
         <is>
-          <t>A-19, TSD §6.2</t>
+          <t>F-PF-16</t>
         </is>
       </c>
       <c r="G275" s="16" t="inlineStr"/>
@@ -11381,12 +11381,12 @@
     <row r="276">
       <c r="A276" s="13" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19c. Finance KaataGo (Super Admin)</t>
         </is>
       </c>
       <c r="B276" s="14" t="inlineStr">
         <is>
-          <t>TC-TS-10</t>
+          <t>TC-PF-24</t>
         </is>
       </c>
       <c r="C276" s="15" t="inlineStr">
@@ -11396,17 +11396,17 @@
       </c>
       <c r="D276" s="13" t="inlineStr">
         <is>
-          <t>Kosongkan satu nomor GL, lalu buat transaksi</t>
+          <t>Saring ke resto A, lalu saring lagi ke resto B yang punya jurnal</t>
         </is>
       </c>
       <c r="E276" s="13" t="inlineStr">
         <is>
-          <t>Jurnal untuk baris itu tidak terbentuk — pastikan gejalanya dikenali penguji</t>
+          <t>Isinya berganti ke jurnal resto B</t>
         </is>
       </c>
       <c r="F276" s="13" t="inlineStr">
         <is>
-          <t>TSD §6.2</t>
+          <t>F-PF-16</t>
         </is>
       </c>
       <c r="G276" s="13" t="inlineStr"/>
@@ -11416,12 +11416,12 @@
     <row r="277">
       <c r="A277" s="16" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19c. Finance KaataGo (Super Admin)</t>
         </is>
       </c>
       <c r="B277" s="17" t="inlineStr">
         <is>
-          <t>TC-TS-11</t>
+          <t>TC-PF-25</t>
         </is>
       </c>
       <c r="C277" s="20" t="inlineStr">
@@ -11431,17 +11431,17 @@
       </c>
       <c r="D277" s="16" t="inlineStr">
         <is>
-          <t>Periksa push_outbox sesudah pengumuman terbit</t>
+          <t>Perhatikan pita di atas layar sesudah menyaring</t>
         </is>
       </c>
       <c r="E277" s="16" t="inlineStr">
         <is>
-          <t>Baris masuk, lalu sent_at terisi</t>
+          <t>Nama restonya tertulis, dengan tombol × untuk melepasnya</t>
         </is>
       </c>
       <c r="F277" s="16" t="inlineStr">
         <is>
-          <t>TSD §8</t>
+          <t>F-PF-16</t>
         </is>
       </c>
       <c r="G277" s="16" t="inlineStr"/>
@@ -11451,12 +11451,12 @@
     <row r="278">
       <c r="A278" s="13" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19c. Finance KaataGo (Super Admin)</t>
         </is>
       </c>
       <c r="B278" s="14" t="inlineStr">
         <is>
-          <t>TC-TS-12</t>
+          <t>TC-PF-26</t>
         </is>
       </c>
       <c r="C278" s="19" t="inlineStr">
@@ -11466,17 +11466,17 @@
       </c>
       <c r="D278" s="13" t="inlineStr">
         <is>
-          <t>Matikan sambungan, pakai aplikasi</t>
+          <t>Buka daftar saringan</t>
         </is>
       </c>
       <c r="E278" s="13" t="inlineStr">
         <is>
-          <t>Katalog tetap tampil; pesanan tunai tetap bisa dibuat</t>
+          <t>Resto yang belum punya jurnal ditandai "Belum ada jurnal"</t>
         </is>
       </c>
       <c r="F278" s="13" t="inlineStr">
         <is>
-          <t>TSD §10, FSD §5.6</t>
+          <t>F-PF-17</t>
         </is>
       </c>
       <c r="G278" s="13" t="inlineStr"/>
@@ -11486,12 +11486,12 @@
     <row r="279">
       <c r="A279" s="16" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19c. Finance KaataGo (Super Admin)</t>
         </is>
       </c>
       <c r="B279" s="17" t="inlineStr">
         <is>
-          <t>TC-TS-13</t>
+          <t>TC-PF-27</t>
         </is>
       </c>
       <c r="C279" s="20" t="inlineStr">
@@ -11501,17 +11501,17 @@
       </c>
       <c r="D279" s="16" t="inlineStr">
         <is>
-          <t>Sambungkan lagi</t>
+          <t>Perhatikan pengelompokan</t>
         </is>
       </c>
       <c r="E279" s="16" t="inlineStr">
         <is>
-          <t>Pesanan yang dibuat saat luring terkirim</t>
+          <t>Per tanggal, bisa dilipat; tanggal terbaru terbuka, sisanya tertutup</t>
         </is>
       </c>
       <c r="F279" s="16" t="inlineStr">
         <is>
-          <t>TSD §10</t>
+          <t>F-PF-18</t>
         </is>
       </c>
       <c r="G279" s="16" t="inlineStr"/>
@@ -11521,12 +11521,12 @@
     <row r="280">
       <c r="A280" s="13" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19c. Finance KaataGo (Super Admin)</t>
         </is>
       </c>
       <c r="B280" s="14" t="inlineStr">
         <is>
-          <t>TC-TS-14</t>
+          <t>TC-PF-28</t>
         </is>
       </c>
       <c r="C280" s="15" t="inlineStr">
@@ -11536,17 +11536,17 @@
       </c>
       <c r="D280" s="13" t="inlineStr">
         <is>
-          <t>Coba bayar QRIS saat luring</t>
+          <t>Buka Mapping GL Account resto mana pun</t>
         </is>
       </c>
       <c r="E280" s="13" t="inlineStr">
         <is>
-          <t>Ditolak dengan jelas — bukan menggantung tanpa kabar</t>
+          <t>GL Diskon punya bagiannya dan nomornya sudah terisi</t>
         </is>
       </c>
       <c r="F280" s="13" t="inlineStr">
         <is>
-          <t>FSD §5.6</t>
+          <t>F-PF-19, F-DS-09</t>
         </is>
       </c>
       <c r="G280" s="13" t="inlineStr"/>
@@ -11556,32 +11556,32 @@
     <row r="281">
       <c r="A281" s="16" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19c. Finance KaataGo (Super Admin)</t>
         </is>
       </c>
       <c r="B281" s="17" t="inlineStr">
         <is>
-          <t>TC-TS-15</t>
-        </is>
-      </c>
-      <c r="C281" s="18" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>TC-PF-29</t>
+        </is>
+      </c>
+      <c r="C281" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D281" s="16" t="inlineStr">
         <is>
-          <t>Panggil create-qris dengan nominal yang dipalsukan di badan permintaan</t>
+          <t>Buka Mapping GL Account KaataGo</t>
         </is>
       </c>
       <c r="E281" s="16" t="inlineStr">
         <is>
-          <t>Nominal yang dipakai tetap dari basis data</t>
+          <t>Ada bagian GL Langganan; penghitung akun tidak pernah menyisakan yang mustahil terisi</t>
         </is>
       </c>
       <c r="F281" s="16" t="inlineStr">
         <is>
-          <t>TSD §7.1</t>
+          <t>F-PF-19</t>
         </is>
       </c>
       <c r="G281" s="16" t="inlineStr"/>
@@ -11591,12 +11591,12 @@
     <row r="282">
       <c r="A282" s="13" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19c. Finance KaataGo (Super Admin)</t>
         </is>
       </c>
       <c r="B282" s="14" t="inlineStr">
         <is>
-          <t>TC-TS-16</t>
+          <t>TC-PF-30</t>
         </is>
       </c>
       <c r="C282" s="15" t="inlineStr">
@@ -11606,17 +11606,17 @@
       </c>
       <c r="D282" s="13" t="inlineStr">
         <is>
-          <t>Tandai pesanan lunas lewat API tanpa lewat webhook</t>
+          <t>Pesan menu berpromo, bayar, buka Jurnal GL</t>
         </is>
       </c>
       <c r="E282" s="13" t="inlineStr">
         <is>
-          <t>Ditolak</t>
+          <t>Baris GL Diskon menyebut nama promonya</t>
         </is>
       </c>
       <c r="F282" s="13" t="inlineStr">
         <is>
-          <t>F-PG-02, TSD §7.1</t>
+          <t>F-PF-20, F-DS-13</t>
         </is>
       </c>
       <c r="G282" s="13" t="inlineStr"/>
@@ -11631,27 +11631,27 @@
       </c>
       <c r="B283" s="17" t="inlineStr">
         <is>
-          <t>TC-TS-17</t>
-        </is>
-      </c>
-      <c r="C283" s="20" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-TS-01</t>
+        </is>
+      </c>
+      <c r="C283" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D283" s="16" t="inlineStr">
         <is>
-          <t>Bongkar APK, cari kunci Xendit/FCM/Resend</t>
+          <t>Panggil GET /rest/v1/orders memakai kunci anon tanpa login</t>
         </is>
       </c>
       <c r="E283" s="16" t="inlineStr">
         <is>
-          <t>Tidak ada satu pun kunci pengirim di dalamnya</t>
+          <t>Tidak mengembalikan pesanan resto mana pun</t>
         </is>
       </c>
       <c r="F283" s="16" t="inlineStr">
         <is>
-          <t>TSD §1.2</t>
+          <t>TSD §5</t>
         </is>
       </c>
       <c r="G283" s="16" t="inlineStr"/>
@@ -11666,27 +11666,27 @@
       </c>
       <c r="B284" s="14" t="inlineStr">
         <is>
-          <t>TC-TS-18</t>
-        </is>
-      </c>
-      <c r="C284" s="19" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-TS-02</t>
+        </is>
+      </c>
+      <c r="C284" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D284" s="13" t="inlineStr">
         <is>
-          <t>Pesanan berpindah status lunas lebih dari sekali</t>
+          <t>Login sebagai karyawan resto A, baca orders resto B lewat API</t>
         </is>
       </c>
       <c r="E284" s="13" t="inlineStr">
         <is>
-          <t>Jurnalnya tetap satu set — tidak ada baris ganda</t>
+          <t>Kosong — bukan galat, tapi juga bukan data</t>
         </is>
       </c>
       <c r="F284" s="13" t="inlineStr">
         <is>
-          <t>TSD §6.5</t>
+          <t>TSD §5</t>
         </is>
       </c>
       <c r="G284" s="13" t="inlineStr"/>
@@ -11701,27 +11701,27 @@
       </c>
       <c r="B285" s="17" t="inlineStr">
         <is>
-          <t>TC-TS-19</t>
-        </is>
-      </c>
-      <c r="C285" s="20" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-TS-03</t>
+        </is>
+      </c>
+      <c r="C285" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D285" s="16" t="inlineStr">
         <is>
-          <t>Hapus resto uji</t>
+          <t>Login sebagai Owner, buka tiap layar resto miliknya</t>
         </is>
       </c>
       <c r="E285" s="16" t="inlineStr">
         <is>
-          <t>Seluruh isinya ikut terhapus, termasuk jurnalnya</t>
+          <t>Tidak ada layar yang kosong karena RLS — owner harus disebut di setiap daftar peran</t>
         </is>
       </c>
       <c r="F285" s="16" t="inlineStr">
         <is>
-          <t>TSD §4.0</t>
+          <t>TSD §5</t>
         </is>
       </c>
       <c r="G285" s="16" t="inlineStr"/>
@@ -11731,12 +11731,12 @@
     <row r="286">
       <c r="A286" s="13" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>Uji Teknis (lingkup TSD)</t>
         </is>
       </c>
       <c r="B286" s="14" t="inlineStr">
         <is>
-          <t>TC-RG-01</t>
+          <t>TC-TS-04</t>
         </is>
       </c>
       <c r="C286" s="15" t="inlineStr">
@@ -11746,17 +11746,17 @@
       </c>
       <c r="D286" s="13" t="inlineStr">
         <is>
-          <t>Nominal QRIS kasir memakai subtotal menu, bukan total tagihan</t>
+          <t>Login sebagai Kasir, baca gl_journal_entries</t>
         </is>
       </c>
       <c r="E286" s="13" t="inlineStr">
         <is>
-          <t>Nominal di layar QRIS = total termasuk service dan PPN</t>
+          <t>Hanya yang terkait catatan yang memang boleh dia lihat</t>
         </is>
       </c>
       <c r="F286" s="13" t="inlineStr">
         <is>
-          <t>F-KS-09</t>
+          <t>F-KS-13, TSD §5.1</t>
         </is>
       </c>
       <c r="G286" s="13" t="inlineStr"/>
@@ -11766,12 +11766,12 @@
     <row r="287">
       <c r="A287" s="16" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>Uji Teknis (lingkup TSD)</t>
         </is>
       </c>
       <c r="B287" s="17" t="inlineStr">
         <is>
-          <t>TC-RG-02</t>
+          <t>TC-TS-05</t>
         </is>
       </c>
       <c r="C287" s="18" t="inlineStr">
@@ -11781,17 +11781,17 @@
       </c>
       <c r="D287" s="16" t="inlineStr">
         <is>
-          <t>Pesanan dilunasi lewat QRIS hilang dari Riwayat Kasir</t>
+          <t>Coba UPDATE products langsung lewat API sebagai pelanggan</t>
         </is>
       </c>
       <c r="E287" s="16" t="inlineStr">
         <is>
-          <t>Semua cara bayar masuk Riwayat Kasir</t>
+          <t>Ditolak; pengurangan stok hanya lewat decrement_stock</t>
         </is>
       </c>
       <c r="F287" s="16" t="inlineStr">
         <is>
-          <t>F-PP-09, A-13</t>
+          <t>TSD §5.2</t>
         </is>
       </c>
       <c r="G287" s="16" t="inlineStr"/>
@@ -11801,12 +11801,12 @@
     <row r="288">
       <c r="A288" s="13" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>Uji Teknis (lingkup TSD)</t>
         </is>
       </c>
       <c r="B288" s="14" t="inlineStr">
         <is>
-          <t>TC-RG-03</t>
+          <t>TC-TS-06</t>
         </is>
       </c>
       <c r="C288" s="15" t="inlineStr">
@@ -11816,17 +11816,17 @@
       </c>
       <c r="D288" s="13" t="inlineStr">
         <is>
-          <t>Pesanan dibatalkan tampil "Menunggu Pembayaran" di Pesanan Masuk</t>
+          <t>Panggil cancel_my_order untuk pesanan milik orang lain</t>
         </is>
       </c>
       <c r="E288" s="13" t="inlineStr">
         <is>
-          <t>Tidak muncul sama sekali</t>
+          <t>Ditolak</t>
         </is>
       </c>
       <c r="F288" s="13" t="inlineStr">
         <is>
-          <t>A-17</t>
+          <t>TSD §5.2</t>
         </is>
       </c>
       <c r="G288" s="13" t="inlineStr"/>
@@ -11836,12 +11836,12 @@
     <row r="289">
       <c r="A289" s="16" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>Uji Teknis (lingkup TSD)</t>
         </is>
       </c>
       <c r="B289" s="17" t="inlineStr">
         <is>
-          <t>TC-RG-04</t>
+          <t>TC-TS-07</t>
         </is>
       </c>
       <c r="C289" s="18" t="inlineStr">
@@ -11851,17 +11851,17 @@
       </c>
       <c r="D289" s="16" t="inlineStr">
         <is>
-          <t>Top up Rp 100.000 tercatat Rp 200.000 di jurnal</t>
+          <t>Jalankan ulang seluruh JALANKAN-INI.sql di database yang sudah terisi</t>
         </is>
       </c>
       <c r="E289" s="16" t="inlineStr">
         <is>
-          <t>Nominalnya sama dengan yang diajukan</t>
+          <t>Selesai tanpa galat; tidak ada data yang berubah</t>
         </is>
       </c>
       <c r="F289" s="16" t="inlineStr">
         <is>
-          <t>F-FN-03</t>
+          <t>TSD §11</t>
         </is>
       </c>
       <c r="G289" s="16" t="inlineStr"/>
@@ -11871,12 +11871,12 @@
     <row r="290">
       <c r="A290" s="13" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>Uji Teknis (lingkup TSD)</t>
         </is>
       </c>
       <c r="B290" s="14" t="inlineStr">
         <is>
-          <t>TC-RG-05</t>
+          <t>TC-TS-08</t>
         </is>
       </c>
       <c r="C290" s="15" t="inlineStr">
@@ -11886,17 +11886,17 @@
       </c>
       <c r="D290" s="13" t="inlineStr">
         <is>
-          <t>Diskon tidak berlaku untuk pesanan mandiri pelanggan</t>
+          <t>Jalankan ulang satu berkas SQL lama saja, misal cash_payment_expiry.sql</t>
         </is>
       </c>
       <c r="E290" s="13" t="inlineStr">
         <is>
-          <t>Berlaku sama di kasir dan HP pelanggan</t>
+          <t>Tidak menyempitkan daftar nilai batasan mana pun</t>
         </is>
       </c>
       <c r="F290" s="13" t="inlineStr">
         <is>
-          <t>A-14</t>
+          <t>TSD §11.1</t>
         </is>
       </c>
       <c r="G290" s="13" t="inlineStr"/>
@@ -11906,12 +11906,12 @@
     <row r="291">
       <c r="A291" s="16" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>Uji Teknis (lingkup TSD)</t>
         </is>
       </c>
       <c r="B291" s="17" t="inlineStr">
         <is>
-          <t>TC-RG-06</t>
+          <t>TC-TS-09</t>
         </is>
       </c>
       <c r="C291" s="18" t="inlineStr">
@@ -11921,17 +11921,17 @@
       </c>
       <c r="D291" s="16" t="inlineStr">
         <is>
-          <t>Promo "beli 2" lolos oleh keranjang berisi dua menu berbeda</t>
+          <t>Buat resto baru dari Super Admin</t>
         </is>
       </c>
       <c r="E291" s="16" t="inlineStr">
         <is>
-          <t>Syarat jumlah dihitung per menu, dan seluruhnya harus terpenuhi</t>
+          <t>Bagan akun GL 12 jenis dan tarif PPN/service langsung terisi</t>
         </is>
       </c>
       <c r="F291" s="16" t="inlineStr">
         <is>
-          <t>F-DS-10, F-DS-12</t>
+          <t>A-19, TSD §6.2</t>
         </is>
       </c>
       <c r="G291" s="16" t="inlineStr"/>
@@ -11941,32 +11941,32 @@
     <row r="292">
       <c r="A292" s="13" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>Uji Teknis (lingkup TSD)</t>
         </is>
       </c>
       <c r="B292" s="14" t="inlineStr">
         <is>
-          <t>TC-RG-07</t>
-        </is>
-      </c>
-      <c r="C292" s="19" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-TS-10</t>
+        </is>
+      </c>
+      <c r="C292" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D292" s="13" t="inlineStr">
         <is>
-          <t>Tombol pilih/hapus di kotak masuk tidak bereaksi sama sekali</t>
+          <t>Kosongkan satu nomor GL, lalu buat transaksi</t>
         </is>
       </c>
       <c r="E292" s="13" t="inlineStr">
         <is>
-          <t>Bekerja di kotak masuk karyawan dan pelanggan</t>
+          <t>Jurnal untuk baris itu tidak terbentuk — pastikan gejalanya dikenali penguji</t>
         </is>
       </c>
       <c r="F292" s="13" t="inlineStr">
         <is>
-          <t>F-IN-15</t>
+          <t>TSD §6.2</t>
         </is>
       </c>
       <c r="G292" s="13" t="inlineStr"/>
@@ -11976,12 +11976,12 @@
     <row r="293">
       <c r="A293" s="16" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>Uji Teknis (lingkup TSD)</t>
         </is>
       </c>
       <c r="B293" s="17" t="inlineStr">
         <is>
-          <t>TC-RG-08</t>
+          <t>TC-TS-11</t>
         </is>
       </c>
       <c r="C293" s="20" t="inlineStr">
@@ -11991,17 +11991,17 @@
       </c>
       <c r="D293" s="16" t="inlineStr">
         <is>
-          <t>Layar Diskon dari hub Kasir menyebut "Belum ada produk di resto ini"</t>
+          <t>Periksa push_outbox sesudah pengumuman terbit</t>
         </is>
       </c>
       <c r="E293" s="16" t="inlineStr">
         <is>
-          <t>Daftar menu termuat</t>
+          <t>Baris masuk, lalu sent_at terisi</t>
         </is>
       </c>
       <c r="F293" s="16" t="inlineStr">
         <is>
-          <t>F-DS-01</t>
+          <t>TSD §8</t>
         </is>
       </c>
       <c r="G293" s="16" t="inlineStr"/>
@@ -12011,12 +12011,12 @@
     <row r="294">
       <c r="A294" s="13" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>Uji Teknis (lingkup TSD)</t>
         </is>
       </c>
       <c r="B294" s="14" t="inlineStr">
         <is>
-          <t>TC-RG-09</t>
+          <t>TC-TS-12</t>
         </is>
       </c>
       <c r="C294" s="19" t="inlineStr">
@@ -12026,17 +12026,17 @@
       </c>
       <c r="D294" s="13" t="inlineStr">
         <is>
-          <t>Kasir tidak bisa membuka detail jurnal — terlihat seperti GL belum dipetakan</t>
+          <t>Matikan sambungan, pakai aplikasi</t>
         </is>
       </c>
       <c r="E294" s="13" t="inlineStr">
         <is>
-          <t>Detail jurnal terbuka</t>
+          <t>Katalog tetap tampil; pesanan tunai tetap bisa dibuat</t>
         </is>
       </c>
       <c r="F294" s="13" t="inlineStr">
         <is>
-          <t>F-KS-13</t>
+          <t>TSD §10, FSD §5.6</t>
         </is>
       </c>
       <c r="G294" s="13" t="inlineStr"/>
@@ -12046,12 +12046,12 @@
     <row r="295">
       <c r="A295" s="16" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>Uji Teknis (lingkup TSD)</t>
         </is>
       </c>
       <c r="B295" s="17" t="inlineStr">
         <is>
-          <t>TC-RG-10</t>
+          <t>TC-TS-13</t>
         </is>
       </c>
       <c r="C295" s="20" t="inlineStr">
@@ -12061,17 +12061,17 @@
       </c>
       <c r="D295" s="16" t="inlineStr">
         <is>
-          <t>Layar dapur meninggalkan jejak warna lama saat tema diganti</t>
+          <t>Sambungkan lagi</t>
         </is>
       </c>
       <c r="E295" s="16" t="inlineStr">
         <is>
-          <t>Seluruh layar berganti bersih</t>
+          <t>Pesanan yang dibuat saat luring terkirim</t>
         </is>
       </c>
       <c r="F295" s="16" t="inlineStr">
         <is>
-          <t>A-18</t>
+          <t>TSD §10</t>
         </is>
       </c>
       <c r="G295" s="16" t="inlineStr"/>
@@ -12081,32 +12081,32 @@
     <row r="296">
       <c r="A296" s="13" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>Uji Teknis (lingkup TSD)</t>
         </is>
       </c>
       <c r="B296" s="14" t="inlineStr">
         <is>
-          <t>TC-RG-11</t>
-        </is>
-      </c>
-      <c r="C296" s="19" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-TS-14</t>
+        </is>
+      </c>
+      <c r="C296" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D296" s="13" t="inlineStr">
         <is>
-          <t>Banner promo menempel di atas, tidak ikut tergulir</t>
+          <t>Coba bayar QRIS saat luring</t>
         </is>
       </c>
       <c r="E296" s="13" t="inlineStr">
         <is>
-          <t>Ikut tergulir bersama menunya</t>
+          <t>Ditolak dengan jelas — bukan menggantung tanpa kabar</t>
         </is>
       </c>
       <c r="F296" s="13" t="inlineStr">
         <is>
-          <t>F-CU-16, A-12</t>
+          <t>FSD §5.6</t>
         </is>
       </c>
       <c r="G296" s="13" t="inlineStr"/>
@@ -12116,32 +12116,32 @@
     <row r="297">
       <c r="A297" s="16" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>Uji Teknis (lingkup TSD)</t>
         </is>
       </c>
       <c r="B297" s="17" t="inlineStr">
         <is>
-          <t>TC-RG-12</t>
-        </is>
-      </c>
-      <c r="C297" s="20" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-TS-15</t>
+        </is>
+      </c>
+      <c r="C297" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D297" s="16" t="inlineStr">
         <is>
-          <t>Owner hanya bisa melihat Info Pembayaran</t>
+          <t>Panggil create-qris dengan nominal yang dipalsukan di badan permintaan</t>
         </is>
       </c>
       <c r="E297" s="16" t="inlineStr">
         <is>
-          <t>Owner bisa mengubahnya</t>
+          <t>Nominal yang dipakai tetap dari basis data</t>
         </is>
       </c>
       <c r="F297" s="16" t="inlineStr">
         <is>
-          <t>F-SD-02</t>
+          <t>TSD §7.1</t>
         </is>
       </c>
       <c r="G297" s="16" t="inlineStr"/>
@@ -12151,12 +12151,12 @@
     <row r="298">
       <c r="A298" s="13" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>Uji Teknis (lingkup TSD)</t>
         </is>
       </c>
       <c r="B298" s="14" t="inlineStr">
         <is>
-          <t>TC-RG-13</t>
+          <t>TC-TS-16</t>
         </is>
       </c>
       <c r="C298" s="15" t="inlineStr">
@@ -12166,17 +12166,17 @@
       </c>
       <c r="D298" s="13" t="inlineStr">
         <is>
-          <t>Migrasi gagal: daftar nilai batasan menyempit saat berkas lama dijalankan ulang</t>
+          <t>Tandai pesanan lunas lewat API tanpa lewat webhook</t>
         </is>
       </c>
       <c r="E298" s="13" t="inlineStr">
         <is>
-          <t>Menjalankan ulang berkas mana pun tidak pernah menolak data yang sudah ada</t>
+          <t>Ditolak</t>
         </is>
       </c>
       <c r="F298" s="13" t="inlineStr">
         <is>
-          <t>TSD §11.1</t>
+          <t>F-PG-02, TSD §7.1</t>
         </is>
       </c>
       <c r="G298" s="13" t="inlineStr"/>
@@ -12186,12 +12186,12 @@
     <row r="299">
       <c r="A299" s="16" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>Uji Teknis (lingkup TSD)</t>
         </is>
       </c>
       <c r="B299" s="17" t="inlineStr">
         <is>
-          <t>TC-RG-14</t>
+          <t>TC-TS-17</t>
         </is>
       </c>
       <c r="C299" s="20" t="inlineStr">
@@ -12201,17 +12201,17 @@
       </c>
       <c r="D299" s="16" t="inlineStr">
         <is>
-          <t>QR meja borongan bernomor 07, berbeda dengan mode satu meja</t>
+          <t>Bongkar APK, cari kunci Xendit/FCM/Resend</t>
         </is>
       </c>
       <c r="E299" s="16" t="inlineStr">
         <is>
-          <t>Keduanya menulis 7</t>
+          <t>Tidak ada satu pun kunci pengirim di dalamnya</t>
         </is>
       </c>
       <c r="F299" s="16" t="inlineStr">
         <is>
-          <t>F-QR-07</t>
+          <t>TSD §1.2</t>
         </is>
       </c>
       <c r="G299" s="16" t="inlineStr"/>
@@ -12221,25 +12221,585 @@
     <row r="300">
       <c r="A300" s="13" t="inlineStr">
         <is>
+          <t>Uji Teknis (lingkup TSD)</t>
+        </is>
+      </c>
+      <c r="B300" s="14" t="inlineStr">
+        <is>
+          <t>TC-TS-18</t>
+        </is>
+      </c>
+      <c r="C300" s="19" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D300" s="13" t="inlineStr">
+        <is>
+          <t>Pesanan berpindah status lunas lebih dari sekali</t>
+        </is>
+      </c>
+      <c r="E300" s="13" t="inlineStr">
+        <is>
+          <t>Jurnalnya tetap satu set — tidak ada baris ganda</t>
+        </is>
+      </c>
+      <c r="F300" s="13" t="inlineStr">
+        <is>
+          <t>TSD §6.5</t>
+        </is>
+      </c>
+      <c r="G300" s="13" t="inlineStr"/>
+      <c r="H300" s="13" t="inlineStr"/>
+      <c r="I300" s="13" t="inlineStr"/>
+    </row>
+    <row r="301">
+      <c r="A301" s="16" t="inlineStr">
+        <is>
+          <t>Uji Teknis (lingkup TSD)</t>
+        </is>
+      </c>
+      <c r="B301" s="17" t="inlineStr">
+        <is>
+          <t>TC-TS-19</t>
+        </is>
+      </c>
+      <c r="C301" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D301" s="16" t="inlineStr">
+        <is>
+          <t>Hapus resto uji</t>
+        </is>
+      </c>
+      <c r="E301" s="16" t="inlineStr">
+        <is>
+          <t>Seluruh isinya ikut terhapus, termasuk jurnalnya</t>
+        </is>
+      </c>
+      <c r="F301" s="16" t="inlineStr">
+        <is>
+          <t>TSD §4.0</t>
+        </is>
+      </c>
+      <c r="G301" s="16" t="inlineStr"/>
+      <c r="H301" s="16" t="inlineStr"/>
+      <c r="I301" s="16" t="inlineStr"/>
+    </row>
+    <row r="302">
+      <c r="A302" s="13" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B302" s="14" t="inlineStr">
+        <is>
+          <t>TC-RG-01</t>
+        </is>
+      </c>
+      <c r="C302" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D302" s="13" t="inlineStr">
+        <is>
+          <t>Nominal QRIS kasir memakai subtotal menu, bukan total tagihan</t>
+        </is>
+      </c>
+      <c r="E302" s="13" t="inlineStr">
+        <is>
+          <t>Nominal di layar QRIS = total termasuk service dan PPN</t>
+        </is>
+      </c>
+      <c r="F302" s="13" t="inlineStr">
+        <is>
+          <t>F-KS-09</t>
+        </is>
+      </c>
+      <c r="G302" s="13" t="inlineStr"/>
+      <c r="H302" s="13" t="inlineStr"/>
+      <c r="I302" s="13" t="inlineStr"/>
+    </row>
+    <row r="303">
+      <c r="A303" s="16" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B303" s="17" t="inlineStr">
+        <is>
+          <t>TC-RG-02</t>
+        </is>
+      </c>
+      <c r="C303" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D303" s="16" t="inlineStr">
+        <is>
+          <t>Pesanan dilunasi lewat QRIS hilang dari Riwayat Kasir</t>
+        </is>
+      </c>
+      <c r="E303" s="16" t="inlineStr">
+        <is>
+          <t>Semua cara bayar masuk Riwayat Kasir</t>
+        </is>
+      </c>
+      <c r="F303" s="16" t="inlineStr">
+        <is>
+          <t>F-PP-09, A-13</t>
+        </is>
+      </c>
+      <c r="G303" s="16" t="inlineStr"/>
+      <c r="H303" s="16" t="inlineStr"/>
+      <c r="I303" s="16" t="inlineStr"/>
+    </row>
+    <row r="304">
+      <c r="A304" s="13" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B304" s="14" t="inlineStr">
+        <is>
+          <t>TC-RG-03</t>
+        </is>
+      </c>
+      <c r="C304" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D304" s="13" t="inlineStr">
+        <is>
+          <t>Pesanan dibatalkan tampil "Menunggu Pembayaran" di Pesanan Masuk</t>
+        </is>
+      </c>
+      <c r="E304" s="13" t="inlineStr">
+        <is>
+          <t>Tidak muncul sama sekali</t>
+        </is>
+      </c>
+      <c r="F304" s="13" t="inlineStr">
+        <is>
+          <t>A-17</t>
+        </is>
+      </c>
+      <c r="G304" s="13" t="inlineStr"/>
+      <c r="H304" s="13" t="inlineStr"/>
+      <c r="I304" s="13" t="inlineStr"/>
+    </row>
+    <row r="305">
+      <c r="A305" s="16" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B305" s="17" t="inlineStr">
+        <is>
+          <t>TC-RG-04</t>
+        </is>
+      </c>
+      <c r="C305" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D305" s="16" t="inlineStr">
+        <is>
+          <t>Top up Rp 100.000 tercatat Rp 200.000 di jurnal</t>
+        </is>
+      </c>
+      <c r="E305" s="16" t="inlineStr">
+        <is>
+          <t>Nominalnya sama dengan yang diajukan</t>
+        </is>
+      </c>
+      <c r="F305" s="16" t="inlineStr">
+        <is>
+          <t>F-FN-03</t>
+        </is>
+      </c>
+      <c r="G305" s="16" t="inlineStr"/>
+      <c r="H305" s="16" t="inlineStr"/>
+      <c r="I305" s="16" t="inlineStr"/>
+    </row>
+    <row r="306">
+      <c r="A306" s="13" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B306" s="14" t="inlineStr">
+        <is>
+          <t>TC-RG-05</t>
+        </is>
+      </c>
+      <c r="C306" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D306" s="13" t="inlineStr">
+        <is>
+          <t>Diskon tidak berlaku untuk pesanan mandiri pelanggan</t>
+        </is>
+      </c>
+      <c r="E306" s="13" t="inlineStr">
+        <is>
+          <t>Berlaku sama di kasir dan HP pelanggan</t>
+        </is>
+      </c>
+      <c r="F306" s="13" t="inlineStr">
+        <is>
+          <t>A-14</t>
+        </is>
+      </c>
+      <c r="G306" s="13" t="inlineStr"/>
+      <c r="H306" s="13" t="inlineStr"/>
+      <c r="I306" s="13" t="inlineStr"/>
+    </row>
+    <row r="307">
+      <c r="A307" s="16" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B307" s="17" t="inlineStr">
+        <is>
+          <t>TC-RG-06</t>
+        </is>
+      </c>
+      <c r="C307" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D307" s="16" t="inlineStr">
+        <is>
+          <t>Promo "beli 2" lolos oleh keranjang berisi dua menu berbeda</t>
+        </is>
+      </c>
+      <c r="E307" s="16" t="inlineStr">
+        <is>
+          <t>Syarat jumlah dihitung per menu, dan seluruhnya harus terpenuhi</t>
+        </is>
+      </c>
+      <c r="F307" s="16" t="inlineStr">
+        <is>
+          <t>F-DS-10, F-DS-12</t>
+        </is>
+      </c>
+      <c r="G307" s="16" t="inlineStr"/>
+      <c r="H307" s="16" t="inlineStr"/>
+      <c r="I307" s="16" t="inlineStr"/>
+    </row>
+    <row r="308">
+      <c r="A308" s="13" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B308" s="14" t="inlineStr">
+        <is>
+          <t>TC-RG-07</t>
+        </is>
+      </c>
+      <c r="C308" s="19" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D308" s="13" t="inlineStr">
+        <is>
+          <t>Tombol pilih/hapus di kotak masuk tidak bereaksi sama sekali</t>
+        </is>
+      </c>
+      <c r="E308" s="13" t="inlineStr">
+        <is>
+          <t>Bekerja di kotak masuk karyawan dan pelanggan</t>
+        </is>
+      </c>
+      <c r="F308" s="13" t="inlineStr">
+        <is>
+          <t>F-IN-15</t>
+        </is>
+      </c>
+      <c r="G308" s="13" t="inlineStr"/>
+      <c r="H308" s="13" t="inlineStr"/>
+      <c r="I308" s="13" t="inlineStr"/>
+    </row>
+    <row r="309">
+      <c r="A309" s="16" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B309" s="17" t="inlineStr">
+        <is>
+          <t>TC-RG-08</t>
+        </is>
+      </c>
+      <c r="C309" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D309" s="16" t="inlineStr">
+        <is>
+          <t>Layar Diskon dari hub Kasir menyebut "Belum ada produk di resto ini"</t>
+        </is>
+      </c>
+      <c r="E309" s="16" t="inlineStr">
+        <is>
+          <t>Daftar menu termuat</t>
+        </is>
+      </c>
+      <c r="F309" s="16" t="inlineStr">
+        <is>
+          <t>F-DS-01</t>
+        </is>
+      </c>
+      <c r="G309" s="16" t="inlineStr"/>
+      <c r="H309" s="16" t="inlineStr"/>
+      <c r="I309" s="16" t="inlineStr"/>
+    </row>
+    <row r="310">
+      <c r="A310" s="13" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B310" s="14" t="inlineStr">
+        <is>
+          <t>TC-RG-09</t>
+        </is>
+      </c>
+      <c r="C310" s="19" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D310" s="13" t="inlineStr">
+        <is>
+          <t>Kasir tidak bisa membuka detail jurnal — terlihat seperti GL belum dipetakan</t>
+        </is>
+      </c>
+      <c r="E310" s="13" t="inlineStr">
+        <is>
+          <t>Detail jurnal terbuka</t>
+        </is>
+      </c>
+      <c r="F310" s="13" t="inlineStr">
+        <is>
+          <t>F-KS-13</t>
+        </is>
+      </c>
+      <c r="G310" s="13" t="inlineStr"/>
+      <c r="H310" s="13" t="inlineStr"/>
+      <c r="I310" s="13" t="inlineStr"/>
+    </row>
+    <row r="311">
+      <c r="A311" s="16" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B311" s="17" t="inlineStr">
+        <is>
+          <t>TC-RG-10</t>
+        </is>
+      </c>
+      <c r="C311" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D311" s="16" t="inlineStr">
+        <is>
+          <t>Layar dapur meninggalkan jejak warna lama saat tema diganti</t>
+        </is>
+      </c>
+      <c r="E311" s="16" t="inlineStr">
+        <is>
+          <t>Seluruh layar berganti bersih</t>
+        </is>
+      </c>
+      <c r="F311" s="16" t="inlineStr">
+        <is>
+          <t>A-18</t>
+        </is>
+      </c>
+      <c r="G311" s="16" t="inlineStr"/>
+      <c r="H311" s="16" t="inlineStr"/>
+      <c r="I311" s="16" t="inlineStr"/>
+    </row>
+    <row r="312">
+      <c r="A312" s="13" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B312" s="14" t="inlineStr">
+        <is>
+          <t>TC-RG-11</t>
+        </is>
+      </c>
+      <c r="C312" s="19" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D312" s="13" t="inlineStr">
+        <is>
+          <t>Banner promo menempel di atas, tidak ikut tergulir</t>
+        </is>
+      </c>
+      <c r="E312" s="13" t="inlineStr">
+        <is>
+          <t>Ikut tergulir bersama menunya</t>
+        </is>
+      </c>
+      <c r="F312" s="13" t="inlineStr">
+        <is>
+          <t>F-CU-16, A-12</t>
+        </is>
+      </c>
+      <c r="G312" s="13" t="inlineStr"/>
+      <c r="H312" s="13" t="inlineStr"/>
+      <c r="I312" s="13" t="inlineStr"/>
+    </row>
+    <row r="313">
+      <c r="A313" s="16" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B313" s="17" t="inlineStr">
+        <is>
+          <t>TC-RG-12</t>
+        </is>
+      </c>
+      <c r="C313" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D313" s="16" t="inlineStr">
+        <is>
+          <t>Owner hanya bisa melihat Info Pembayaran</t>
+        </is>
+      </c>
+      <c r="E313" s="16" t="inlineStr">
+        <is>
+          <t>Owner bisa mengubahnya</t>
+        </is>
+      </c>
+      <c r="F313" s="16" t="inlineStr">
+        <is>
+          <t>F-SD-02</t>
+        </is>
+      </c>
+      <c r="G313" s="16" t="inlineStr"/>
+      <c r="H313" s="16" t="inlineStr"/>
+      <c r="I313" s="16" t="inlineStr"/>
+    </row>
+    <row r="314">
+      <c r="A314" s="13" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B314" s="14" t="inlineStr">
+        <is>
+          <t>TC-RG-13</t>
+        </is>
+      </c>
+      <c r="C314" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D314" s="13" t="inlineStr">
+        <is>
+          <t>Migrasi gagal: daftar nilai batasan menyempit saat berkas lama dijalankan ulang</t>
+        </is>
+      </c>
+      <c r="E314" s="13" t="inlineStr">
+        <is>
+          <t>Menjalankan ulang berkas mana pun tidak pernah menolak data yang sudah ada</t>
+        </is>
+      </c>
+      <c r="F314" s="13" t="inlineStr">
+        <is>
+          <t>TSD §11.1</t>
+        </is>
+      </c>
+      <c r="G314" s="13" t="inlineStr"/>
+      <c r="H314" s="13" t="inlineStr"/>
+      <c r="I314" s="13" t="inlineStr"/>
+    </row>
+    <row r="315">
+      <c r="A315" s="16" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B315" s="17" t="inlineStr">
+        <is>
+          <t>TC-RG-14</t>
+        </is>
+      </c>
+      <c r="C315" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D315" s="16" t="inlineStr">
+        <is>
+          <t>QR meja borongan bernomor 07, berbeda dengan mode satu meja</t>
+        </is>
+      </c>
+      <c r="E315" s="16" t="inlineStr">
+        <is>
+          <t>Keduanya menulis 7</t>
+        </is>
+      </c>
+      <c r="F315" s="16" t="inlineStr">
+        <is>
+          <t>F-QR-07</t>
+        </is>
+      </c>
+      <c r="G315" s="16" t="inlineStr"/>
+      <c r="H315" s="16" t="inlineStr"/>
+      <c r="I315" s="16" t="inlineStr"/>
+    </row>
+    <row r="316">
+      <c r="A316" s="13" t="inlineStr">
+        <is>
           <t>Uji Ujung-ke-Ujung</t>
         </is>
       </c>
-      <c r="B300" s="14" t="inlineStr">
+      <c r="B316" s="14" t="inlineStr">
         <is>
           <t>E2E-09</t>
         </is>
       </c>
-      <c r="C300" s="15" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D300" s="13" t="inlineStr">
+      <c r="C316" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D316" s="13" t="inlineStr">
         <is>
           <t>Satu siklus langganan penuh</t>
         </is>
       </c>
-      <c r="E300" s="13" t="inlineStr">
+      <c r="E316" s="13" t="inlineStr">
         <is>
           <t>1. Super Admin setel resto uji: Rp 150.000, jatuh tempo 3 hari lagi, tenggang 1 hari
 2. Terbitkan tagihan → periksa muncul di tab Tagihan berstatus Belum Dibayar
@@ -12253,37 +12813,37 @@
 10. Periksa Dashboard Xendit → dana masuk ke akun KaataGo, bukan sub-akun resto</t>
         </is>
       </c>
-      <c r="F300" s="13" t="inlineStr">
+      <c r="F316" s="13" t="inlineStr">
         <is>
           <t>F-BL-07 … F-BL-18, TSD §7.3</t>
         </is>
       </c>
-      <c r="G300" s="13" t="inlineStr"/>
-      <c r="H300" s="13" t="inlineStr"/>
-      <c r="I300" s="13" t="inlineStr"/>
-    </row>
-    <row r="301">
-      <c r="A301" s="16" t="inlineStr">
+      <c r="G316" s="13" t="inlineStr"/>
+      <c r="H316" s="13" t="inlineStr"/>
+      <c r="I316" s="13" t="inlineStr"/>
+    </row>
+    <row r="317">
+      <c r="A317" s="16" t="inlineStr">
         <is>
           <t>Uji Ujung-ke-Ujung</t>
         </is>
       </c>
-      <c r="B301" s="17" t="inlineStr">
+      <c r="B317" s="17" t="inlineStr">
         <is>
           <t>E2E-01</t>
         </is>
       </c>
-      <c r="C301" s="18" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D301" s="16" t="inlineStr">
+      <c r="C317" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D317" s="16" t="inlineStr">
         <is>
           <t>Pelanggan bayar QRIS</t>
         </is>
       </c>
-      <c r="E301" s="16" t="inlineStr">
+      <c r="E317" s="16" t="inlineStr">
         <is>
           <t>1. Pelanggan scan QR meja → pilih 2 menu → Dine In → isi nama
 2. Pilih QRIS → bayar sungguhan dari aplikasi bank
@@ -12295,37 +12855,37 @@
 8. Periksa Saldo → masuk Non Cash, bukan Cash</t>
         </is>
       </c>
-      <c r="F301" s="16" t="inlineStr">
+      <c r="F317" s="16" t="inlineStr">
         <is>
           <t>F-CU-09, F-PG-02, F-CH-06, TSD §6, TSD §7.1</t>
         </is>
       </c>
-      <c r="G301" s="16" t="inlineStr"/>
-      <c r="H301" s="16" t="inlineStr"/>
-      <c r="I301" s="16" t="inlineStr"/>
-    </row>
-    <row r="302">
-      <c r="A302" s="13" t="inlineStr">
+      <c r="G317" s="16" t="inlineStr"/>
+      <c r="H317" s="16" t="inlineStr"/>
+      <c r="I317" s="16" t="inlineStr"/>
+    </row>
+    <row r="318">
+      <c r="A318" s="13" t="inlineStr">
         <is>
           <t>Uji Ujung-ke-Ujung</t>
         </is>
       </c>
-      <c r="B302" s="14" t="inlineStr">
+      <c r="B318" s="14" t="inlineStr">
         <is>
           <t>E2E-02</t>
         </is>
       </c>
-      <c r="C302" s="15" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D302" s="13" t="inlineStr">
+      <c r="C318" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D318" s="13" t="inlineStr">
         <is>
           <t>Pelanggan bayar tunai di kasir</t>
         </is>
       </c>
-      <c r="E302" s="13" t="inlineStr">
+      <c r="E318" s="13" t="inlineStr">
         <is>
           <t>1. Pelanggan pesan → pilih Tunai → catat nomor pesanannya
 2. Periksa layar pelanggan → hitungan mundur 30 menit berjalan
@@ -12337,74 +12897,74 @@
 8. Periksa Saldo Cash → bertambah sebesar totalnya</t>
         </is>
       </c>
-      <c r="F302" s="13" t="inlineStr">
+      <c r="F318" s="13" t="inlineStr">
         <is>
           <t>F-CU-09, F-PP-01, F-PP-06, F-PP-07, F-CH-06, A-02, A-13</t>
         </is>
       </c>
-      <c r="G302" s="13" t="inlineStr"/>
-      <c r="H302" s="13" t="inlineStr"/>
-      <c r="I302" s="13" t="inlineStr"/>
-    </row>
-    <row r="303">
-      <c r="A303" s="16" t="inlineStr">
+      <c r="G318" s="13" t="inlineStr"/>
+      <c r="H318" s="13" t="inlineStr"/>
+      <c r="I318" s="13" t="inlineStr"/>
+    </row>
+    <row r="319">
+      <c r="A319" s="16" t="inlineStr">
         <is>
           <t>Uji Ujung-ke-Ujung</t>
         </is>
       </c>
-      <c r="B303" s="17" t="inlineStr">
+      <c r="B319" s="17" t="inlineStr">
         <is>
           <t>E2E-03</t>
         </is>
       </c>
-      <c r="C303" s="18" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D303" s="16" t="inlineStr">
+      <c r="C319" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D319" s="16" t="inlineStr">
         <is>
           <t>Tunai dengan cara bayar diganti</t>
         </is>
       </c>
-      <c r="E303" s="16" t="inlineStr">
+      <c r="E319" s="16" t="inlineStr">
         <is>
           <t>1. Ulangi E2E-02, tapi pada langkah 4 ganti cara bayarnya ke QRIS.
 2. Pesanannya harus tetap masuk Riwayat Kasir, dan masuk Non Cash
 3. di Saldo.</t>
         </is>
       </c>
-      <c r="F303" s="16" t="inlineStr">
+      <c r="F319" s="16" t="inlineStr">
         <is>
           <t>F-PP-09, A-13, TSD §4.2</t>
         </is>
       </c>
-      <c r="G303" s="16" t="inlineStr"/>
-      <c r="H303" s="16" t="inlineStr"/>
-      <c r="I303" s="16" t="inlineStr"/>
-    </row>
-    <row r="304">
-      <c r="A304" s="13" t="inlineStr">
+      <c r="G319" s="16" t="inlineStr"/>
+      <c r="H319" s="16" t="inlineStr"/>
+      <c r="I319" s="16" t="inlineStr"/>
+    </row>
+    <row r="320">
+      <c r="A320" s="13" t="inlineStr">
         <is>
           <t>Uji Ujung-ke-Ujung</t>
         </is>
       </c>
-      <c r="B304" s="14" t="inlineStr">
+      <c r="B320" s="14" t="inlineStr">
         <is>
           <t>E2E-04</t>
         </is>
       </c>
-      <c r="C304" s="15" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D304" s="13" t="inlineStr">
+      <c r="C320" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D320" s="13" t="inlineStr">
         <is>
           <t>Setor tunai ke rekening</t>
         </is>
       </c>
-      <c r="E304" s="13" t="inlineStr">
+      <c r="E320" s="13" t="inlineStr">
         <is>
           <t>1. Kasir buka Setor Saldo Cash → catat tunai di laci
 2. Ajukan setoran sebesar sebagian dari itu, lampirkan bukti
@@ -12415,73 +12975,73 @@
 7. Periksa Jurnal GL → titipan suspense dilepas, dana masuk GL Total Saldo</t>
         </is>
       </c>
-      <c r="F304" s="13" t="inlineStr">
+      <c r="F320" s="13" t="inlineStr">
         <is>
           <t>F-SD-01, F-SD-05, A-05, TSD §6.4</t>
         </is>
       </c>
-      <c r="G304" s="13" t="inlineStr"/>
-      <c r="H304" s="13" t="inlineStr"/>
-      <c r="I304" s="13" t="inlineStr"/>
-    </row>
-    <row r="305">
-      <c r="A305" s="16" t="inlineStr">
+      <c r="G320" s="13" t="inlineStr"/>
+      <c r="H320" s="13" t="inlineStr"/>
+      <c r="I320" s="13" t="inlineStr"/>
+    </row>
+    <row r="321">
+      <c r="A321" s="16" t="inlineStr">
         <is>
           <t>Uji Ujung-ke-Ujung</t>
         </is>
       </c>
-      <c r="B305" s="17" t="inlineStr">
+      <c r="B321" s="17" t="inlineStr">
         <is>
           <t>E2E-05</t>
         </is>
       </c>
-      <c r="C305" s="18" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D305" s="16" t="inlineStr">
+      <c r="C321" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D321" s="16" t="inlineStr">
         <is>
           <t>Top up petty cash</t>
         </is>
       </c>
-      <c r="E305" s="16" t="inlineStr">
+      <c r="E321" s="16" t="inlineStr">
         <is>
           <t>1. Sama polanya dengan E2E-04, lewat GL Suspense Petty Cash. Top up
 2. Rp 100.000 harus menambah Petty Cash Rp 100.000 — bukan Rp 200.000.</t>
         </is>
       </c>
-      <c r="F305" s="16" t="inlineStr">
+      <c r="F321" s="16" t="inlineStr">
         <is>
           <t>F-FN-03, TSD §6.4</t>
         </is>
       </c>
-      <c r="G305" s="16" t="inlineStr"/>
-      <c r="H305" s="16" t="inlineStr"/>
-      <c r="I305" s="16" t="inlineStr"/>
-    </row>
-    <row r="306">
-      <c r="A306" s="13" t="inlineStr">
+      <c r="G321" s="16" t="inlineStr"/>
+      <c r="H321" s="16" t="inlineStr"/>
+      <c r="I321" s="16" t="inlineStr"/>
+    </row>
+    <row r="322">
+      <c r="A322" s="13" t="inlineStr">
         <is>
           <t>Uji Ujung-ke-Ujung</t>
         </is>
       </c>
-      <c r="B306" s="14" t="inlineStr">
+      <c r="B322" s="14" t="inlineStr">
         <is>
           <t>E2E-06</t>
         </is>
       </c>
-      <c r="C306" s="15" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D306" s="13" t="inlineStr">
+      <c r="C322" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D322" s="13" t="inlineStr">
         <is>
           <t>Promo bundling dari HP pelanggan</t>
         </is>
       </c>
-      <c r="E306" s="13" t="inlineStr">
+      <c r="E322" s="13" t="inlineStr">
         <is>
           <t>1. Admin buat promo: Nasi Goreng Minimal 2 + Es Teh Minimal 1, potongan 30%
 2. Pelanggan pesan 2 Nasi Goreng saja → tidak ada potongan
@@ -12492,37 +13052,37 @@
 7. Admin hapus promonya → cetak ulang struk tadi → potongannya tetap tertulis</t>
         </is>
       </c>
-      <c r="F306" s="13" t="inlineStr">
+      <c r="F322" s="13" t="inlineStr">
         <is>
           <t>F-DS-10, F-DS-12, F-CU-17, F-DS-08, F-DS-09, A-14</t>
         </is>
       </c>
-      <c r="G306" s="13" t="inlineStr"/>
-      <c r="H306" s="13" t="inlineStr"/>
-      <c r="I306" s="13" t="inlineStr"/>
-    </row>
-    <row r="307">
-      <c r="A307" s="16" t="inlineStr">
+      <c r="G322" s="13" t="inlineStr"/>
+      <c r="H322" s="13" t="inlineStr"/>
+      <c r="I322" s="13" t="inlineStr"/>
+    </row>
+    <row r="323">
+      <c r="A323" s="16" t="inlineStr">
         <is>
           <t>Uji Ujung-ke-Ujung</t>
         </is>
       </c>
-      <c r="B307" s="17" t="inlineStr">
+      <c r="B323" s="17" t="inlineStr">
         <is>
           <t>E2E-07</t>
         </is>
       </c>
-      <c r="C307" s="18" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D307" s="16" t="inlineStr">
+      <c r="C323" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D323" s="16" t="inlineStr">
         <is>
           <t>Pembatalan oleh pelanggan</t>
         </is>
       </c>
-      <c r="E307" s="16" t="inlineStr">
+      <c r="E323" s="16" t="inlineStr">
         <is>
           <t>1. Pelanggan pesan, pilih Tunai
 2. Batalkan dari Pesanan Saya → berhasil
@@ -12532,37 +13092,37 @@
 6. Periksa Riwayat Kasir → tidak ikut terhitung</t>
         </is>
       </c>
-      <c r="F307" s="16" t="inlineStr">
+      <c r="F323" s="16" t="inlineStr">
         <is>
           <t>F-CN-01, A-17</t>
         </is>
       </c>
-      <c r="G307" s="16" t="inlineStr"/>
-      <c r="H307" s="16" t="inlineStr"/>
-      <c r="I307" s="16" t="inlineStr"/>
-    </row>
-    <row r="308">
-      <c r="A308" s="13" t="inlineStr">
+      <c r="G323" s="16" t="inlineStr"/>
+      <c r="H323" s="16" t="inlineStr"/>
+      <c r="I323" s="16" t="inlineStr"/>
+    </row>
+    <row r="324">
+      <c r="A324" s="13" t="inlineStr">
         <is>
           <t>Uji Ujung-ke-Ujung</t>
         </is>
       </c>
-      <c r="B308" s="14" t="inlineStr">
+      <c r="B324" s="14" t="inlineStr">
         <is>
           <t>E2E-08</t>
         </is>
       </c>
-      <c r="C308" s="15" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D308" s="13" t="inlineStr">
+      <c r="C324" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D324" s="13" t="inlineStr">
         <is>
           <t>Isolasi antar cabang</t>
         </is>
       </c>
-      <c r="E308" s="13" t="inlineStr">
+      <c r="E324" s="13" t="inlineStr">
         <is>
           <t>1. Dengan akun Owner yang memiliki dua resto: buat transaksi, promo, dan
 2. pengumuman di resto A, lalu berpindah ke resto B. Tidak satu pun
@@ -12570,19 +13130,19 @@
 4. dan kotak masuk.</t>
         </is>
       </c>
-      <c r="F308" s="13" t="inlineStr">
+      <c r="F324" s="13" t="inlineStr">
         <is>
           <t>F-AD-08, F-IN-10, A-10</t>
         </is>
       </c>
-      <c r="G308" s="13" t="inlineStr"/>
-      <c r="H308" s="13" t="inlineStr"/>
-      <c r="I308" s="13" t="inlineStr"/>
+      <c r="G324" s="13" t="inlineStr"/>
+      <c r="H324" s="13" t="inlineStr"/>
+      <c r="I324" s="13" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I308"/>
+  <autoFilter ref="A1:I324"/>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G308" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G324" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Lulus,Gagal,Terblokir,Dilewati"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Jurnal Semua Resto hanya resto klien, dan renumber tanpa tabel sementara
Pembukuan KaataGo disaring keluar. Barisnya memang tersimpan di tabel
yang sama, tapi mencampurnya membuat total debit/kredit menjumlahkan
dua pembukuan yang tidak punya hubungan: penjualan resto, dan tagihan
yang kami terbitkan kepada mereka.

Disaring di kueri, bukan sesudah data sampai — baris platform yang ikut
terangkut memakan jatah batas 1.000 baris, dan yang terpotong justru
jurnal resto yang dicari.

Tabel sementara di berkas renumber diganti daftar sebaris: ia hanya
hidup di satu sesi, dan SQL Editor Supabase bisa menjalankan tiap
pernyataan lewat koneksi berbeda. Galatnya lalu muncul di pernyataan
KEDUA, bukan pada yang membuat tabelnya — jadi yang membacanya
menyangka UPDATE-nya yang salah.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/TEST-CASE-KAATAGO.xlsx
+++ b/docs/TEST-CASE-KAATAGO.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cara Lampirkan Capture" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kasus Uji'!$A$1:$I$324</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kasus Uji'!$A$1:$I$328</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Defect'!$A$4:$V$64</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -691,23 +691,23 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIF('Kasus Uji'!C2:C324,"P1")</f>
+        <f>COUNTIF('Kasus Uji'!C2:C328,"P1")</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C324,"P1",'Kasus Uji'!G2:G324,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C328,"P1",'Kasus Uji'!G2:G328,"Lulus")</f>
         <v/>
       </c>
       <c r="D5" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C324,"P1",'Kasus Uji'!G2:G324,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C328,"P1",'Kasus Uji'!G2:G328,"Gagal")</f>
         <v/>
       </c>
       <c r="E5" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C324,"P1",'Kasus Uji'!G2:G324,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C328,"P1",'Kasus Uji'!G2:G328,"Terblokir")</f>
         <v/>
       </c>
       <c r="F5" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C324,"P1",'Kasus Uji'!G2:G324,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C328,"P1",'Kasus Uji'!G2:G328,"Dilewati")</f>
         <v/>
       </c>
       <c r="G5" s="5">
@@ -722,23 +722,23 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('Kasus Uji'!C2:C324,"P2")</f>
+        <f>COUNTIF('Kasus Uji'!C2:C328,"P2")</f>
         <v/>
       </c>
       <c r="C6" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C324,"P2",'Kasus Uji'!G2:G324,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C328,"P2",'Kasus Uji'!G2:G328,"Lulus")</f>
         <v/>
       </c>
       <c r="D6" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C324,"P2",'Kasus Uji'!G2:G324,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C328,"P2",'Kasus Uji'!G2:G328,"Gagal")</f>
         <v/>
       </c>
       <c r="E6" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C324,"P2",'Kasus Uji'!G2:G324,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C328,"P2",'Kasus Uji'!G2:G328,"Terblokir")</f>
         <v/>
       </c>
       <c r="F6" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C324,"P2",'Kasus Uji'!G2:G324,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C328,"P2",'Kasus Uji'!G2:G328,"Dilewati")</f>
         <v/>
       </c>
       <c r="G6" s="5">
@@ -753,23 +753,23 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('Kasus Uji'!C2:C324,"P3")</f>
+        <f>COUNTIF('Kasus Uji'!C2:C328,"P3")</f>
         <v/>
       </c>
       <c r="C7" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C324,"P3",'Kasus Uji'!G2:G324,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C328,"P3",'Kasus Uji'!G2:G328,"Lulus")</f>
         <v/>
       </c>
       <c r="D7" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C324,"P3",'Kasus Uji'!G2:G324,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C328,"P3",'Kasus Uji'!G2:G328,"Gagal")</f>
         <v/>
       </c>
       <c r="E7" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C324,"P3",'Kasus Uji'!G2:G324,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C328,"P3",'Kasus Uji'!G2:G328,"Terblokir")</f>
         <v/>
       </c>
       <c r="F7" s="5">
-        <f>COUNTIFS('Kasus Uji'!C2:C324,"P3",'Kasus Uji'!G2:G324,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!C2:C328,"P3",'Kasus Uji'!G2:G328,"Dilewati")</f>
         <v/>
       </c>
       <c r="G7" s="5">
@@ -859,23 +859,23 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A324,"Pelanggan")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A328,"Pelanggan")</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pelanggan",'Kasus Uji'!G2:G324,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Pelanggan",'Kasus Uji'!G2:G328,"Lulus")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pelanggan",'Kasus Uji'!G2:G324,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Pelanggan",'Kasus Uji'!G2:G328,"Gagal")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pelanggan",'Kasus Uji'!G2:G324,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Pelanggan",'Kasus Uji'!G2:G328,"Terblokir")</f>
         <v/>
       </c>
       <c r="F12" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pelanggan",'Kasus Uji'!G2:G324,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Pelanggan",'Kasus Uji'!G2:G328,"Dilewati")</f>
         <v/>
       </c>
       <c r="G12" s="5">
@@ -890,23 +890,23 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A324,"Kasir")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A328,"Kasir")</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Kasir",'Kasus Uji'!G2:G324,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Kasir",'Kasus Uji'!G2:G328,"Lulus")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Kasir",'Kasus Uji'!G2:G324,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Kasir",'Kasus Uji'!G2:G328,"Gagal")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Kasir",'Kasus Uji'!G2:G324,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Kasir",'Kasus Uji'!G2:G328,"Terblokir")</f>
         <v/>
       </c>
       <c r="F13" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Kasir",'Kasus Uji'!G2:G324,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Kasir",'Kasus Uji'!G2:G328,"Dilewati")</f>
         <v/>
       </c>
       <c r="G13" s="5">
@@ -921,23 +921,23 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A324,"Pending Payment")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A328,"Pending Payment")</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pending Payment",'Kasus Uji'!G2:G324,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Pending Payment",'Kasus Uji'!G2:G328,"Lulus")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pending Payment",'Kasus Uji'!G2:G324,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Pending Payment",'Kasus Uji'!G2:G328,"Gagal")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pending Payment",'Kasus Uji'!G2:G324,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Pending Payment",'Kasus Uji'!G2:G328,"Terblokir")</f>
         <v/>
       </c>
       <c r="F14" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pending Payment",'Kasus Uji'!G2:G324,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Pending Payment",'Kasus Uji'!G2:G328,"Dilewati")</f>
         <v/>
       </c>
       <c r="G14" s="5">
@@ -952,23 +952,23 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A324,"Dapur")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A328,"Dapur")</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Dapur",'Kasus Uji'!G2:G324,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Dapur",'Kasus Uji'!G2:G328,"Lulus")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Dapur",'Kasus Uji'!G2:G324,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Dapur",'Kasus Uji'!G2:G328,"Gagal")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Dapur",'Kasus Uji'!G2:G324,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Dapur",'Kasus Uji'!G2:G328,"Terblokir")</f>
         <v/>
       </c>
       <c r="F15" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Dapur",'Kasus Uji'!G2:G324,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Dapur",'Kasus Uji'!G2:G328,"Dilewati")</f>
         <v/>
       </c>
       <c r="G15" s="5">
@@ -983,23 +983,23 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A324,"Keuangan")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A328,"Keuangan")</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Keuangan",'Kasus Uji'!G2:G324,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Keuangan",'Kasus Uji'!G2:G328,"Lulus")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Keuangan",'Kasus Uji'!G2:G324,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Keuangan",'Kasus Uji'!G2:G328,"Gagal")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Keuangan",'Kasus Uji'!G2:G324,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Keuangan",'Kasus Uji'!G2:G328,"Terblokir")</f>
         <v/>
       </c>
       <c r="F16" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Keuangan",'Kasus Uji'!G2:G324,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Keuangan",'Kasus Uji'!G2:G328,"Dilewati")</f>
         <v/>
       </c>
       <c r="G16" s="5">
@@ -1014,23 +1014,23 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A324,"Setor Saldo Cash")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A328,"Setor Saldo Cash")</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Setor Saldo Cash",'Kasus Uji'!G2:G324,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Setor Saldo Cash",'Kasus Uji'!G2:G328,"Lulus")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Setor Saldo Cash",'Kasus Uji'!G2:G324,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Setor Saldo Cash",'Kasus Uji'!G2:G328,"Gagal")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Setor Saldo Cash",'Kasus Uji'!G2:G324,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Setor Saldo Cash",'Kasus Uji'!G2:G328,"Terblokir")</f>
         <v/>
       </c>
       <c r="F17" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Setor Saldo Cash",'Kasus Uji'!G2:G324,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Setor Saldo Cash",'Kasus Uji'!G2:G328,"Dilewati")</f>
         <v/>
       </c>
       <c r="G17" s="5">
@@ -1045,23 +1045,23 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A324,"Katalog &amp; Pengaturan")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A328,"Katalog &amp; Pengaturan")</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Katalog &amp; Pengaturan",'Kasus Uji'!G2:G324,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Katalog &amp; Pengaturan",'Kasus Uji'!G2:G328,"Lulus")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Katalog &amp; Pengaturan",'Kasus Uji'!G2:G324,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Katalog &amp; Pengaturan",'Kasus Uji'!G2:G328,"Gagal")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Katalog &amp; Pengaturan",'Kasus Uji'!G2:G324,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Katalog &amp; Pengaturan",'Kasus Uji'!G2:G328,"Terblokir")</f>
         <v/>
       </c>
       <c r="F18" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Katalog &amp; Pengaturan",'Kasus Uji'!G2:G324,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Katalog &amp; Pengaturan",'Kasus Uji'!G2:G328,"Dilewati")</f>
         <v/>
       </c>
       <c r="G18" s="5">
@@ -1076,23 +1076,23 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A324,"QR Meja")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A328,"QR Meja")</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"QR Meja",'Kasus Uji'!G2:G324,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"QR Meja",'Kasus Uji'!G2:G328,"Lulus")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"QR Meja",'Kasus Uji'!G2:G324,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"QR Meja",'Kasus Uji'!G2:G328,"Gagal")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"QR Meja",'Kasus Uji'!G2:G324,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"QR Meja",'Kasus Uji'!G2:G328,"Terblokir")</f>
         <v/>
       </c>
       <c r="F19" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"QR Meja",'Kasus Uji'!G2:G324,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"QR Meja",'Kasus Uji'!G2:G328,"Dilewati")</f>
         <v/>
       </c>
       <c r="G19" s="5">
@@ -1107,23 +1107,23 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A324,"Diskon")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A328,"Diskon")</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Diskon",'Kasus Uji'!G2:G324,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Diskon",'Kasus Uji'!G2:G328,"Lulus")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Diskon",'Kasus Uji'!G2:G324,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Diskon",'Kasus Uji'!G2:G328,"Gagal")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Diskon",'Kasus Uji'!G2:G324,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Diskon",'Kasus Uji'!G2:G328,"Terblokir")</f>
         <v/>
       </c>
       <c r="F20" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Diskon",'Kasus Uji'!G2:G324,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Diskon",'Kasus Uji'!G2:G328,"Dilewati")</f>
         <v/>
       </c>
       <c r="G20" s="5">
@@ -1138,23 +1138,23 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A324,"Kotak Masuk &amp; Pengumuman")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A328,"Kotak Masuk &amp; Pengumuman")</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Kotak Masuk &amp; Pengumuman",'Kasus Uji'!G2:G324,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Kotak Masuk &amp; Pengumuman",'Kasus Uji'!G2:G328,"Lulus")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Kotak Masuk &amp; Pengumuman",'Kasus Uji'!G2:G324,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Kotak Masuk &amp; Pengumuman",'Kasus Uji'!G2:G328,"Gagal")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Kotak Masuk &amp; Pengumuman",'Kasus Uji'!G2:G324,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Kotak Masuk &amp; Pengumuman",'Kasus Uji'!G2:G328,"Terblokir")</f>
         <v/>
       </c>
       <c r="F21" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Kotak Masuk &amp; Pengumuman",'Kasus Uji'!G2:G324,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Kotak Masuk &amp; Pengumuman",'Kasus Uji'!G2:G328,"Dilewati")</f>
         <v/>
       </c>
       <c r="G21" s="5">
@@ -1169,23 +1169,23 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A324,"Pembayaran QRIS")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A328,"Pembayaran QRIS")</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pembayaran QRIS",'Kasus Uji'!G2:G324,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Pembayaran QRIS",'Kasus Uji'!G2:G328,"Lulus")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pembayaran QRIS",'Kasus Uji'!G2:G324,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Pembayaran QRIS",'Kasus Uji'!G2:G328,"Gagal")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pembayaran QRIS",'Kasus Uji'!G2:G324,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Pembayaran QRIS",'Kasus Uji'!G2:G328,"Terblokir")</f>
         <v/>
       </c>
       <c r="F22" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pembayaran QRIS",'Kasus Uji'!G2:G324,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Pembayaran QRIS",'Kasus Uji'!G2:G328,"Dilewati")</f>
         <v/>
       </c>
       <c r="G22" s="5">
@@ -1200,23 +1200,23 @@
         </is>
       </c>
       <c r="B23" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A324,"Pembatalan &amp; Kedaluwarsa")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A328,"Pembatalan &amp; Kedaluwarsa")</f>
         <v/>
       </c>
       <c r="C23" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pembatalan &amp; Kedaluwarsa",'Kasus Uji'!G2:G324,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Pembatalan &amp; Kedaluwarsa",'Kasus Uji'!G2:G328,"Lulus")</f>
         <v/>
       </c>
       <c r="D23" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pembatalan &amp; Kedaluwarsa",'Kasus Uji'!G2:G324,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Pembatalan &amp; Kedaluwarsa",'Kasus Uji'!G2:G328,"Gagal")</f>
         <v/>
       </c>
       <c r="E23" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pembatalan &amp; Kedaluwarsa",'Kasus Uji'!G2:G324,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Pembatalan &amp; Kedaluwarsa",'Kasus Uji'!G2:G328,"Terblokir")</f>
         <v/>
       </c>
       <c r="F23" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pembatalan &amp; Kedaluwarsa",'Kasus Uji'!G2:G324,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Pembatalan &amp; Kedaluwarsa",'Kasus Uji'!G2:G328,"Dilewati")</f>
         <v/>
       </c>
       <c r="G23" s="5">
@@ -1231,23 +1231,23 @@
         </is>
       </c>
       <c r="B24" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A324,"Sesi Meja &amp; Identitas")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A328,"Sesi Meja &amp; Identitas")</f>
         <v/>
       </c>
       <c r="C24" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Sesi Meja &amp; Identitas",'Kasus Uji'!G2:G324,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Sesi Meja &amp; Identitas",'Kasus Uji'!G2:G328,"Lulus")</f>
         <v/>
       </c>
       <c r="D24" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Sesi Meja &amp; Identitas",'Kasus Uji'!G2:G324,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Sesi Meja &amp; Identitas",'Kasus Uji'!G2:G328,"Gagal")</f>
         <v/>
       </c>
       <c r="E24" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Sesi Meja &amp; Identitas",'Kasus Uji'!G2:G324,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Sesi Meja &amp; Identitas",'Kasus Uji'!G2:G328,"Terblokir")</f>
         <v/>
       </c>
       <c r="F24" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Sesi Meja &amp; Identitas",'Kasus Uji'!G2:G324,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Sesi Meja &amp; Identitas",'Kasus Uji'!G2:G328,"Dilewati")</f>
         <v/>
       </c>
       <c r="G24" s="5">
@@ -1262,23 +1262,23 @@
         </is>
       </c>
       <c r="B25" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A324,"Tampilan")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A328,"Tampilan")</f>
         <v/>
       </c>
       <c r="C25" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Tampilan",'Kasus Uji'!G2:G324,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Tampilan",'Kasus Uji'!G2:G328,"Lulus")</f>
         <v/>
       </c>
       <c r="D25" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Tampilan",'Kasus Uji'!G2:G324,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Tampilan",'Kasus Uji'!G2:G328,"Gagal")</f>
         <v/>
       </c>
       <c r="E25" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Tampilan",'Kasus Uji'!G2:G324,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Tampilan",'Kasus Uji'!G2:G328,"Terblokir")</f>
         <v/>
       </c>
       <c r="F25" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Tampilan",'Kasus Uji'!G2:G324,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Tampilan",'Kasus Uji'!G2:G328,"Dilewati")</f>
         <v/>
       </c>
       <c r="G25" s="5">
@@ -1293,23 +1293,23 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A324,"Super Admin")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A328,"Super Admin")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Super Admin",'Kasus Uji'!G2:G324,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Super Admin",'Kasus Uji'!G2:G328,"Lulus")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Super Admin",'Kasus Uji'!G2:G324,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Super Admin",'Kasus Uji'!G2:G328,"Gagal")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Super Admin",'Kasus Uji'!G2:G324,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Super Admin",'Kasus Uji'!G2:G328,"Terblokir")</f>
         <v/>
       </c>
       <c r="F26" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Super Admin",'Kasus Uji'!G2:G324,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Super Admin",'Kasus Uji'!G2:G328,"Dilewati")</f>
         <v/>
       </c>
       <c r="G26" s="5">
@@ -1324,23 +1324,23 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A324,"Pembaruan Aplikasi")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A328,"Pembaruan Aplikasi")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pembaruan Aplikasi",'Kasus Uji'!G2:G324,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Pembaruan Aplikasi",'Kasus Uji'!G2:G328,"Lulus")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pembaruan Aplikasi",'Kasus Uji'!G2:G324,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Pembaruan Aplikasi",'Kasus Uji'!G2:G328,"Gagal")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pembaruan Aplikasi",'Kasus Uji'!G2:G324,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Pembaruan Aplikasi",'Kasus Uji'!G2:G328,"Terblokir")</f>
         <v/>
       </c>
       <c r="F27" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Pembaruan Aplikasi",'Kasus Uji'!G2:G324,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Pembaruan Aplikasi",'Kasus Uji'!G2:G328,"Dilewati")</f>
         <v/>
       </c>
       <c r="G27" s="5">
@@ -1355,23 +1355,23 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A324,"## 19b. Langganan &amp; Tagihan Resto")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A328,"## 19b. Langganan &amp; Tagihan Resto")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"## 19b. Langganan &amp; Tagihan Resto",'Kasus Uji'!G2:G324,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"## 19b. Langganan &amp; Tagihan Resto",'Kasus Uji'!G2:G328,"Lulus")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"## 19b. Langganan &amp; Tagihan Resto",'Kasus Uji'!G2:G324,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"## 19b. Langganan &amp; Tagihan Resto",'Kasus Uji'!G2:G328,"Gagal")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"## 19b. Langganan &amp; Tagihan Resto",'Kasus Uji'!G2:G324,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"## 19b. Langganan &amp; Tagihan Resto",'Kasus Uji'!G2:G328,"Terblokir")</f>
         <v/>
       </c>
       <c r="F28" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"## 19b. Langganan &amp; Tagihan Resto",'Kasus Uji'!G2:G324,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"## 19b. Langganan &amp; Tagihan Resto",'Kasus Uji'!G2:G328,"Dilewati")</f>
         <v/>
       </c>
       <c r="G28" s="5">
@@ -1386,23 +1386,23 @@
         </is>
       </c>
       <c r="B29" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A324,"## 19c. Finance KaataGo (Super Admin)")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A328,"## 19c. Finance KaataGo (Super Admin)")</f>
         <v/>
       </c>
       <c r="C29" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"## 19c. Finance KaataGo (Super Admin)",'Kasus Uji'!G2:G324,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"## 19c. Finance KaataGo (Super Admin)",'Kasus Uji'!G2:G328,"Lulus")</f>
         <v/>
       </c>
       <c r="D29" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"## 19c. Finance KaataGo (Super Admin)",'Kasus Uji'!G2:G324,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"## 19c. Finance KaataGo (Super Admin)",'Kasus Uji'!G2:G328,"Gagal")</f>
         <v/>
       </c>
       <c r="E29" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"## 19c. Finance KaataGo (Super Admin)",'Kasus Uji'!G2:G324,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"## 19c. Finance KaataGo (Super Admin)",'Kasus Uji'!G2:G328,"Terblokir")</f>
         <v/>
       </c>
       <c r="F29" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"## 19c. Finance KaataGo (Super Admin)",'Kasus Uji'!G2:G324,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"## 19c. Finance KaataGo (Super Admin)",'Kasus Uji'!G2:G328,"Dilewati")</f>
         <v/>
       </c>
       <c r="G29" s="5">
@@ -1417,23 +1417,23 @@
         </is>
       </c>
       <c r="B30" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A324,"Uji Teknis (lingkup TSD)")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A328,"Uji Teknis (lingkup TSD)")</f>
         <v/>
       </c>
       <c r="C30" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Uji Teknis (lingkup TSD)",'Kasus Uji'!G2:G324,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Uji Teknis (lingkup TSD)",'Kasus Uji'!G2:G328,"Lulus")</f>
         <v/>
       </c>
       <c r="D30" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Uji Teknis (lingkup TSD)",'Kasus Uji'!G2:G324,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Uji Teknis (lingkup TSD)",'Kasus Uji'!G2:G328,"Gagal")</f>
         <v/>
       </c>
       <c r="E30" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Uji Teknis (lingkup TSD)",'Kasus Uji'!G2:G324,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Uji Teknis (lingkup TSD)",'Kasus Uji'!G2:G328,"Terblokir")</f>
         <v/>
       </c>
       <c r="F30" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Uji Teknis (lingkup TSD)",'Kasus Uji'!G2:G324,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Uji Teknis (lingkup TSD)",'Kasus Uji'!G2:G328,"Dilewati")</f>
         <v/>
       </c>
       <c r="G30" s="5">
@@ -1448,23 +1448,23 @@
         </is>
       </c>
       <c r="B31" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A324,"Regresi — bug yang pernah terjadi")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A328,"Regresi — bug yang pernah terjadi")</f>
         <v/>
       </c>
       <c r="C31" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Regresi — bug yang pernah terjadi",'Kasus Uji'!G2:G324,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Regresi — bug yang pernah terjadi",'Kasus Uji'!G2:G328,"Lulus")</f>
         <v/>
       </c>
       <c r="D31" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Regresi — bug yang pernah terjadi",'Kasus Uji'!G2:G324,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Regresi — bug yang pernah terjadi",'Kasus Uji'!G2:G328,"Gagal")</f>
         <v/>
       </c>
       <c r="E31" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Regresi — bug yang pernah terjadi",'Kasus Uji'!G2:G324,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Regresi — bug yang pernah terjadi",'Kasus Uji'!G2:G328,"Terblokir")</f>
         <v/>
       </c>
       <c r="F31" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Regresi — bug yang pernah terjadi",'Kasus Uji'!G2:G324,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Regresi — bug yang pernah terjadi",'Kasus Uji'!G2:G328,"Dilewati")</f>
         <v/>
       </c>
       <c r="G31" s="5">
@@ -1479,23 +1479,23 @@
         </is>
       </c>
       <c r="B32" s="5">
-        <f>COUNTIF('Kasus Uji'!A2:A324,"Uji Ujung-ke-Ujung")</f>
+        <f>COUNTIF('Kasus Uji'!A2:A328,"Uji Ujung-ke-Ujung")</f>
         <v/>
       </c>
       <c r="C32" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Uji Ujung-ke-Ujung",'Kasus Uji'!G2:G324,"Lulus")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Uji Ujung-ke-Ujung",'Kasus Uji'!G2:G328,"Lulus")</f>
         <v/>
       </c>
       <c r="D32" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Uji Ujung-ke-Ujung",'Kasus Uji'!G2:G324,"Gagal")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Uji Ujung-ke-Ujung",'Kasus Uji'!G2:G328,"Gagal")</f>
         <v/>
       </c>
       <c r="E32" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Uji Ujung-ke-Ujung",'Kasus Uji'!G2:G324,"Terblokir")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Uji Ujung-ke-Ujung",'Kasus Uji'!G2:G328,"Terblokir")</f>
         <v/>
       </c>
       <c r="F32" s="5">
-        <f>COUNTIFS('Kasus Uji'!A2:A324,"Uji Ujung-ke-Ujung",'Kasus Uji'!G2:G324,"Dilewati")</f>
+        <f>COUNTIFS('Kasus Uji'!A2:A328,"Uji Ujung-ke-Ujung",'Kasus Uji'!G2:G328,"Dilewati")</f>
         <v/>
       </c>
       <c r="G32" s="5">
@@ -1727,7 +1727,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I324"/>
+  <dimension ref="A1:I328"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -11626,12 +11626,12 @@
     <row r="283">
       <c r="A283" s="16" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19c. Finance KaataGo (Super Admin)</t>
         </is>
       </c>
       <c r="B283" s="17" t="inlineStr">
         <is>
-          <t>TC-TS-01</t>
+          <t>TC-PF-31</t>
         </is>
       </c>
       <c r="C283" s="18" t="inlineStr">
@@ -11641,17 +11641,17 @@
       </c>
       <c r="D283" s="16" t="inlineStr">
         <is>
-          <t>Panggil GET /rest/v1/orders memakai kunci anon tanpa login</t>
+          <t>Buka Jurnal GL Semua Resto sesudah ada tagihan langganan lunas</t>
         </is>
       </c>
       <c r="E283" s="16" t="inlineStr">
         <is>
-          <t>Tidak mengembalikan pesanan resto mana pun</t>
+          <t>Baris pendapatan langganan tidak muncul di sana</t>
         </is>
       </c>
       <c r="F283" s="16" t="inlineStr">
         <is>
-          <t>TSD §5</t>
+          <t>F-PF-21</t>
         </is>
       </c>
       <c r="G283" s="16" t="inlineStr"/>
@@ -11661,12 +11661,12 @@
     <row r="284">
       <c r="A284" s="13" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19c. Finance KaataGo (Super Admin)</t>
         </is>
       </c>
       <c r="B284" s="14" t="inlineStr">
         <is>
-          <t>TC-TS-02</t>
+          <t>TC-PF-32</t>
         </is>
       </c>
       <c r="C284" s="15" t="inlineStr">
@@ -11676,17 +11676,17 @@
       </c>
       <c r="D284" s="13" t="inlineStr">
         <is>
-          <t>Login sebagai karyawan resto A, baca orders resto B lewat API</t>
+          <t>Buka daftar saringan resto</t>
         </is>
       </c>
       <c r="E284" s="13" t="inlineStr">
         <is>
-          <t>Kosong — bukan galat, tapi juga bukan data</t>
+          <t>KaataGo tidak ada di daftarnya</t>
         </is>
       </c>
       <c r="F284" s="13" t="inlineStr">
         <is>
-          <t>TSD §5</t>
+          <t>F-PF-21</t>
         </is>
       </c>
       <c r="G284" s="13" t="inlineStr"/>
@@ -11696,12 +11696,12 @@
     <row r="285">
       <c r="A285" s="16" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19c. Finance KaataGo (Super Admin)</t>
         </is>
       </c>
       <c r="B285" s="17" t="inlineStr">
         <is>
-          <t>TC-TS-03</t>
+          <t>TC-PF-33</t>
         </is>
       </c>
       <c r="C285" s="18" t="inlineStr">
@@ -11711,17 +11711,17 @@
       </c>
       <c r="D285" s="16" t="inlineStr">
         <is>
-          <t>Login sebagai Owner, buka tiap layar resto miliknya</t>
+          <t>Buka Jurnal GL KaataGo</t>
         </is>
       </c>
       <c r="E285" s="16" t="inlineStr">
         <is>
-          <t>Tidak ada layar yang kosong karena RLS — owner harus disebut di setiap daftar peran</t>
+          <t>Pendapatan langganan ada di sana, dan Saldo Total tidak nol</t>
         </is>
       </c>
       <c r="F285" s="16" t="inlineStr">
         <is>
-          <t>TSD §5</t>
+          <t>F-PF-07</t>
         </is>
       </c>
       <c r="G285" s="16" t="inlineStr"/>
@@ -11731,32 +11731,32 @@
     <row r="286">
       <c r="A286" s="13" t="inlineStr">
         <is>
-          <t>Uji Teknis (lingkup TSD)</t>
+          <t>## 19c. Finance KaataGo (Super Admin)</t>
         </is>
       </c>
       <c r="B286" s="14" t="inlineStr">
         <is>
-          <t>TC-TS-04</t>
-        </is>
-      </c>
-      <c r="C286" s="15" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>TC-PF-34</t>
+        </is>
+      </c>
+      <c r="C286" s="19" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D286" s="13" t="inlineStr">
         <is>
-          <t>Login sebagai Kasir, baca gl_journal_entries</t>
+          <t>Periksa nomor akun di Jurnal GL KaataGo</t>
         </is>
       </c>
       <c r="E286" s="13" t="inlineStr">
         <is>
-          <t>Hanya yang terkait catatan yang memang boleh dia lihat</t>
+          <t>Golongan 11xxxxx, berbeda dari 19xxxxx milik resto</t>
         </is>
       </c>
       <c r="F286" s="13" t="inlineStr">
         <is>
-          <t>F-KS-13, TSD §5.1</t>
+          <t>F-PF-08</t>
         </is>
       </c>
       <c r="G286" s="13" t="inlineStr"/>
@@ -11771,7 +11771,7 @@
       </c>
       <c r="B287" s="17" t="inlineStr">
         <is>
-          <t>TC-TS-05</t>
+          <t>TC-TS-01</t>
         </is>
       </c>
       <c r="C287" s="18" t="inlineStr">
@@ -11781,17 +11781,17 @@
       </c>
       <c r="D287" s="16" t="inlineStr">
         <is>
-          <t>Coba UPDATE products langsung lewat API sebagai pelanggan</t>
+          <t>Panggil GET /rest/v1/orders memakai kunci anon tanpa login</t>
         </is>
       </c>
       <c r="E287" s="16" t="inlineStr">
         <is>
-          <t>Ditolak; pengurangan stok hanya lewat decrement_stock</t>
+          <t>Tidak mengembalikan pesanan resto mana pun</t>
         </is>
       </c>
       <c r="F287" s="16" t="inlineStr">
         <is>
-          <t>TSD §5.2</t>
+          <t>TSD §5</t>
         </is>
       </c>
       <c r="G287" s="16" t="inlineStr"/>
@@ -11806,7 +11806,7 @@
       </c>
       <c r="B288" s="14" t="inlineStr">
         <is>
-          <t>TC-TS-06</t>
+          <t>TC-TS-02</t>
         </is>
       </c>
       <c r="C288" s="15" t="inlineStr">
@@ -11816,17 +11816,17 @@
       </c>
       <c r="D288" s="13" t="inlineStr">
         <is>
-          <t>Panggil cancel_my_order untuk pesanan milik orang lain</t>
+          <t>Login sebagai karyawan resto A, baca orders resto B lewat API</t>
         </is>
       </c>
       <c r="E288" s="13" t="inlineStr">
         <is>
-          <t>Ditolak</t>
+          <t>Kosong — bukan galat, tapi juga bukan data</t>
         </is>
       </c>
       <c r="F288" s="13" t="inlineStr">
         <is>
-          <t>TSD §5.2</t>
+          <t>TSD §5</t>
         </is>
       </c>
       <c r="G288" s="13" t="inlineStr"/>
@@ -11841,7 +11841,7 @@
       </c>
       <c r="B289" s="17" t="inlineStr">
         <is>
-          <t>TC-TS-07</t>
+          <t>TC-TS-03</t>
         </is>
       </c>
       <c r="C289" s="18" t="inlineStr">
@@ -11851,17 +11851,17 @@
       </c>
       <c r="D289" s="16" t="inlineStr">
         <is>
-          <t>Jalankan ulang seluruh JALANKAN-INI.sql di database yang sudah terisi</t>
+          <t>Login sebagai Owner, buka tiap layar resto miliknya</t>
         </is>
       </c>
       <c r="E289" s="16" t="inlineStr">
         <is>
-          <t>Selesai tanpa galat; tidak ada data yang berubah</t>
+          <t>Tidak ada layar yang kosong karena RLS — owner harus disebut di setiap daftar peran</t>
         </is>
       </c>
       <c r="F289" s="16" t="inlineStr">
         <is>
-          <t>TSD §11</t>
+          <t>TSD §5</t>
         </is>
       </c>
       <c r="G289" s="16" t="inlineStr"/>
@@ -11876,7 +11876,7 @@
       </c>
       <c r="B290" s="14" t="inlineStr">
         <is>
-          <t>TC-TS-08</t>
+          <t>TC-TS-04</t>
         </is>
       </c>
       <c r="C290" s="15" t="inlineStr">
@@ -11886,17 +11886,17 @@
       </c>
       <c r="D290" s="13" t="inlineStr">
         <is>
-          <t>Jalankan ulang satu berkas SQL lama saja, misal cash_payment_expiry.sql</t>
+          <t>Login sebagai Kasir, baca gl_journal_entries</t>
         </is>
       </c>
       <c r="E290" s="13" t="inlineStr">
         <is>
-          <t>Tidak menyempitkan daftar nilai batasan mana pun</t>
+          <t>Hanya yang terkait catatan yang memang boleh dia lihat</t>
         </is>
       </c>
       <c r="F290" s="13" t="inlineStr">
         <is>
-          <t>TSD §11.1</t>
+          <t>F-KS-13, TSD §5.1</t>
         </is>
       </c>
       <c r="G290" s="13" t="inlineStr"/>
@@ -11911,7 +11911,7 @@
       </c>
       <c r="B291" s="17" t="inlineStr">
         <is>
-          <t>TC-TS-09</t>
+          <t>TC-TS-05</t>
         </is>
       </c>
       <c r="C291" s="18" t="inlineStr">
@@ -11921,17 +11921,17 @@
       </c>
       <c r="D291" s="16" t="inlineStr">
         <is>
-          <t>Buat resto baru dari Super Admin</t>
+          <t>Coba UPDATE products langsung lewat API sebagai pelanggan</t>
         </is>
       </c>
       <c r="E291" s="16" t="inlineStr">
         <is>
-          <t>Bagan akun GL 12 jenis dan tarif PPN/service langsung terisi</t>
+          <t>Ditolak; pengurangan stok hanya lewat decrement_stock</t>
         </is>
       </c>
       <c r="F291" s="16" t="inlineStr">
         <is>
-          <t>A-19, TSD §6.2</t>
+          <t>TSD §5.2</t>
         </is>
       </c>
       <c r="G291" s="16" t="inlineStr"/>
@@ -11946,7 +11946,7 @@
       </c>
       <c r="B292" s="14" t="inlineStr">
         <is>
-          <t>TC-TS-10</t>
+          <t>TC-TS-06</t>
         </is>
       </c>
       <c r="C292" s="15" t="inlineStr">
@@ -11956,17 +11956,17 @@
       </c>
       <c r="D292" s="13" t="inlineStr">
         <is>
-          <t>Kosongkan satu nomor GL, lalu buat transaksi</t>
+          <t>Panggil cancel_my_order untuk pesanan milik orang lain</t>
         </is>
       </c>
       <c r="E292" s="13" t="inlineStr">
         <is>
-          <t>Jurnal untuk baris itu tidak terbentuk — pastikan gejalanya dikenali penguji</t>
+          <t>Ditolak</t>
         </is>
       </c>
       <c r="F292" s="13" t="inlineStr">
         <is>
-          <t>TSD §6.2</t>
+          <t>TSD §5.2</t>
         </is>
       </c>
       <c r="G292" s="13" t="inlineStr"/>
@@ -11981,27 +11981,27 @@
       </c>
       <c r="B293" s="17" t="inlineStr">
         <is>
-          <t>TC-TS-11</t>
-        </is>
-      </c>
-      <c r="C293" s="20" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-TS-07</t>
+        </is>
+      </c>
+      <c r="C293" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D293" s="16" t="inlineStr">
         <is>
-          <t>Periksa push_outbox sesudah pengumuman terbit</t>
+          <t>Jalankan ulang seluruh JALANKAN-INI.sql di database yang sudah terisi</t>
         </is>
       </c>
       <c r="E293" s="16" t="inlineStr">
         <is>
-          <t>Baris masuk, lalu sent_at terisi</t>
+          <t>Selesai tanpa galat; tidak ada data yang berubah</t>
         </is>
       </c>
       <c r="F293" s="16" t="inlineStr">
         <is>
-          <t>TSD §8</t>
+          <t>TSD §11</t>
         </is>
       </c>
       <c r="G293" s="16" t="inlineStr"/>
@@ -12016,27 +12016,27 @@
       </c>
       <c r="B294" s="14" t="inlineStr">
         <is>
-          <t>TC-TS-12</t>
-        </is>
-      </c>
-      <c r="C294" s="19" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-TS-08</t>
+        </is>
+      </c>
+      <c r="C294" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D294" s="13" t="inlineStr">
         <is>
-          <t>Matikan sambungan, pakai aplikasi</t>
+          <t>Jalankan ulang satu berkas SQL lama saja, misal cash_payment_expiry.sql</t>
         </is>
       </c>
       <c r="E294" s="13" t="inlineStr">
         <is>
-          <t>Katalog tetap tampil; pesanan tunai tetap bisa dibuat</t>
+          <t>Tidak menyempitkan daftar nilai batasan mana pun</t>
         </is>
       </c>
       <c r="F294" s="13" t="inlineStr">
         <is>
-          <t>TSD §10, FSD §5.6</t>
+          <t>TSD §11.1</t>
         </is>
       </c>
       <c r="G294" s="13" t="inlineStr"/>
@@ -12051,27 +12051,27 @@
       </c>
       <c r="B295" s="17" t="inlineStr">
         <is>
-          <t>TC-TS-13</t>
-        </is>
-      </c>
-      <c r="C295" s="20" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-TS-09</t>
+        </is>
+      </c>
+      <c r="C295" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D295" s="16" t="inlineStr">
         <is>
-          <t>Sambungkan lagi</t>
+          <t>Buat resto baru dari Super Admin</t>
         </is>
       </c>
       <c r="E295" s="16" t="inlineStr">
         <is>
-          <t>Pesanan yang dibuat saat luring terkirim</t>
+          <t>Bagan akun GL 12 jenis dan tarif PPN/service langsung terisi</t>
         </is>
       </c>
       <c r="F295" s="16" t="inlineStr">
         <is>
-          <t>TSD §10</t>
+          <t>A-19, TSD §6.2</t>
         </is>
       </c>
       <c r="G295" s="16" t="inlineStr"/>
@@ -12086,7 +12086,7 @@
       </c>
       <c r="B296" s="14" t="inlineStr">
         <is>
-          <t>TC-TS-14</t>
+          <t>TC-TS-10</t>
         </is>
       </c>
       <c r="C296" s="15" t="inlineStr">
@@ -12096,17 +12096,17 @@
       </c>
       <c r="D296" s="13" t="inlineStr">
         <is>
-          <t>Coba bayar QRIS saat luring</t>
+          <t>Kosongkan satu nomor GL, lalu buat transaksi</t>
         </is>
       </c>
       <c r="E296" s="13" t="inlineStr">
         <is>
-          <t>Ditolak dengan jelas — bukan menggantung tanpa kabar</t>
+          <t>Jurnal untuk baris itu tidak terbentuk — pastikan gejalanya dikenali penguji</t>
         </is>
       </c>
       <c r="F296" s="13" t="inlineStr">
         <is>
-          <t>FSD §5.6</t>
+          <t>TSD §6.2</t>
         </is>
       </c>
       <c r="G296" s="13" t="inlineStr"/>
@@ -12121,27 +12121,27 @@
       </c>
       <c r="B297" s="17" t="inlineStr">
         <is>
-          <t>TC-TS-15</t>
-        </is>
-      </c>
-      <c r="C297" s="18" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>TC-TS-11</t>
+        </is>
+      </c>
+      <c r="C297" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D297" s="16" t="inlineStr">
         <is>
-          <t>Panggil create-qris dengan nominal yang dipalsukan di badan permintaan</t>
+          <t>Periksa push_outbox sesudah pengumuman terbit</t>
         </is>
       </c>
       <c r="E297" s="16" t="inlineStr">
         <is>
-          <t>Nominal yang dipakai tetap dari basis data</t>
+          <t>Baris masuk, lalu sent_at terisi</t>
         </is>
       </c>
       <c r="F297" s="16" t="inlineStr">
         <is>
-          <t>TSD §7.1</t>
+          <t>TSD §8</t>
         </is>
       </c>
       <c r="G297" s="16" t="inlineStr"/>
@@ -12156,27 +12156,27 @@
       </c>
       <c r="B298" s="14" t="inlineStr">
         <is>
-          <t>TC-TS-16</t>
-        </is>
-      </c>
-      <c r="C298" s="15" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>TC-TS-12</t>
+        </is>
+      </c>
+      <c r="C298" s="19" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D298" s="13" t="inlineStr">
         <is>
-          <t>Tandai pesanan lunas lewat API tanpa lewat webhook</t>
+          <t>Matikan sambungan, pakai aplikasi</t>
         </is>
       </c>
       <c r="E298" s="13" t="inlineStr">
         <is>
-          <t>Ditolak</t>
+          <t>Katalog tetap tampil; pesanan tunai tetap bisa dibuat</t>
         </is>
       </c>
       <c r="F298" s="13" t="inlineStr">
         <is>
-          <t>F-PG-02, TSD §7.1</t>
+          <t>TSD §10, FSD §5.6</t>
         </is>
       </c>
       <c r="G298" s="13" t="inlineStr"/>
@@ -12191,7 +12191,7 @@
       </c>
       <c r="B299" s="17" t="inlineStr">
         <is>
-          <t>TC-TS-17</t>
+          <t>TC-TS-13</t>
         </is>
       </c>
       <c r="C299" s="20" t="inlineStr">
@@ -12201,17 +12201,17 @@
       </c>
       <c r="D299" s="16" t="inlineStr">
         <is>
-          <t>Bongkar APK, cari kunci Xendit/FCM/Resend</t>
+          <t>Sambungkan lagi</t>
         </is>
       </c>
       <c r="E299" s="16" t="inlineStr">
         <is>
-          <t>Tidak ada satu pun kunci pengirim di dalamnya</t>
+          <t>Pesanan yang dibuat saat luring terkirim</t>
         </is>
       </c>
       <c r="F299" s="16" t="inlineStr">
         <is>
-          <t>TSD §1.2</t>
+          <t>TSD §10</t>
         </is>
       </c>
       <c r="G299" s="16" t="inlineStr"/>
@@ -12226,27 +12226,27 @@
       </c>
       <c r="B300" s="14" t="inlineStr">
         <is>
-          <t>TC-TS-18</t>
-        </is>
-      </c>
-      <c r="C300" s="19" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-TS-14</t>
+        </is>
+      </c>
+      <c r="C300" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D300" s="13" t="inlineStr">
         <is>
-          <t>Pesanan berpindah status lunas lebih dari sekali</t>
+          <t>Coba bayar QRIS saat luring</t>
         </is>
       </c>
       <c r="E300" s="13" t="inlineStr">
         <is>
-          <t>Jurnalnya tetap satu set — tidak ada baris ganda</t>
+          <t>Ditolak dengan jelas — bukan menggantung tanpa kabar</t>
         </is>
       </c>
       <c r="F300" s="13" t="inlineStr">
         <is>
-          <t>TSD §6.5</t>
+          <t>FSD §5.6</t>
         </is>
       </c>
       <c r="G300" s="13" t="inlineStr"/>
@@ -12261,27 +12261,27 @@
       </c>
       <c r="B301" s="17" t="inlineStr">
         <is>
-          <t>TC-TS-19</t>
-        </is>
-      </c>
-      <c r="C301" s="20" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-TS-15</t>
+        </is>
+      </c>
+      <c r="C301" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D301" s="16" t="inlineStr">
         <is>
-          <t>Hapus resto uji</t>
+          <t>Panggil create-qris dengan nominal yang dipalsukan di badan permintaan</t>
         </is>
       </c>
       <c r="E301" s="16" t="inlineStr">
         <is>
-          <t>Seluruh isinya ikut terhapus, termasuk jurnalnya</t>
+          <t>Nominal yang dipakai tetap dari basis data</t>
         </is>
       </c>
       <c r="F301" s="16" t="inlineStr">
         <is>
-          <t>TSD §4.0</t>
+          <t>TSD §7.1</t>
         </is>
       </c>
       <c r="G301" s="16" t="inlineStr"/>
@@ -12291,12 +12291,12 @@
     <row r="302">
       <c r="A302" s="13" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>Uji Teknis (lingkup TSD)</t>
         </is>
       </c>
       <c r="B302" s="14" t="inlineStr">
         <is>
-          <t>TC-RG-01</t>
+          <t>TC-TS-16</t>
         </is>
       </c>
       <c r="C302" s="15" t="inlineStr">
@@ -12306,17 +12306,17 @@
       </c>
       <c r="D302" s="13" t="inlineStr">
         <is>
-          <t>Nominal QRIS kasir memakai subtotal menu, bukan total tagihan</t>
+          <t>Tandai pesanan lunas lewat API tanpa lewat webhook</t>
         </is>
       </c>
       <c r="E302" s="13" t="inlineStr">
         <is>
-          <t>Nominal di layar QRIS = total termasuk service dan PPN</t>
+          <t>Ditolak</t>
         </is>
       </c>
       <c r="F302" s="13" t="inlineStr">
         <is>
-          <t>F-KS-09</t>
+          <t>F-PG-02, TSD §7.1</t>
         </is>
       </c>
       <c r="G302" s="13" t="inlineStr"/>
@@ -12326,32 +12326,32 @@
     <row r="303">
       <c r="A303" s="16" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>Uji Teknis (lingkup TSD)</t>
         </is>
       </c>
       <c r="B303" s="17" t="inlineStr">
         <is>
-          <t>TC-RG-02</t>
-        </is>
-      </c>
-      <c r="C303" s="18" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>TC-TS-17</t>
+        </is>
+      </c>
+      <c r="C303" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D303" s="16" t="inlineStr">
         <is>
-          <t>Pesanan dilunasi lewat QRIS hilang dari Riwayat Kasir</t>
+          <t>Bongkar APK, cari kunci Xendit/FCM/Resend</t>
         </is>
       </c>
       <c r="E303" s="16" t="inlineStr">
         <is>
-          <t>Semua cara bayar masuk Riwayat Kasir</t>
+          <t>Tidak ada satu pun kunci pengirim di dalamnya</t>
         </is>
       </c>
       <c r="F303" s="16" t="inlineStr">
         <is>
-          <t>F-PP-09, A-13</t>
+          <t>TSD §1.2</t>
         </is>
       </c>
       <c r="G303" s="16" t="inlineStr"/>
@@ -12361,32 +12361,32 @@
     <row r="304">
       <c r="A304" s="13" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>Uji Teknis (lingkup TSD)</t>
         </is>
       </c>
       <c r="B304" s="14" t="inlineStr">
         <is>
-          <t>TC-RG-03</t>
-        </is>
-      </c>
-      <c r="C304" s="15" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>TC-TS-18</t>
+        </is>
+      </c>
+      <c r="C304" s="19" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D304" s="13" t="inlineStr">
         <is>
-          <t>Pesanan dibatalkan tampil "Menunggu Pembayaran" di Pesanan Masuk</t>
+          <t>Pesanan berpindah status lunas lebih dari sekali</t>
         </is>
       </c>
       <c r="E304" s="13" t="inlineStr">
         <is>
-          <t>Tidak muncul sama sekali</t>
+          <t>Jurnalnya tetap satu set — tidak ada baris ganda</t>
         </is>
       </c>
       <c r="F304" s="13" t="inlineStr">
         <is>
-          <t>A-17</t>
+          <t>TSD §6.5</t>
         </is>
       </c>
       <c r="G304" s="13" t="inlineStr"/>
@@ -12396,32 +12396,32 @@
     <row r="305">
       <c r="A305" s="16" t="inlineStr">
         <is>
-          <t>Regresi — bug yang pernah terjadi</t>
+          <t>Uji Teknis (lingkup TSD)</t>
         </is>
       </c>
       <c r="B305" s="17" t="inlineStr">
         <is>
-          <t>TC-RG-04</t>
-        </is>
-      </c>
-      <c r="C305" s="18" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>TC-TS-19</t>
+        </is>
+      </c>
+      <c r="C305" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D305" s="16" t="inlineStr">
         <is>
-          <t>Top up Rp 100.000 tercatat Rp 200.000 di jurnal</t>
+          <t>Hapus resto uji</t>
         </is>
       </c>
       <c r="E305" s="16" t="inlineStr">
         <is>
-          <t>Nominalnya sama dengan yang diajukan</t>
+          <t>Seluruh isinya ikut terhapus, termasuk jurnalnya</t>
         </is>
       </c>
       <c r="F305" s="16" t="inlineStr">
         <is>
-          <t>F-FN-03</t>
+          <t>TSD §4.0</t>
         </is>
       </c>
       <c r="G305" s="16" t="inlineStr"/>
@@ -12436,7 +12436,7 @@
       </c>
       <c r="B306" s="14" t="inlineStr">
         <is>
-          <t>TC-RG-05</t>
+          <t>TC-RG-01</t>
         </is>
       </c>
       <c r="C306" s="15" t="inlineStr">
@@ -12446,17 +12446,17 @@
       </c>
       <c r="D306" s="13" t="inlineStr">
         <is>
-          <t>Diskon tidak berlaku untuk pesanan mandiri pelanggan</t>
+          <t>Nominal QRIS kasir memakai subtotal menu, bukan total tagihan</t>
         </is>
       </c>
       <c r="E306" s="13" t="inlineStr">
         <is>
-          <t>Berlaku sama di kasir dan HP pelanggan</t>
+          <t>Nominal di layar QRIS = total termasuk service dan PPN</t>
         </is>
       </c>
       <c r="F306" s="13" t="inlineStr">
         <is>
-          <t>A-14</t>
+          <t>F-KS-09</t>
         </is>
       </c>
       <c r="G306" s="13" t="inlineStr"/>
@@ -12471,7 +12471,7 @@
       </c>
       <c r="B307" s="17" t="inlineStr">
         <is>
-          <t>TC-RG-06</t>
+          <t>TC-RG-02</t>
         </is>
       </c>
       <c r="C307" s="18" t="inlineStr">
@@ -12481,17 +12481,17 @@
       </c>
       <c r="D307" s="16" t="inlineStr">
         <is>
-          <t>Promo "beli 2" lolos oleh keranjang berisi dua menu berbeda</t>
+          <t>Pesanan dilunasi lewat QRIS hilang dari Riwayat Kasir</t>
         </is>
       </c>
       <c r="E307" s="16" t="inlineStr">
         <is>
-          <t>Syarat jumlah dihitung per menu, dan seluruhnya harus terpenuhi</t>
+          <t>Semua cara bayar masuk Riwayat Kasir</t>
         </is>
       </c>
       <c r="F307" s="16" t="inlineStr">
         <is>
-          <t>F-DS-10, F-DS-12</t>
+          <t>F-PP-09, A-13</t>
         </is>
       </c>
       <c r="G307" s="16" t="inlineStr"/>
@@ -12506,27 +12506,27 @@
       </c>
       <c r="B308" s="14" t="inlineStr">
         <is>
-          <t>TC-RG-07</t>
-        </is>
-      </c>
-      <c r="C308" s="19" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-RG-03</t>
+        </is>
+      </c>
+      <c r="C308" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D308" s="13" t="inlineStr">
         <is>
-          <t>Tombol pilih/hapus di kotak masuk tidak bereaksi sama sekali</t>
+          <t>Pesanan dibatalkan tampil "Menunggu Pembayaran" di Pesanan Masuk</t>
         </is>
       </c>
       <c r="E308" s="13" t="inlineStr">
         <is>
-          <t>Bekerja di kotak masuk karyawan dan pelanggan</t>
+          <t>Tidak muncul sama sekali</t>
         </is>
       </c>
       <c r="F308" s="13" t="inlineStr">
         <is>
-          <t>F-IN-15</t>
+          <t>A-17</t>
         </is>
       </c>
       <c r="G308" s="13" t="inlineStr"/>
@@ -12541,27 +12541,27 @@
       </c>
       <c r="B309" s="17" t="inlineStr">
         <is>
-          <t>TC-RG-08</t>
-        </is>
-      </c>
-      <c r="C309" s="20" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-RG-04</t>
+        </is>
+      </c>
+      <c r="C309" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D309" s="16" t="inlineStr">
         <is>
-          <t>Layar Diskon dari hub Kasir menyebut "Belum ada produk di resto ini"</t>
+          <t>Top up Rp 100.000 tercatat Rp 200.000 di jurnal</t>
         </is>
       </c>
       <c r="E309" s="16" t="inlineStr">
         <is>
-          <t>Daftar menu termuat</t>
+          <t>Nominalnya sama dengan yang diajukan</t>
         </is>
       </c>
       <c r="F309" s="16" t="inlineStr">
         <is>
-          <t>F-DS-01</t>
+          <t>F-FN-03</t>
         </is>
       </c>
       <c r="G309" s="16" t="inlineStr"/>
@@ -12576,27 +12576,27 @@
       </c>
       <c r="B310" s="14" t="inlineStr">
         <is>
-          <t>TC-RG-09</t>
-        </is>
-      </c>
-      <c r="C310" s="19" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-RG-05</t>
+        </is>
+      </c>
+      <c r="C310" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D310" s="13" t="inlineStr">
         <is>
-          <t>Kasir tidak bisa membuka detail jurnal — terlihat seperti GL belum dipetakan</t>
+          <t>Diskon tidak berlaku untuk pesanan mandiri pelanggan</t>
         </is>
       </c>
       <c r="E310" s="13" t="inlineStr">
         <is>
-          <t>Detail jurnal terbuka</t>
+          <t>Berlaku sama di kasir dan HP pelanggan</t>
         </is>
       </c>
       <c r="F310" s="13" t="inlineStr">
         <is>
-          <t>F-KS-13</t>
+          <t>A-14</t>
         </is>
       </c>
       <c r="G310" s="13" t="inlineStr"/>
@@ -12611,27 +12611,27 @@
       </c>
       <c r="B311" s="17" t="inlineStr">
         <is>
-          <t>TC-RG-10</t>
-        </is>
-      </c>
-      <c r="C311" s="20" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TC-RG-06</t>
+        </is>
+      </c>
+      <c r="C311" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D311" s="16" t="inlineStr">
         <is>
-          <t>Layar dapur meninggalkan jejak warna lama saat tema diganti</t>
+          <t>Promo "beli 2" lolos oleh keranjang berisi dua menu berbeda</t>
         </is>
       </c>
       <c r="E311" s="16" t="inlineStr">
         <is>
-          <t>Seluruh layar berganti bersih</t>
+          <t>Syarat jumlah dihitung per menu, dan seluruhnya harus terpenuhi</t>
         </is>
       </c>
       <c r="F311" s="16" t="inlineStr">
         <is>
-          <t>A-18</t>
+          <t>F-DS-10, F-DS-12</t>
         </is>
       </c>
       <c r="G311" s="16" t="inlineStr"/>
@@ -12646,7 +12646,7 @@
       </c>
       <c r="B312" s="14" t="inlineStr">
         <is>
-          <t>TC-RG-11</t>
+          <t>TC-RG-07</t>
         </is>
       </c>
       <c r="C312" s="19" t="inlineStr">
@@ -12656,17 +12656,17 @@
       </c>
       <c r="D312" s="13" t="inlineStr">
         <is>
-          <t>Banner promo menempel di atas, tidak ikut tergulir</t>
+          <t>Tombol pilih/hapus di kotak masuk tidak bereaksi sama sekali</t>
         </is>
       </c>
       <c r="E312" s="13" t="inlineStr">
         <is>
-          <t>Ikut tergulir bersama menunya</t>
+          <t>Bekerja di kotak masuk karyawan dan pelanggan</t>
         </is>
       </c>
       <c r="F312" s="13" t="inlineStr">
         <is>
-          <t>F-CU-16, A-12</t>
+          <t>F-IN-15</t>
         </is>
       </c>
       <c r="G312" s="13" t="inlineStr"/>
@@ -12681,7 +12681,7 @@
       </c>
       <c r="B313" s="17" t="inlineStr">
         <is>
-          <t>TC-RG-12</t>
+          <t>TC-RG-08</t>
         </is>
       </c>
       <c r="C313" s="20" t="inlineStr">
@@ -12691,17 +12691,17 @@
       </c>
       <c r="D313" s="16" t="inlineStr">
         <is>
-          <t>Owner hanya bisa melihat Info Pembayaran</t>
+          <t>Layar Diskon dari hub Kasir menyebut "Belum ada produk di resto ini"</t>
         </is>
       </c>
       <c r="E313" s="16" t="inlineStr">
         <is>
-          <t>Owner bisa mengubahnya</t>
+          <t>Daftar menu termuat</t>
         </is>
       </c>
       <c r="F313" s="16" t="inlineStr">
         <is>
-          <t>F-SD-02</t>
+          <t>F-DS-01</t>
         </is>
       </c>
       <c r="G313" s="16" t="inlineStr"/>
@@ -12716,27 +12716,27 @@
       </c>
       <c r="B314" s="14" t="inlineStr">
         <is>
-          <t>TC-RG-13</t>
-        </is>
-      </c>
-      <c r="C314" s="15" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>TC-RG-09</t>
+        </is>
+      </c>
+      <c r="C314" s="19" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D314" s="13" t="inlineStr">
         <is>
-          <t>Migrasi gagal: daftar nilai batasan menyempit saat berkas lama dijalankan ulang</t>
+          <t>Kasir tidak bisa membuka detail jurnal — terlihat seperti GL belum dipetakan</t>
         </is>
       </c>
       <c r="E314" s="13" t="inlineStr">
         <is>
-          <t>Menjalankan ulang berkas mana pun tidak pernah menolak data yang sudah ada</t>
+          <t>Detail jurnal terbuka</t>
         </is>
       </c>
       <c r="F314" s="13" t="inlineStr">
         <is>
-          <t>TSD §11.1</t>
+          <t>F-KS-13</t>
         </is>
       </c>
       <c r="G314" s="13" t="inlineStr"/>
@@ -12751,7 +12751,7 @@
       </c>
       <c r="B315" s="17" t="inlineStr">
         <is>
-          <t>TC-RG-14</t>
+          <t>TC-RG-10</t>
         </is>
       </c>
       <c r="C315" s="20" t="inlineStr">
@@ -12761,17 +12761,17 @@
       </c>
       <c r="D315" s="16" t="inlineStr">
         <is>
-          <t>QR meja borongan bernomor 07, berbeda dengan mode satu meja</t>
+          <t>Layar dapur meninggalkan jejak warna lama saat tema diganti</t>
         </is>
       </c>
       <c r="E315" s="16" t="inlineStr">
         <is>
-          <t>Keduanya menulis 7</t>
+          <t>Seluruh layar berganti bersih</t>
         </is>
       </c>
       <c r="F315" s="16" t="inlineStr">
         <is>
-          <t>F-QR-07</t>
+          <t>A-18</t>
         </is>
       </c>
       <c r="G315" s="16" t="inlineStr"/>
@@ -12781,25 +12781,165 @@
     <row r="316">
       <c r="A316" s="13" t="inlineStr">
         <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B316" s="14" t="inlineStr">
+        <is>
+          <t>TC-RG-11</t>
+        </is>
+      </c>
+      <c r="C316" s="19" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D316" s="13" t="inlineStr">
+        <is>
+          <t>Banner promo menempel di atas, tidak ikut tergulir</t>
+        </is>
+      </c>
+      <c r="E316" s="13" t="inlineStr">
+        <is>
+          <t>Ikut tergulir bersama menunya</t>
+        </is>
+      </c>
+      <c r="F316" s="13" t="inlineStr">
+        <is>
+          <t>F-CU-16, A-12</t>
+        </is>
+      </c>
+      <c r="G316" s="13" t="inlineStr"/>
+      <c r="H316" s="13" t="inlineStr"/>
+      <c r="I316" s="13" t="inlineStr"/>
+    </row>
+    <row r="317">
+      <c r="A317" s="16" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B317" s="17" t="inlineStr">
+        <is>
+          <t>TC-RG-12</t>
+        </is>
+      </c>
+      <c r="C317" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D317" s="16" t="inlineStr">
+        <is>
+          <t>Owner hanya bisa melihat Info Pembayaran</t>
+        </is>
+      </c>
+      <c r="E317" s="16" t="inlineStr">
+        <is>
+          <t>Owner bisa mengubahnya</t>
+        </is>
+      </c>
+      <c r="F317" s="16" t="inlineStr">
+        <is>
+          <t>F-SD-02</t>
+        </is>
+      </c>
+      <c r="G317" s="16" t="inlineStr"/>
+      <c r="H317" s="16" t="inlineStr"/>
+      <c r="I317" s="16" t="inlineStr"/>
+    </row>
+    <row r="318">
+      <c r="A318" s="13" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B318" s="14" t="inlineStr">
+        <is>
+          <t>TC-RG-13</t>
+        </is>
+      </c>
+      <c r="C318" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D318" s="13" t="inlineStr">
+        <is>
+          <t>Migrasi gagal: daftar nilai batasan menyempit saat berkas lama dijalankan ulang</t>
+        </is>
+      </c>
+      <c r="E318" s="13" t="inlineStr">
+        <is>
+          <t>Menjalankan ulang berkas mana pun tidak pernah menolak data yang sudah ada</t>
+        </is>
+      </c>
+      <c r="F318" s="13" t="inlineStr">
+        <is>
+          <t>TSD §11.1</t>
+        </is>
+      </c>
+      <c r="G318" s="13" t="inlineStr"/>
+      <c r="H318" s="13" t="inlineStr"/>
+      <c r="I318" s="13" t="inlineStr"/>
+    </row>
+    <row r="319">
+      <c r="A319" s="16" t="inlineStr">
+        <is>
+          <t>Regresi — bug yang pernah terjadi</t>
+        </is>
+      </c>
+      <c r="B319" s="17" t="inlineStr">
+        <is>
+          <t>TC-RG-14</t>
+        </is>
+      </c>
+      <c r="C319" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D319" s="16" t="inlineStr">
+        <is>
+          <t>QR meja borongan bernomor 07, berbeda dengan mode satu meja</t>
+        </is>
+      </c>
+      <c r="E319" s="16" t="inlineStr">
+        <is>
+          <t>Keduanya menulis 7</t>
+        </is>
+      </c>
+      <c r="F319" s="16" t="inlineStr">
+        <is>
+          <t>F-QR-07</t>
+        </is>
+      </c>
+      <c r="G319" s="16" t="inlineStr"/>
+      <c r="H319" s="16" t="inlineStr"/>
+      <c r="I319" s="16" t="inlineStr"/>
+    </row>
+    <row r="320">
+      <c r="A320" s="13" t="inlineStr">
+        <is>
           <t>Uji Ujung-ke-Ujung</t>
         </is>
       </c>
-      <c r="B316" s="14" t="inlineStr">
+      <c r="B320" s="14" t="inlineStr">
         <is>
           <t>E2E-09</t>
         </is>
       </c>
-      <c r="C316" s="15" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D316" s="13" t="inlineStr">
+      <c r="C320" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D320" s="13" t="inlineStr">
         <is>
           <t>Satu siklus langganan penuh</t>
         </is>
       </c>
-      <c r="E316" s="13" t="inlineStr">
+      <c r="E320" s="13" t="inlineStr">
         <is>
           <t>1. Super Admin setel resto uji: Rp 150.000, jatuh tempo 3 hari lagi, tenggang 1 hari
 2. Terbitkan tagihan → periksa muncul di tab Tagihan berstatus Belum Dibayar
@@ -12813,37 +12953,37 @@
 10. Periksa Dashboard Xendit → dana masuk ke akun KaataGo, bukan sub-akun resto</t>
         </is>
       </c>
-      <c r="F316" s="13" t="inlineStr">
+      <c r="F320" s="13" t="inlineStr">
         <is>
           <t>F-BL-07 … F-BL-18, TSD §7.3</t>
         </is>
       </c>
-      <c r="G316" s="13" t="inlineStr"/>
-      <c r="H316" s="13" t="inlineStr"/>
-      <c r="I316" s="13" t="inlineStr"/>
-    </row>
-    <row r="317">
-      <c r="A317" s="16" t="inlineStr">
+      <c r="G320" s="13" t="inlineStr"/>
+      <c r="H320" s="13" t="inlineStr"/>
+      <c r="I320" s="13" t="inlineStr"/>
+    </row>
+    <row r="321">
+      <c r="A321" s="16" t="inlineStr">
         <is>
           <t>Uji Ujung-ke-Ujung</t>
         </is>
       </c>
-      <c r="B317" s="17" t="inlineStr">
+      <c r="B321" s="17" t="inlineStr">
         <is>
           <t>E2E-01</t>
         </is>
       </c>
-      <c r="C317" s="18" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D317" s="16" t="inlineStr">
+      <c r="C321" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D321" s="16" t="inlineStr">
         <is>
           <t>Pelanggan bayar QRIS</t>
         </is>
       </c>
-      <c r="E317" s="16" t="inlineStr">
+      <c r="E321" s="16" t="inlineStr">
         <is>
           <t>1. Pelanggan scan QR meja → pilih 2 menu → Dine In → isi nama
 2. Pilih QRIS → bayar sungguhan dari aplikasi bank
@@ -12855,37 +12995,37 @@
 8. Periksa Saldo → masuk Non Cash, bukan Cash</t>
         </is>
       </c>
-      <c r="F317" s="16" t="inlineStr">
+      <c r="F321" s="16" t="inlineStr">
         <is>
           <t>F-CU-09, F-PG-02, F-CH-06, TSD §6, TSD §7.1</t>
         </is>
       </c>
-      <c r="G317" s="16" t="inlineStr"/>
-      <c r="H317" s="16" t="inlineStr"/>
-      <c r="I317" s="16" t="inlineStr"/>
-    </row>
-    <row r="318">
-      <c r="A318" s="13" t="inlineStr">
+      <c r="G321" s="16" t="inlineStr"/>
+      <c r="H321" s="16" t="inlineStr"/>
+      <c r="I321" s="16" t="inlineStr"/>
+    </row>
+    <row r="322">
+      <c r="A322" s="13" t="inlineStr">
         <is>
           <t>Uji Ujung-ke-Ujung</t>
         </is>
       </c>
-      <c r="B318" s="14" t="inlineStr">
+      <c r="B322" s="14" t="inlineStr">
         <is>
           <t>E2E-02</t>
         </is>
       </c>
-      <c r="C318" s="15" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D318" s="13" t="inlineStr">
+      <c r="C322" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D322" s="13" t="inlineStr">
         <is>
           <t>Pelanggan bayar tunai di kasir</t>
         </is>
       </c>
-      <c r="E318" s="13" t="inlineStr">
+      <c r="E322" s="13" t="inlineStr">
         <is>
           <t>1. Pelanggan pesan → pilih Tunai → catat nomor pesanannya
 2. Periksa layar pelanggan → hitungan mundur 30 menit berjalan
@@ -12897,74 +13037,74 @@
 8. Periksa Saldo Cash → bertambah sebesar totalnya</t>
         </is>
       </c>
-      <c r="F318" s="13" t="inlineStr">
+      <c r="F322" s="13" t="inlineStr">
         <is>
           <t>F-CU-09, F-PP-01, F-PP-06, F-PP-07, F-CH-06, A-02, A-13</t>
         </is>
       </c>
-      <c r="G318" s="13" t="inlineStr"/>
-      <c r="H318" s="13" t="inlineStr"/>
-      <c r="I318" s="13" t="inlineStr"/>
-    </row>
-    <row r="319">
-      <c r="A319" s="16" t="inlineStr">
+      <c r="G322" s="13" t="inlineStr"/>
+      <c r="H322" s="13" t="inlineStr"/>
+      <c r="I322" s="13" t="inlineStr"/>
+    </row>
+    <row r="323">
+      <c r="A323" s="16" t="inlineStr">
         <is>
           <t>Uji Ujung-ke-Ujung</t>
         </is>
       </c>
-      <c r="B319" s="17" t="inlineStr">
+      <c r="B323" s="17" t="inlineStr">
         <is>
           <t>E2E-03</t>
         </is>
       </c>
-      <c r="C319" s="18" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D319" s="16" t="inlineStr">
+      <c r="C323" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D323" s="16" t="inlineStr">
         <is>
           <t>Tunai dengan cara bayar diganti</t>
         </is>
       </c>
-      <c r="E319" s="16" t="inlineStr">
+      <c r="E323" s="16" t="inlineStr">
         <is>
           <t>1. Ulangi E2E-02, tapi pada langkah 4 ganti cara bayarnya ke QRIS.
 2. Pesanannya harus tetap masuk Riwayat Kasir, dan masuk Non Cash
 3. di Saldo.</t>
         </is>
       </c>
-      <c r="F319" s="16" t="inlineStr">
+      <c r="F323" s="16" t="inlineStr">
         <is>
           <t>F-PP-09, A-13, TSD §4.2</t>
         </is>
       </c>
-      <c r="G319" s="16" t="inlineStr"/>
-      <c r="H319" s="16" t="inlineStr"/>
-      <c r="I319" s="16" t="inlineStr"/>
-    </row>
-    <row r="320">
-      <c r="A320" s="13" t="inlineStr">
+      <c r="G323" s="16" t="inlineStr"/>
+      <c r="H323" s="16" t="inlineStr"/>
+      <c r="I323" s="16" t="inlineStr"/>
+    </row>
+    <row r="324">
+      <c r="A324" s="13" t="inlineStr">
         <is>
           <t>Uji Ujung-ke-Ujung</t>
         </is>
       </c>
-      <c r="B320" s="14" t="inlineStr">
+      <c r="B324" s="14" t="inlineStr">
         <is>
           <t>E2E-04</t>
         </is>
       </c>
-      <c r="C320" s="15" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D320" s="13" t="inlineStr">
+      <c r="C324" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D324" s="13" t="inlineStr">
         <is>
           <t>Setor tunai ke rekening</t>
         </is>
       </c>
-      <c r="E320" s="13" t="inlineStr">
+      <c r="E324" s="13" t="inlineStr">
         <is>
           <t>1. Kasir buka Setor Saldo Cash → catat tunai di laci
 2. Ajukan setoran sebesar sebagian dari itu, lampirkan bukti
@@ -12975,73 +13115,73 @@
 7. Periksa Jurnal GL → titipan suspense dilepas, dana masuk GL Total Saldo</t>
         </is>
       </c>
-      <c r="F320" s="13" t="inlineStr">
+      <c r="F324" s="13" t="inlineStr">
         <is>
           <t>F-SD-01, F-SD-05, A-05, TSD §6.4</t>
         </is>
       </c>
-      <c r="G320" s="13" t="inlineStr"/>
-      <c r="H320" s="13" t="inlineStr"/>
-      <c r="I320" s="13" t="inlineStr"/>
-    </row>
-    <row r="321">
-      <c r="A321" s="16" t="inlineStr">
+      <c r="G324" s="13" t="inlineStr"/>
+      <c r="H324" s="13" t="inlineStr"/>
+      <c r="I324" s="13" t="inlineStr"/>
+    </row>
+    <row r="325">
+      <c r="A325" s="16" t="inlineStr">
         <is>
           <t>Uji Ujung-ke-Ujung</t>
         </is>
       </c>
-      <c r="B321" s="17" t="inlineStr">
+      <c r="B325" s="17" t="inlineStr">
         <is>
           <t>E2E-05</t>
         </is>
       </c>
-      <c r="C321" s="18" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D321" s="16" t="inlineStr">
+      <c r="C325" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D325" s="16" t="inlineStr">
         <is>
           <t>Top up petty cash</t>
         </is>
       </c>
-      <c r="E321" s="16" t="inlineStr">
+      <c r="E325" s="16" t="inlineStr">
         <is>
           <t>1. Sama polanya dengan E2E-04, lewat GL Suspense Petty Cash. Top up
 2. Rp 100.000 harus menambah Petty Cash Rp 100.000 — bukan Rp 200.000.</t>
         </is>
       </c>
-      <c r="F321" s="16" t="inlineStr">
+      <c r="F325" s="16" t="inlineStr">
         <is>
           <t>F-FN-03, TSD §6.4</t>
         </is>
       </c>
-      <c r="G321" s="16" t="inlineStr"/>
-      <c r="H321" s="16" t="inlineStr"/>
-      <c r="I321" s="16" t="inlineStr"/>
-    </row>
-    <row r="322">
-      <c r="A322" s="13" t="inlineStr">
+      <c r="G325" s="16" t="inlineStr"/>
+      <c r="H325" s="16" t="inlineStr"/>
+      <c r="I325" s="16" t="inlineStr"/>
+    </row>
+    <row r="326">
+      <c r="A326" s="13" t="inlineStr">
         <is>
           <t>Uji Ujung-ke-Ujung</t>
         </is>
       </c>
-      <c r="B322" s="14" t="inlineStr">
+      <c r="B326" s="14" t="inlineStr">
         <is>
           <t>E2E-06</t>
         </is>
       </c>
-      <c r="C322" s="15" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D322" s="13" t="inlineStr">
+      <c r="C326" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D326" s="13" t="inlineStr">
         <is>
           <t>Promo bundling dari HP pelanggan</t>
         </is>
       </c>
-      <c r="E322" s="13" t="inlineStr">
+      <c r="E326" s="13" t="inlineStr">
         <is>
           <t>1. Admin buat promo: Nasi Goreng Minimal 2 + Es Teh Minimal 1, potongan 30%
 2. Pelanggan pesan 2 Nasi Goreng saja → tidak ada potongan
@@ -13052,37 +13192,37 @@
 7. Admin hapus promonya → cetak ulang struk tadi → potongannya tetap tertulis</t>
         </is>
       </c>
-      <c r="F322" s="13" t="inlineStr">
+      <c r="F326" s="13" t="inlineStr">
         <is>
           <t>F-DS-10, F-DS-12, F-CU-17, F-DS-08, F-DS-09, A-14</t>
         </is>
       </c>
-      <c r="G322" s="13" t="inlineStr"/>
-      <c r="H322" s="13" t="inlineStr"/>
-      <c r="I322" s="13" t="inlineStr"/>
-    </row>
-    <row r="323">
-      <c r="A323" s="16" t="inlineStr">
+      <c r="G326" s="13" t="inlineStr"/>
+      <c r="H326" s="13" t="inlineStr"/>
+      <c r="I326" s="13" t="inlineStr"/>
+    </row>
+    <row r="327">
+      <c r="A327" s="16" t="inlineStr">
         <is>
           <t>Uji Ujung-ke-Ujung</t>
         </is>
       </c>
-      <c r="B323" s="17" t="inlineStr">
+      <c r="B327" s="17" t="inlineStr">
         <is>
           <t>E2E-07</t>
         </is>
       </c>
-      <c r="C323" s="18" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D323" s="16" t="inlineStr">
+      <c r="C327" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D327" s="16" t="inlineStr">
         <is>
           <t>Pembatalan oleh pelanggan</t>
         </is>
       </c>
-      <c r="E323" s="16" t="inlineStr">
+      <c r="E327" s="16" t="inlineStr">
         <is>
           <t>1. Pelanggan pesan, pilih Tunai
 2. Batalkan dari Pesanan Saya → berhasil
@@ -13092,37 +13232,37 @@
 6. Periksa Riwayat Kasir → tidak ikut terhitung</t>
         </is>
       </c>
-      <c r="F323" s="16" t="inlineStr">
+      <c r="F327" s="16" t="inlineStr">
         <is>
           <t>F-CN-01, A-17</t>
         </is>
       </c>
-      <c r="G323" s="16" t="inlineStr"/>
-      <c r="H323" s="16" t="inlineStr"/>
-      <c r="I323" s="16" t="inlineStr"/>
-    </row>
-    <row r="324">
-      <c r="A324" s="13" t="inlineStr">
+      <c r="G327" s="16" t="inlineStr"/>
+      <c r="H327" s="16" t="inlineStr"/>
+      <c r="I327" s="16" t="inlineStr"/>
+    </row>
+    <row r="328">
+      <c r="A328" s="13" t="inlineStr">
         <is>
           <t>Uji Ujung-ke-Ujung</t>
         </is>
       </c>
-      <c r="B324" s="14" t="inlineStr">
+      <c r="B328" s="14" t="inlineStr">
         <is>
           <t>E2E-08</t>
         </is>
       </c>
-      <c r="C324" s="15" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D324" s="13" t="inlineStr">
+      <c r="C328" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D328" s="13" t="inlineStr">
         <is>
           <t>Isolasi antar cabang</t>
         </is>
       </c>
-      <c r="E324" s="13" t="inlineStr">
+      <c r="E328" s="13" t="inlineStr">
         <is>
           <t>1. Dengan akun Owner yang memiliki dua resto: buat transaksi, promo, dan
 2. pengumuman di resto A, lalu berpindah ke resto B. Tidak satu pun
@@ -13130,19 +13270,19 @@
 4. dan kotak masuk.</t>
         </is>
       </c>
-      <c r="F324" s="13" t="inlineStr">
+      <c r="F328" s="13" t="inlineStr">
         <is>
           <t>F-AD-08, F-IN-10, A-10</t>
         </is>
       </c>
-      <c r="G324" s="13" t="inlineStr"/>
-      <c r="H324" s="13" t="inlineStr"/>
-      <c r="I324" s="13" t="inlineStr"/>
+      <c r="G328" s="13" t="inlineStr"/>
+      <c r="H328" s="13" t="inlineStr"/>
+      <c r="I328" s="13" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I324"/>
+  <autoFilter ref="A1:I328"/>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G324" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G328" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Lulus,Gagal,Terblokir,Dilewati"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>